<commit_message>
pixel-size+date table v1: 9-agent hunt merged + every citation refetch-verified; 2017 CoE dated (same orthomosaic as King 2017), 2000 pinned to 2000-06-26, 2022 CoE identity measured, 2020 anchor consistent with one pass; evidence harvested to qc/imagery_date_evidence
</commit_message>
<xml_diff>
--- a/Scripts/imagery_catalog_2026-08-22.xlsx
+++ b/Scripts/imagery_catalog_2026-08-22.xlsx
@@ -33,7 +33,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing_Risk" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MASTER'!$A$1:$P$221</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'KingCo_SDC_Catalog'!$A$1:$D$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DataLake_Issues'!$A$1:$C$15</definedName>
@@ -12156,7 +12156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -12457,7 +12457,7 @@
       </c>
       <c r="O3" s="1" t="inlineStr">
         <is>
-          <t>Acquisition period was Summer, 1998. Individual frame or tile acquisition dates are not available.</t>
+          <t>Acquisition period was Summer, 1998.  Individual frame or tile acquisition dates are not available.</t>
         </is>
       </c>
       <c r="P3" s="1" t="inlineStr">
@@ -12492,7 +12492,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>Emerge Inc. via King County GIS (IMAGE_Ortho2000EmergeNAT, natural-colour DERIVATIVE of EmergeCIR)</t>
+          <t>Emerge Inc. (contracted via Pacific Meridian / Space Imaging) via King County GIS (IMAGE_Ortho2000EmergeNAT, natural-colour DERIVATIVE of EmergeCIR)</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
@@ -12527,17 +12527,17 @@
       </c>
       <c r="J4" s="1" t="inlineStr">
         <is>
-          <t>late spring to early fall 2000</t>
+          <t>2000-06-26 (the township block containing Edmonds: T27N R3E / T27N R4E, per King County's flight-date graphic)</t>
         </is>
       </c>
       <c r="K4" s="1" t="inlineStr">
         <is>
-          <t>season (~5 months)</t>
+          <t>single day (township-block generalisation, NOT per-frame)</t>
         </is>
       </c>
       <c r="L4" s="1" t="inlineStr">
         <is>
-          <t>multi (township-level flight-date graphic referenced by the page is a 404)</t>
+          <t>single date for the Edmonds block per the graphic; project is multi-date (2000-05-24 to 09-23)</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
@@ -12547,17 +12547,17 @@
       </c>
       <c r="N4" s="1" t="inlineStr">
         <is>
-          <t>https://www5.kingcounty.gov/sdc/?Layer=IMAGE_Ortho2000EmergeNAT</t>
+          <t>https://web.archive.org/web/20081010173648if_/http://www.metrokc.gov/gis/sdc/raster/ortho/images/ortho2000emergegeneralflightdate.jpg</t>
         </is>
       </c>
       <c r="O4" s="1" t="inlineStr">
         <is>
-          <t>collected in lat spring to early fall 2000 [sic]. Detailed photodate information is not available.</t>
+          <t>2000-06-26 (callout label on the peach block containing cells t27r03, t27r04, t27r05, t28r04, t28r05). The live SDC page: 'Detailed photodate information is not available. A general overview at the township-level for data capture dates can interpolated from https://www5.kingcounty.gov/sdc/raster/ortho/images/ortho2000emergegeneralflightdate.jpg'</t>
         </is>
       </c>
       <c r="P4" s="1" t="inlineStr">
         <is>
-          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 18. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). Sensor Kodak DSC460CIR: no blue light recorded, all three held bands NIR-contaminated (Retractions). Wayback target for an agent: https://www5.kingcounty.gov/sdc/raster/ortho/images/ortho2000emergegeneralflightdate.jpg (404 live).</t>
+          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 18. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). The graphic 404s live; the ONLY Wayback capture (CDX domain search on metrokc.gov, capture 20081010173648) was read by the agent and re-read by the session lead (qc/imagery_date_evidence/king2000/). Edmonds township identity from BLM PLSS (T27N R03E at -122.3775,47.8107; T27N R04E at -122.3150,47.8100). Per-tile YYYYMMDD dates once existed in vendor filenames but King renamed tiles to tileXX.tif; the surviving index is emerge_nat.dbf. Sensor Kodak DSC460CIR: 'Blue light is outside the filter's bandpass, so that none of the incident blue light reaches the sensor' (archived EmergeCIR FGDC).</t>
         </is>
       </c>
       <c r="Q4" s="1" t="inlineStr">
@@ -12565,9 +12565,21 @@
           <t>grid/true MEASURED; effective MEASURED (Effective_Resolution); native PUBLISHED</t>
         </is>
       </c>
-      <c r="R4" s="1" t="inlineStr"/>
-      <c r="S4" s="1" t="inlineStr"/>
-      <c r="T4" s="1" t="inlineStr"/>
+      <c r="R4" s="1" t="inlineStr">
+        <is>
+          <t>2000-05-24 to 2000-09-23 (countywide project window, Currentness_Reference: Acquisition date)</t>
+        </is>
+      </c>
+      <c r="S4" s="1" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20040102162255if_/http://www.metrokc.gov/gis/sdc/raster/ortho/Ortho2000EmergeCIRMetadata.html</t>
+        </is>
+      </c>
+      <c r="T4" s="1" t="inlineStr">
+        <is>
+          <t>Time_Period_of_Content: Time_Period_Information: Range_of_Dates/Times: Beginning_Date:  20000524 Ending_Date:  20000923 Currentness_Reference:  Acquisition date</t>
+        </is>
+      </c>
       <c r="U4" s="1" t="inlineStr">
         <is>
           <t>held imagery</t>
@@ -12587,7 +12599,7 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>USGS High Resolution Orthoimagery Seattle/Tacoma 2002 (Selkirk Remote Sensing) as retiled by King County (IMAGE_Ortho2002USGSNAT)</t>
+          <t>USGS High Resolution Orthoimagery, Seattle/Tacoma 2002 (Homeland Security; flown by Selkirk Remote Sensing) as retiled by King County (IMAGE_Ortho2002USGSNAT)</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
@@ -12617,62 +12629,62 @@
       </c>
       <c r="I5" s="1" t="inlineStr">
         <is>
-          <t>33 acquired, delivered at 30.48 (1 ft)</t>
+          <t>33 acquired; delivered grid 0.98 ft = 29.9-30.0 cm (NOT 30.48): tile names '_02n098' = 98/100 ft; WA state copy LowPS 0.9846 ftUS = 30.01 cm</t>
         </is>
       </c>
       <c r="J5" s="1" t="inlineStr">
         <is>
+          <t>NOT FOUND for the Edmonds pixels. CONTESTED product-level date 2002-06-11 (two named Selkirk frames near Bellevue, ~24 km south)</t>
+        </is>
+      </c>
+      <c r="K5" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L5" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K5" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L5" s="1" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
       <c r="N5" s="1" t="inlineStr">
         <is>
-          <t>https://www5.kingcounty.gov/sdc/?Layer=IMAGE_Ortho2002USGSNAT</t>
+          <t>https://web.archive.org/web/20040225060658if_/http://www.metrokc.gov/gis/sdc/raster/ortho/Ortho2002USGSNATMetadata.html</t>
         </is>
       </c>
       <c r="O5" s="1" t="inlineStr">
         <is>
-          <t>(no acquisition statement on the page; catalog LastUpdated 2003-01-01 is maintenance metadata)</t>
+          <t>Description_of_Geographic_Extent: WRIA 8 Bounding_Coordinates: West_Bounding_Coordinate:  -122.05233309 East_Bounding_Coordinate:  -122.03790177 North_Bounding_Coordinate:  47.60259646 South_Bounding_Coordinate:  47.58876645</t>
         </is>
       </c>
       <c r="P5" s="1" t="inlineStr">
         <is>
-          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 18. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). Over Edmonds the cache serves the USGS/NGA Seattle-Tacoma product, NOT IMAGE_Ortho2002KCNAT (which is 'acquired in July 2002' but covers the county-only project). AGENT TARGET: USGS HRO Seattle/Tacoma FGDC metadata (EarthExplorer / TNM / Wayback) carries the per-project acquisition dates.</t>
+          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 18. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). The live SDC page for this layer returns HTTP 500 (2026-08-23, 3 attempts) - cite the archived FGDC. Over Edmonds the cache serves the USGS/NGA Seattle-Tacoma product, NOT IMAGE_Ortho2002KCNAT ('acquired in July 2002', county-only project). The archived FGDC's top-level block self-labels 'Beginning_Date: 20020611 Ending_Date: 20020611 Currentness_Reference: Publication date', while its lineage block labels the same date 'Aerial photography used in orthorectification' for frames 1192_6574_089 / 1193_6574_090 and 'Field control and ABGPS' 20020611-20020620. No per-frame or per-township index exists for 2002 (CDX sweep of both King hosts: the 2000 graphic is the only flight-date graphic ever published). HRO is retired from The National Map; ScienceBase has no project record. Remaining route: EarthExplorer HRO entity-level FGDC (M2M login).</t>
         </is>
       </c>
       <c r="Q5" s="1" t="inlineStr">
         <is>
-          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED (REST description: 'acquired at a resolution of 0.33 meter per pixel ... resampled to 1 foot per pixel')</t>
+          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED (archived FGDC + WA state service)</t>
         </is>
       </c>
       <c r="R5" s="1" t="inlineStr">
         <is>
-          <t>July 2002 (sibling product IMAGE_Ortho2002KCNAT — does NOT serve Edmonds)</t>
+          <t>2002-06-11 (product-level; CONTESTED currentness - see notes)</t>
         </is>
       </c>
       <c r="S5" s="1" t="inlineStr">
         <is>
-          <t>https://www5.kingcounty.gov/sdc/?Layer=IMAGE_Ortho2002KCNAT</t>
+          <t>https://web.archive.org/web/20040225060658if_/http://www.metrokc.gov/gis/sdc/raster/ortho/Ortho2002USGSNATMetadata.html</t>
         </is>
       </c>
       <c r="T5" s="1" t="inlineStr">
         <is>
-          <t>Natural color orthophotography acquired in July 2002</t>
+          <t>Source_Time_Period_of_Content: Time_Period_Information: Single_Date/Time: Calendar_Date:  20020611 Source_Citation_Abbreviation:  1192_6574_089 Source_Contribution:  Aerial photography used in orthorectification</t>
         </is>
       </c>
       <c r="U5" s="1" t="inlineStr">
@@ -12739,7 +12751,7 @@
       </c>
       <c r="L6" s="1" t="inlineStr">
         <is>
-          <t>unknown (no per-frame index exists before 2007)</t>
+          <t>unknown (no per-frame index exists before 2007; no finer date exists in King County's archive - established by CDX sweep, not assumed)</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
@@ -12749,27 +12761,39 @@
       </c>
       <c r="N6" s="1" t="inlineStr">
         <is>
+          <t>https://web.archive.org/web/20061008084602if_/http://www.metrokc.gov/gis/sdc/raster/ortho/Ortho2005AexpNatMetadata.html</t>
+        </is>
+      </c>
+      <c r="O6" s="1" t="inlineStr">
+        <is>
+          <t>Time_Period_of_Content: Time_Period_Information: Range_of_Dates/Times: Beginning_Date:  200507 Ending_Date:  200507 Currentness_Reference:  Ground Condition</t>
+        </is>
+      </c>
+      <c r="P6" s="1" t="inlineStr">
+        <is>
+          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 19. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). Held grid 20.1 cm vs 1 ft native = 1.5x oversampled, and the file resolves at 80.7 cm - coarser than 2000's nominal grid. Delivery (Aug 2006, portable hard drive) is NOT the flight date. The record's Bounding_Coordinates (North 47.74) are JUNK and would exclude Edmonds; the published extent graphic (Ortho2005AexpNatExtent.jpg, archived) shows Edmonds inside coverage.</t>
+        </is>
+      </c>
+      <c r="Q6" s="1" t="inlineStr">
+        <is>
+          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED</t>
+        </is>
+      </c>
+      <c r="R6" s="1" t="inlineStr">
+        <is>
+          <t>July 2005</t>
+        </is>
+      </c>
+      <c r="S6" s="1" t="inlineStr">
+        <is>
           <t>https://www5.kingcounty.gov/sdc/?Layer=IMAGE_Ortho2005AerialsExpressNAT</t>
         </is>
       </c>
-      <c r="O6" s="1" t="inlineStr">
+      <c r="T6" s="1" t="inlineStr">
         <is>
           <t>Year 2005 (July)</t>
         </is>
       </c>
-      <c r="P6" s="1" t="inlineStr">
-        <is>
-          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 19. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). Held grid 20.1 cm vs 1 ft native = 1.5x oversampled, and the file resolves at 80.7 cm — coarser than 2000's nominal grid.</t>
-        </is>
-      </c>
-      <c r="Q6" s="1" t="inlineStr">
-        <is>
-          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED</t>
-        </is>
-      </c>
-      <c r="R6" s="1" t="inlineStr"/>
-      <c r="S6" s="1" t="inlineStr"/>
-      <c r="T6" s="1" t="inlineStr"/>
       <c r="U6" s="1" t="inlineStr">
         <is>
           <t>held imagery</t>
@@ -12849,12 +12873,12 @@
       </c>
       <c r="O7" s="1" t="inlineStr">
         <is>
-          <t>SHOTDATE field, 1078 frames intersecting the city polygon (query 2026-08-23)</t>
+          <t>SHOTDATE field, 1078 frames intersecting the city polygon (query 2026-08-23; refetch-verified: field exists, all six days non-zero countywide)</t>
         </is>
       </c>
       <c r="P7" s="1" t="inlineStr">
         <is>
-          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 19. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). MEASURED 2026-08-23: King County public nadir-frame index queried with the Edmonds city POLYGON (City Boundry/Edmonds Boundry.shp, esriSpatialRelIntersects); counts are frames intersecting the city, not the mosaic's seam assignment. Which frame feeds each mosaic pixel is NOT recorded, so the mosaic over any given crown is one of these days, unknown which. SDC page: 'Final version 2007 (July)' — the August frames show 'July' is a simplification.</t>
+          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 19. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). MEASURED 2026-08-23: King County public nadir-frame index queried with the Edmonds city POLYGON (City Boundry/Edmonds Boundry.shp, esriSpatialRelIntersects); counts are frames intersecting the city, not the mosaic's seam assignment. Which frame feeds each mosaic pixel is NOT recorded, so the mosaic over any given crown is one of these days, unknown which. SDC page: 'Final version 2007 (July)' - the August frames show 'July' is a simplification.</t>
         </is>
       </c>
       <c r="Q7" s="1" t="inlineStr">
@@ -12956,7 +12980,7 @@
       </c>
       <c r="O8" s="1" t="inlineStr">
         <is>
-          <t>SHOTDATE/YYYYMMDD fields, 472 frames intersecting the city polygon (query 2026-08-23)</t>
+          <t>SHOTDATE/YYYYMMDD fields, 472 frames intersecting the city polygon (query 2026-08-23; refetch-verified)</t>
         </is>
       </c>
       <c r="P8" s="1" t="inlineStr">
@@ -13026,7 +13050,7 @@
       </c>
       <c r="J9" s="1" t="inlineStr">
         <is>
-          <t>2012-03-23 (30 photo centres, 13:25-13:44) and 2012-04-07 (45 photo centres, 12:08-12:46)</t>
+          <t>2012-03-23 (30 photo centres in the city, 13:25-13:44 local) and 2012-04-07 (45 photo centres, 12:08-12:46 local)</t>
         </is>
       </c>
       <c r="K9" s="1" t="inlineStr">
@@ -13036,7 +13060,7 @@
       </c>
       <c r="L9" s="1" t="inlineStr">
         <is>
-          <t>MULTI (2 days)</t>
+          <t>MULTI (2 days) - and the split is MEASURABLE per location: north Edmonds = Mar 23 geometry (6/7 sites), south Edmonds includes Apr 7 geometry (shadow solar dating, qc/imagery_date_evidence/shadow_dating_2020/ctrl_scored.csv)</t>
         </is>
       </c>
       <c r="M9" s="6" t="inlineStr">
@@ -13056,7 +13080,7 @@
       </c>
       <c r="P9" s="1" t="inlineStr">
         <is>
-          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 19. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). MEASURED 2026-08-23: King County public nadir-frame index queried with the Edmonds city POLYGON (City Boundry/Edmonds Boundry.shp, esriSpatialRelIntersects); counts are frames intersecting the city, not the mosaic's seam assignment. Which frame feeds each mosaic pixel is NOT recorded, so the mosaic over any given crown is one of these days, unknown which. Leaf-off to barely budding. Countywide window PUBLISHED on the SDC page (alt). Index RESOLUTION field = 1 (Apr 7) / 2 (Mar 23), units not stated.</t>
+          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 19. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). MEASURED 2026-08-23: King County public nadir-frame index queried with the Edmonds city POLYGON (City Boundry/Edmonds Boundry.shp, esriSpatialRelIntersects); counts are frames intersecting the city, not the mosaic's seam assignment. Which frame feeds each mosaic pixel is NOT recorded, so the mosaic over any given crown is one of these days, unknown which. Leaf-off to barely budding. Index times are LOCAL (13:35 UTC would put the sun below the horizon). Over the wider bbox the windows are 13:25-13:46 (Mar 23, n=61) and 11:51-13:11 (Apr 7, n=184). Index RESOLUTION field = 1 (Apr 7) / 2 (Mar 23), units not stated. Used as the POSITIVE CONTROL for shadow-geometry dating: 8/10 sites recovered an azimuth inside a real flight window (chance 0.197, P=6.9e-5).</t>
         </is>
       </c>
       <c r="Q9" s="1" t="inlineStr">
@@ -13158,7 +13182,7 @@
       </c>
       <c r="O10" s="1" t="inlineStr">
         <is>
-          <t>ShotDate/YYYYMMDD fields, 688 frames intersecting the city polygon (query 2026-08-23)</t>
+          <t>ShotDate/YYYYMMDD fields, 688 frames intersecting the city polygon (query 2026-08-23; refetch-verified)</t>
         </is>
       </c>
       <c r="P10" s="1" t="inlineStr">
@@ -13253,12 +13277,12 @@
       </c>
       <c r="O11" s="1" t="inlineStr">
         <is>
-          <t>ShotDate/YYYYMMDD fields, 701 frames intersecting the city polygon (query 2026-08-23)</t>
+          <t>ShotDate/YYYYMMDD fields, 701 frames intersecting the city polygon (query 2026-08-23; refetch-verified)</t>
         </is>
       </c>
       <c r="P11" s="1" t="inlineStr">
         <is>
-          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 20. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). MEASURED 2026-08-23: King County public nadir-frame index queried with the Edmonds city POLYGON (City Boundry/Edmonds Boundry.shp, esriSpatialRelIntersects); counts are frames intersecting the city, not the mosaic's seam assignment. Which frame feeds each mosaic pixel is NOT recorded, so the mosaic over any given crown is one of these days, unknown which. LEAF-OFF. This held file is the Pictometry KCNAT product; the three-way 2015 CONTEST (Apr 8/9/17 GeoTerra 2.7 in / Aug 7 4.8 in UFMP) belongs to the City of Edmonds 2015 SERVICE, a different product — see the CoE 2015 row.</t>
+          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 20. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). MEASURED 2026-08-23: King County public nadir-frame index queried with the Edmonds city POLYGON (City Boundry/Edmonds Boundry.shp, esriSpatialRelIntersects); counts are frames intersecting the city, not the mosaic's seam assignment. Which frame feeds each mosaic pixel is NOT recorded, so the mosaic over any given crown is one of these days, unknown which. LEAF-OFF. This held file is the Pictometry KCNAT product and is PIXEL-DISTINCT from the City of Edmonds 2015 basemap (tile correlation r=0.04-0.56 at 5 sites vs 0.99 control) - the 2015 CONTEST belongs to the CoE service row, not here. Weather note: 2015-02-15 was flown (CLR, 10 sm all day) with a maximum solar elevation of only 29.3 deg - a 30-deg sun floor is falsified by a known flight day.</t>
         </is>
       </c>
       <c r="Q11" s="1" t="inlineStr">
@@ -13348,12 +13372,12 @@
       </c>
       <c r="O12" s="1" t="inlineStr">
         <is>
-          <t>ShotDate/YYYYMMDD fields, 710 frames intersecting the city polygon (query 2026-08-23)</t>
+          <t>ShotDate/YYYYMMDD fields, 710 frames intersecting the city polygon (query 2026-08-23; an independent re-query returned 695, all 15 missing on May 10 - residual geometry handling, same days)</t>
         </is>
       </c>
       <c r="P12" s="1" t="inlineStr">
         <is>
-          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 20. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). MEASURED 2026-08-23: King County public nadir-frame index queried with the Edmonds city POLYGON (City Boundry/Edmonds Boundry.shp, esriSpatialRelIntersects); counts are frames intersecting the city, not the mosaic's seam assignment. Which frame feeds each mosaic pixel is NOT recorded, so the mosaic over any given crown is one of these days, unknown which. Resolves the May 18 discrepancy in MASTER: May 18 frames (n=215) fall inside the wider bbox -122.42,47.76,-122.32,47.87 but outside the city polygon. Countywide capture window 2017-02-17 to 2017-10-30 (PUBLISHED, SDC index change history).</t>
+          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 20. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). MEASURED 2026-08-23: King County public nadir-frame index queried with the Edmonds city POLYGON (City Boundry/Edmonds Boundry.shp, esriSpatialRelIntersects); counts are frames intersecting the city, not the mosaic's seam assignment. Which frame feeds each mosaic pixel is NOT recorded, so the mosaic over any given crown is one of these days, unknown which. Resolves the May 18 discrepancy in MASTER: May 18 frames (n=215) fall inside the wider bbox -122.42,47.76,-122.32,47.87 but outside the city polygon. Countywide capture 'from mid-February through October of 2017' (gisandyou.org, King County GIS). Frame counts track flyable hours (May 4 fog until 09:53 + afternoon thunderstorm -&gt; n=16; May 9/10 clear 08:53-16:53 -&gt; n=192/364). This file is the SAME ORTHOMOSAIC as 2017_coe_rgb.tif (see that row).</t>
         </is>
       </c>
       <c r="Q12" s="1" t="inlineStr">
@@ -13443,7 +13467,7 @@
       </c>
       <c r="O13" s="1" t="inlineStr">
         <is>
-          <t>ShotDate field (date only, no time), 1234 frames intersecting the city polygon (query 2026-08-23)</t>
+          <t>ShotDate field (date only; the layer carries Time_UTC/Time_PDT separately), 1234 frames intersecting the city polygon (query 2026-08-23; refetch-verified)</t>
         </is>
       </c>
       <c r="P13" s="1" t="inlineStr">
@@ -13538,7 +13562,7 @@
       </c>
       <c r="O14" s="1" t="inlineStr">
         <is>
-          <t>ShotDate field, 662 frames intersecting the city polygon (query 2026-08-23)</t>
+          <t>ShotDate field, 662 frames intersecting the city polygon (query 2026-08-23; refetch-verified)</t>
         </is>
       </c>
       <c r="P14" s="1" t="inlineStr">
@@ -13633,12 +13657,12 @@
       </c>
       <c r="O15" s="1" t="inlineStr">
         <is>
-          <t>ShotDate field, 1125 frames intersecting the city polygon (query 2026-08-23)</t>
+          <t>ShotDate field, 1125 frames intersecting the city polygon (query 2026-08-23; refetch-verified)</t>
         </is>
       </c>
       <c r="P15" s="1" t="inlineStr">
         <is>
-          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 20. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). MEASURED 2026-08-23: King County public nadir-frame index queried with the Edmonds city POLYGON (City Boundry/Edmonds Boundry.shp, esriSpatialRelIntersects); counts are frames intersecting the city, not the mosaic's seam assignment. Which frame feeds each mosaic pixel is NOT recorded, so the mosaic over any given crown is one of these days, unknown which.</t>
+          <t>Held pixels are an export of the KingCo_Aerial_YYYY ArcGIS tile cache (gismaps.kingcounty.gov), EPSG:3857, JPEG-quantised; grid is exactly Web-Mercator LOD 20. In-file metadata: NONE (sweep 2026-08-23: no DateTime/Software/XMP/IPTC/EXIF/GDAL_METADATA in any held raster). MEASURED 2026-08-23: King County public nadir-frame index queried with the Edmonds city POLYGON (City Boundry/Edmonds Boundry.shp, esriSpatialRelIntersects); counts are frames intersecting the city, not the mosaic's seam assignment. Which frame feeds each mosaic pixel is NOT recorded, so the mosaic over any given crown is one of these days, unknown which. A 2025 index (ORTHO_IMAGE25_AREA_3074, 'Index to 2025 Pictometry nadir images', 3 in west / 6 in east) now exists on the same org and was NOT queried over Edmonds - a follow-up would date 2025 the same way.</t>
         </is>
       </c>
       <c r="Q15" s="1" t="inlineStr">
@@ -13680,7 +13704,7 @@
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>Hexagon Imagery Program (HXIP) via Snohomish County Imagery/Aerial_2016 ImageServer</t>
+          <t>Hexagon Imagery Program (HXIP; 'Seattle' Urban Area Coverage tier of the WA Statewide Imagery Consortium) via Snohomish County Imagery/Aerial_2016 ImageServer (mosaic gdb HXIP_2016_SNOHOMISH.gdb)</t>
         </is>
       </c>
       <c r="D16" s="1" t="inlineStr">
@@ -13710,22 +13734,22 @@
       </c>
       <c r="I16" s="1" t="inlineStr">
         <is>
-          <t>30.48 (1 ft): county mosaic-catalog LowPS=1 and item pixelSizeX=1 for every primary tile over Edmonds (MEASURED 2026-08-23); the 2016 consortium 6-in (15 cm) buy-up exists over Edmonds but is NOT what the county serves</t>
+          <t>30.48 (1 ft): county mosaic-catalog LowPS=1 and item pixelSizeX=1 for every primary tile over Edmonds (MEASURED); the consortium's 15 cm (6 in) 2016 product exists over Edmonds but the county serves a 1-ft delivery</t>
         </is>
       </c>
       <c r="J16" s="1" t="inlineStr">
         <is>
-          <t>2016-08-11 (16:52) and 2016-08-12 (09:05, 09:30) — WA consortium 2016 6-in footprints over Edmonds</t>
+          <t>2016-08-12 morning (consortium sorties 09:05 / 09:30 PDT; a 09:50 sortie also lies within the city bbox) - CONDITIONAL on the county 1-ft product being the same flight as the dated 15 cm consortium product. The 2016-08-11 16:52 sortie is EXCLUDED for the held extent (shadows point WNW = morning sun)</t>
         </is>
       </c>
       <c r="K16" s="1" t="inlineStr">
         <is>
-          <t>window of 2 days, 3 sorties</t>
+          <t>window of 2 days by the consortium labels (Aug 11-12); held pixels consistent with Aug 12 only</t>
         </is>
       </c>
       <c r="L16" s="1" t="inlineStr">
         <is>
-          <t>MULTI (2 days / 3 sorties over the city; footprint = quarter-quarter quads)</t>
+          <t>consortium labels: MULTI (2 days, 3-4 sorties over the city); held file: shadow azimuth uniformly morning (283-295 deg over 24 windows, R=1.00) - consistent with a single morning, single date NOT proven</t>
         </is>
       </c>
       <c r="M16" s="7" t="inlineStr">
@@ -13740,12 +13764,12 @@
       </c>
       <c r="O16" s="1" t="inlineStr">
         <is>
-          <t>SDATE '08/11/2016 16:52' (SUNEL 31) / '08/12/2016 09:05' (SUNEL 34) / '08/12/2016 09:30' (SUNEL 37), THEMENAME hxip_m_4712213/4712214_*_10_15, 11 footprints intersecting the city bbox</t>
+          <t>SDATE '08/11/2016 16:52' (SUNEL 31) / '08/12/2016 09:05' (SUNEL 34) / '08/12/2016 09:30' (SUNEL 37), THEMENAME hxip_m_4712213/4712214_*_10_15; city-centroid point query returns hxip_m_4712213_se2_10_15, SDATE '08/12/2016 09:30', SUNEL 37, ACCURACY '0.68m (ce 95%)'</t>
         </is>
       </c>
       <c r="P16" s="1" t="inlineStr">
         <is>
-          <t>Held file = export of the county service (window means identical to exportImage, 2026-08-23) and pixel-DISTINCT from Aerial_2015 and Aerial_2017. Why INFERRED not PUBLISHED: the dated footprints are the 15 cm consortium product; the county's 1-ft tiles are a different delivery of (presumably) the same flight — the county mosaic was built from a geodatabase literally named HXIP_2015_Snohomishv3 (service /info/metadata lineage), so the 2015-08-07 HXIP 1-ft flight was a live alternative until the pixel test excluded it. OPEN: held-file shadows in the footprint labelled 16:52 point WEST (morning), so either that SDATE is UTC (=09:52 PDT) or the county product is a different sortie. Geocortex blurb 'acquired in August 2016' is mis-titled '2017 Aerial Photos'.</t>
+          <t>Held file = export of the county service (window means identical to exportImage) and pixel-DISTINCT from Aerial_2015 and Aerial_2017 (MEASURED). SDATE is LOCAL clock time: a 7034-footprint fit of published SUNEL vs pvlib gives RMSE 6.9 deg for UTC-7 vs 55.6 for UTC, and 09:05 read as UTC puts the sun 26 deg below the horizon. The county gdb is HXIP_2016_SNOHOMISH.gdb (the 'HXIP_2015' tokens in the lineage are a stale parent-folder / dataset-name carry-over, not 2015 imagery); the 2015-08-07 flight is excluded three ways (pixel comparison, afternoon vs morning shadows, lineage). 6-in coverage reached Edmonds because it lies inside the Valtus/Hexagon 'Seattle' UAC polygon, not via a county buy-up. The Geocortex blurb 'acquired in August 2016 as part of a Washington Statewide Imagery consortium. Pixel size of the raster is 6 inch' sits on a layer titled '2017 Aerial Photos' and contradicts the county's 1-ft tiles - CONTESTED, month-level corroboration only. Both Aug 11 and Aug 12 2016 were flyable at all three ASOS stations (Aug 11 morning marine stratus at KPAE only). C-CAP 2016 Snohomish (InPort 53263) says its source imagery is 'NAIP ... summer 2016' but no WA NAIP 2016 exists - most plausibly this HXIP flight. Held file is a study-area CROP (lon -122.404..-122.316, lat 47.783..47.828).</t>
         </is>
       </c>
       <c r="Q16" s="1" t="inlineStr">
@@ -13755,7 +13779,7 @@
       </c>
       <c r="R16" s="1" t="inlineStr">
         <is>
-          <t>2015-08-07 15:31 (HXIP 2015 1-ft flight; EXCLUDED by pixel comparison against Aerial_2015)</t>
+          <t>2015-08-07 15:31 (HXIP 2015 1-ft flight = the NAIP 2015 delivery; EXCLUDED for this file)</t>
         </is>
       </c>
       <c r="S16" s="1" t="inlineStr">
@@ -13787,7 +13811,7 @@
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>HXIP via Snohomish County Imagery/Aerial_2021 ImageServer</t>
+          <t>HXIP via Snohomish County Imagery/Aerial_2021 ImageServer (mosaic gdb HXIP_2021_SNOHOMISH.gdb - a Hexagon delivery, not EagleView)</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
@@ -13827,12 +13851,12 @@
       </c>
       <c r="K17" s="1" t="inlineStr">
         <is>
-          <t>window of 140 days</t>
+          <t>window of 140 days (weather trims to 108 feasible days; 18 late days never reach 30 deg sun)</t>
         </is>
       </c>
       <c r="L17" s="1" t="inlineStr">
         <is>
-          <t>unknown (countywide window only)</t>
+          <t>unknown; held crop flown in the AFTERNOON (shadow azimuth 67-91 deg = sun at 247-256 deg, uniform over 24 windows) - a time-of-day constraint, not a date</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
@@ -13852,7 +13876,7 @@
       </c>
       <c r="P17" s="1" t="inlineStr">
         <is>
-          <t>AGENT TARGET: a WA consortium 2021 flight-date footprint layer (as exists for 2015-2020) would narrow this to days. Service metadata carries no date (sweep 2026-08-23).</t>
+          <t>CLOSED LEADS: no WA consortium flight-date layer exists for 2021 or later (all 68 WAGeoservices services + 225 items enumerated; series ends 2020); the mosaic-catalog schema has no date field at all; WA NAIP 2021 does not cover quad 47122 (eastern WA only), so no NAIP ride-along date. Remaining route: the Hexagon flight log via Snohomish County DoIT, or the consortium contact (Joanne Markert, WA OCIO). Weather elimination (ASOS KPAE+KSEA+KBFI, criterion calibrated to 46/46 known Edmonds flight days; 2021-06-25..11-11): 32 of 140 days eliminated; longest feasible blocks Jul 22-Aug 6, Jul 2-15, Aug 9-19. ELIMINATES ONLY - no surviving day is favoured. Per-day table: qc/imagery_date_evidence/weather/flyable_days.csv.</t>
         </is>
       </c>
       <c r="Q17" s="1" t="inlineStr">
@@ -13882,7 +13906,7 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>City of Edmonds Basemap/2017_Aerial_Cached (source raster 2017_Aerial.tif, 0.25 ftUS EPSG:2285); acquirer NOT ESTABLISHED</t>
+          <t>City of Edmonds Basemap/2017_Aerial_Cached (source raster 2017_Aerial.tif, 0.25 ftUS EPSG:2285, JPEG); CONTENT = King County IMAGE_Ortho2017KCNAT (Pictometry International, 3-in 'Neighborhood' tier covering southwestern Snohomish County) - MEASURED identity</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
@@ -13912,52 +13936,64 @@
       </c>
       <c r="I18" s="1" t="inlineStr">
         <is>
-          <t>7.62 (0.25 ftUS source raster)</t>
+          <t>7.62 (0.25 ftUS source raster; service pixelSizeX 0.07620015240030481 m = 0.250000 ftUS exactly)</t>
         </is>
       </c>
       <c r="J18" s="1" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>2017-05-04 to 2017-05-10 (5 days over the city: May 4 n=16, May 6 90, May 8 48, May 9 192, May 10 364) - transferred from the King County per-frame index because the two files are the SAME ORTHOMOSAIC</t>
         </is>
       </c>
       <c r="K18" s="1" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>window of 7 days, 5 flight days</t>
         </is>
       </c>
       <c r="L18" s="1" t="inlineStr">
         <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="M18" s="5" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
+          <t>MULTI (5 days)</t>
+        </is>
+      </c>
+      <c r="M18" s="6" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
         </is>
       </c>
       <c r="N18" s="1" t="inlineStr">
         <is>
-          <t>https://weblink.edmondswa.gov/WebLink/0/edoc/1654952/</t>
+          <t>https://services.arcgis.com/Ej0PsM5Aw677QF1W/arcgis/rest/services/ORTHO_IMAGE17_AREA_2685/FeatureServer/0/query</t>
         </is>
       </c>
       <c r="O18" s="1" t="inlineStr">
         <is>
-          <t>In 2017 flyovers and imagery was done by the consultant who did the public engagement, PlanIt Geo, for Pierce, Snohomish and King Counties as part of a stormwater modeling project.</t>
+          <t>Identity MEASURED 2026-08-23: held 2017_coe_rgb.tif (2x boxcar-downsampled) vs 2017_king_rgb.tif over a 12x12 grid on the city polygon, 66 valid 512-px windows -&gt; r min 0.9568, p5 0.9786, median 0.9923, max 0.9966, MAE median 3.54 DN; live services 2017_Aerial_Cached vs KingCo_Aerial_2017 LOD-20 tiles at 5 sites r = 0.9876-0.9935. Identical vehicles in identical stalls and identical building relief displacement -&gt; same orthorectification, not merely the same flight.</t>
         </is>
       </c>
       <c r="P18" s="1" t="inlineStr">
         <is>
-          <t>The quote (council minutes 2023-07-25 p.15) is WEAK: conflates collector with analytics consultant. Candidate: King County 2017 flight 2017-05-04..05-10 over Edmonds (MEASURED on 2017_king_rgb.tif) — attribution to the city file UNPROVEN; Snohomish Aerial_2017 is a 1-ft HXIP product (2017-08-15/21) and cannot be a 3-in source. AGENT TARGET: 2017 CoE contract/budget line, sibling products, neighbour cities.</t>
+          <t>Retires the 8.5-month candidate window and the council-minutes line (2023-07-25 p.15, 'PlanIt Geo ... 2017 flyovers') as evidence - the 2019 UFMP was written by Davey Resource Group and its canopy work used Aug 2015 imagery; PlanIt Geo appears nowhere in it. No City of Edmonds document naming the 2017 vendor was found; attribution rests on measured pixel identity plus King County's published coverage statement (alt). Snohomish County's own 2017 product is a 1-ft HXIP flight (2017-08-15/21) and cannot be a 3-in source. Grid note: the held grid is exactly LOD 21, which King's tile endpoint does not serve (404 at L21) but Edmonds' does - consistent with a city-service export. Method detail: qc/imagery_date_evidence/coe2017_identity/.</t>
         </is>
       </c>
       <c r="Q18" s="1" t="inlineStr">
         <is>
-          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED (service source-raster XML)</t>
-        </is>
-      </c>
-      <c r="R18" s="1" t="inlineStr"/>
-      <c r="S18" s="1" t="inlineStr"/>
-      <c r="T18" s="1" t="inlineStr"/>
+          <t>grid/true MEASURED; effective MEASURED; native MEASURED (live service)</t>
+        </is>
+      </c>
+      <c r="R18" s="1" t="inlineStr">
+        <is>
+          <t>mid-February through October 2017 (countywide), with SW Snohomish at 3 in</t>
+        </is>
+      </c>
+      <c r="S18" s="1" t="inlineStr">
+        <is>
+          <t>https://gisandyou.org/2018/05/25/2017-aerial-imagery-in-imap/</t>
+        </is>
+      </c>
+      <c r="T18" s="1" t="inlineStr">
+        <is>
+          <t>The imagery was captured by Pictometry International Corp. from mid-February through October of 2017. The original photos have a resolution of 3 inches per pixel ("Neighborhood" scale in Pictometry terminology) over urbanized, western King County ... Also covered at the Neighborhood resolution level in the 2017 imagery are southwestern Snohomish County</t>
+        </is>
+      </c>
       <c r="U18" s="1" t="inlineStr">
         <is>
           <t>held imagery</t>
@@ -13977,7 +14013,7 @@
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>City of Edmonds Basemap/2020_Aerial_Cached; source = Snohomish County 2020 EagleView/Pictometry regional project (WASNOH20_3in) per the 2021 ILA</t>
+          <t>City of Edmonds Basemap/2020_Aerial_Cached (MrSID/MG4 mosaic, GeoExpress 10.0.1.5035, input GeoTIFF set 665,235,977,256 B); source = Snohomish County 2020 EagleView/Pictometry regional project WASNOH20_3in per the 2021 ILA; product identity corroborated by Everett's copy ('Aerial Photos 2020 Pictometry Mosiac 3 inch resolution urban areas', 0.25 ftUS)</t>
         </is>
       </c>
       <c r="D19" s="1" t="inlineStr">
@@ -14007,22 +14043,22 @@
       </c>
       <c r="I19" s="1" t="inlineStr">
         <is>
-          <t>7.62 (0.25 ftUS; county Aerial_2020 LowCellSize 0.25, dimResol 0.250000 ftUS)</t>
+          <t>7.62 (0.25 ftUS; county Aerial_2020 LowCellSize 0.25, dimResol 0.250000 ftUS; Everett Image2020jp2 pixelSizeX 0.25 in EPSG:2285)</t>
         </is>
       </c>
       <c r="J19" s="1" t="inlineStr">
         <is>
-          <t>2020-04-13 to 2020-07-13</t>
+          <t>2020-04-13 to 2020-07-13 (county window; the single published window is the UNION of the 3-in urban and 9-in rural sub-projects - unlike 2022/2024 the county did not publish them separately). Shadow solar geometry excludes the head: 2020-04-25 to 07-13 survive (80 of 92 days)</t>
         </is>
       </c>
       <c r="K19" s="1" t="inlineStr">
         <is>
-          <t>window of 92 days</t>
+          <t>window of 80-92 days</t>
         </is>
       </c>
       <c r="L19" s="1" t="inlineStr">
         <is>
-          <t>unknown — whether the Edmonds AOI is single- or multi-date is UNRESOLVED and outranks the date</t>
+          <t>CONSISTENT WITH ONE CONTINUOUS PASS, single date NOT PROVEN: 10 QC-passing sites of 34 on a ~850 m city-wide grid give sun azimuths 120.8-192.5 deg = local times ~10:22-13:39 PDT straddling solar noon, increasing monotonically east-to-west (az vs lon r=-0.75, p=0.013; permutation p=0.026) - the signature of successive flight lines in one pass, not of day-blocks. Not excluded: several dates each flown at the same time of day.</t>
         </is>
       </c>
       <c r="M19" s="7" t="inlineStr">
@@ -14042,12 +14078,12 @@
       </c>
       <c r="P19" s="1" t="inlineStr">
         <is>
-          <t>Chain: ILA 2021 (Laserfiche id 1462454) Work Order p.14 'Upon completion of the 2020, 2022 and 2024 EagleView regional aerial imagery acquisition projects ... County will provide Edmonds with orthogonal imagery'; city service keyProperties carry NO acquisition date (MrSID/MG4 mosaic lost it). The window is PUBLISHED for the county product; the link to the city file is documented by contract but inferential. DEFINITIVE PIN = EagleView flight log / photo-centre index via Snohomish County DoIT (PRR citing Contract Routing Form No. 20210127) or a CONNECTExplorer capture-date screenshot (city holds up to 10 accounts).</t>
+          <t>ILA 2021 (Laserfiche id 1462454, repo=Edmonds) Work Order p.14: 'Upon completion of the 2020, 2022 and 2024 EagleView regional aerial imagery acquisition projects ... County will provide Edmonds with orthogonal imagery for Edmonds's identified area of interest'. Contract vehicle for a records request: King County RFP 1166-18-PCR (EagleView Technology Corp) via Snohomish County Piggyback PB-19-14BC (Legistar matter 2024-1168). DEFINITIVE PIN = EagleView flight log / photo-centre index via Snohomish County DoIT (Viggo Forde), or a CONNECTExplorer capture-date screenshot (Edmonds holds up to ten accounts under the ILA). City keyProperties (correct endpoint &lt;ImageServer&gt;/keyProperties?f=json; /info/keyProperties 400s on this server, positive control Edmonds_Marsh_2018 returns acquisitionStartDate 2018-08-01T16:22:13+00:00 / End 16:52:13) carry NO date: IMAGE__MODIFICATIONS 'COMPRESSED EMBEDDED MASKED MOSAICKED' - a validated null. Everett's 2020 copy is JPEG2000 and also carries no date; no 2020 MrSID twin with a surviving date was found. A per-frame index CANNOT exist on the county service (mosaic catalog = two whole-project items WASNOH20_3in / WASNOH20_9in). HAZARD: a SECOND 2020 acquisition covers Edmonds - the WA consortium 6-in Hexagon/ADS100 flight of 2020-08-27/28 (program window 2020-08-03..09-06) - DO NOT borrow its date (see context row). Shadow dating (qc/imagery_date_evidence/shadow_dating_2020/): azimuth is reliable (2012 control 8/10 in-window), elevation reads LOW and saturates above ~45 deg, so 2020 elevations are lower bounds - hence no calendar date. 2020 ortho co-registered to 2012 within &lt;=1.5 WM m. Weather elimination (ASOS KPAE+KSEA+KBFI, criterion calibrated to 46/46 known Edmonds flight days; 2020-04-13..07-13): 22 of 92 days eliminated; longest feasible blocks May 7-15 (9 d), Apr 13-17, May 26-30, Jun 1-5, Jun 22-26. ELIMINATES ONLY - no surviving day is favoured. Per-day table: qc/imagery_date_evidence/weather/flyable_days.csv.</t>
         </is>
       </c>
       <c r="Q19" s="1" t="inlineStr">
         <is>
-          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED (county service)</t>
+          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED (county + Everett services)</t>
         </is>
       </c>
       <c r="R19" s="1" t="inlineStr">
@@ -14057,7 +14093,7 @@
       </c>
       <c r="S19" s="1" t="inlineStr">
         <is>
-          <t>https://weblink.edmondswa.gov/WebLink/DocView.aspx?id=1462454&amp;dbid=0&amp;repo=EdmondsWA</t>
+          <t>https://weblink.edmondswa.gov/WebLink/DocView.aspx?id=1462454&amp;dbid=0&amp;repo=Edmonds</t>
         </is>
       </c>
       <c r="T19" s="1" t="inlineStr">
@@ -14084,7 +14120,7 @@
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>City of Edmonds Basemap/2022_Aerial_Cached; source = Snohomish County 2022 regional project (WASNOH22_3in) per the 2021 ILA</t>
+          <t>City of Edmonds Basemap/2022_Aerial_Cached; = Snohomish County 2022 regional project WASNOH22_3in. IDENTITY MEASURED: the Edmonds and Everett 2022 MrSIDs are the same county encode (identical input-set byte count 675,609,635,568 B, GeoExpress 10.0.1.5035, EPSG:2285 ftUS geokeys)</t>
         </is>
       </c>
       <c r="D20" s="1" t="inlineStr">
@@ -14114,12 +14150,12 @@
       </c>
       <c r="I20" s="1" t="inlineStr">
         <is>
-          <t>7.62 (0.25 ftUS; county Aerial_2022 LowCellSize 0.25; MrSID input GeoTIFF geokeys EPSG:2285 ftUS)</t>
+          <t>7.62 (0.25 ftUS; county Aerial_2022 LowCellSize 0.25; MrSID input GeoTIFF geokeys 'Linear_Foot_US_Survey' / 2285)</t>
         </is>
       </c>
       <c r="J20" s="1" t="inlineStr">
         <is>
-          <t>2022-04-06 to 2022-07-11 (urban 3 in)</t>
+          <t>2022-04-06 to 2022-07-11 (urban 3 in); the rural 9-in sub-project ran 2022-05-31 to 08-11 and does not apply to Edmonds</t>
         </is>
       </c>
       <c r="K20" s="1" t="inlineStr">
@@ -14132,9 +14168,9 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="M20" s="7" t="inlineStr">
-        <is>
-          <t>INFERRED</t>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="N20" s="1" t="inlineStr">
@@ -14144,32 +14180,32 @@
       </c>
       <c r="O20" s="1" t="inlineStr">
         <is>
-          <t>The 2022 3 inch resolution aerial photos in the urban areas, were captured between April 6, 2022 and July, 11 2022.</t>
+          <t>The 2022 3 inch resolution aerial photos in the urban areas, were captured between April 6, 2022 and July, 11 2022. The 2022 9 inch resolution aerial photos in the rural areas, were captured between May, 31 2022 and August, 11 2022.</t>
         </is>
       </c>
       <c r="P20" s="1" t="inlineStr">
         <is>
-          <t>Same chain and same definitive pin as 2020 (one PRR covers 2020/2022/2024).</t>
+          <t>Upgraded INFERRED -&gt; PUBLISHED 2026-08-23: the window is published for a product whose identity with the held file is now measured (byte-count identity of the input set with Everett's Image2022_3in_sid, 'Aerial Photos 2022 Pictometry Mosaic 3 inch resolution urban areas'), not only contractual. Same definitive pin as 2020 (one PRR covers 2020/2022/2024). Weather elimination (ASOS KPAE+KSEA+KBFI, criterion calibrated to 46/46 known Edmonds flight days; 2022-04-06..07-11): 19 of 97 days eliminated (weakest of the four windows - a settled spring); longest feasible block May 16-28 (13 d). ELIMINATES ONLY - no surviving day is favoured. Per-day table: qc/imagery_date_evidence/weather/flyable_days.csv.</t>
         </is>
       </c>
       <c r="Q20" s="1" t="inlineStr">
         <is>
-          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED (county service)</t>
+          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED (county + Everett services)</t>
         </is>
       </c>
       <c r="R20" s="1" t="inlineStr">
         <is>
-          <t>(ILA text)</t>
+          <t>(Everett keyProperties - identity proof)</t>
         </is>
       </c>
       <c r="S20" s="1" t="inlineStr">
         <is>
-          <t>https://weblink.edmondswa.gov/WebLink/DocView.aspx?id=1462454&amp;dbid=0&amp;repo=EdmondsWA</t>
+          <t>https://gismaps.everettwa.gov/manarcgis/rest/services/Imagery/Image2022_3in_sid/ImageServer/keyProperties?f=json</t>
         </is>
       </c>
       <c r="T20" s="1" t="inlineStr">
         <is>
-          <t>Upon completion of the 2020, 2022 and 2024 EagleView regional aerial imagery acquisition projects ...</t>
+          <t>"IMAGE__ENCODING_APPLICATION":"GeoExpress 10.0.1.5035","IMAGE__FORMAT":"MrSID/MG4","IMAGE__INPUT_FILE_SIZE":"675609635568.000000","IMAGE__INPUT_FORMAT":"GeoTIFF" ... "IMAGE__MODIFICATIONS":"COMPRESSED EMBEDDED MASKED MOSAICKED"</t>
         </is>
       </c>
       <c r="U20" s="1" t="inlineStr">
@@ -14191,7 +14227,7 @@
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>City of Edmonds Basemap/2024_Aerial_Cached (Edmonds2024.sid); source = Snohomish County 2024 regional project (WASNOH24_3in) per the 2021 ILA</t>
+          <t>City of Edmonds Basemap/2024_Aerial_Cached (MapServer over Edmonds2024.sid - no ImageServer, so no keyProperties resource exists); source = Snohomish County 2024 regional project WASNOH24_3in per the 2021 ILA</t>
         </is>
       </c>
       <c r="D21" s="1" t="inlineStr">
@@ -14226,12 +14262,12 @@
       </c>
       <c r="J21" s="1" t="inlineStr">
         <is>
-          <t>2024-03-31 to 2024-05-31 (urban 3 in)</t>
+          <t>2024-03-31 to 2024-05-31 (urban 3 in); the rural 9-in sub-project ran 2024-03-16 to 06-09</t>
         </is>
       </c>
       <c r="K21" s="1" t="inlineStr">
         <is>
-          <t>window of 61 days</t>
+          <t>window of 62 days</t>
         </is>
       </c>
       <c r="L21" s="1" t="inlineStr">
@@ -14251,12 +14287,12 @@
       </c>
       <c r="O21" s="1" t="inlineStr">
         <is>
-          <t>The 2024 3 inch resolution aerial photos in the urban areas, were captured between March 31, 2024 and May, 31 2024.</t>
+          <t>The 2024 3 inch resolution aerial photos in the urban areas, were captured between March 31, 2024 and May, 31 2024. The 2024 9 inch resolution aerial photos in the rural areas, were captured between March, 16 2024 and June, 9 2024.</t>
         </is>
       </c>
       <c r="P21" s="1" t="inlineStr">
         <is>
-          <t>Same chain and same definitive pin as 2020.</t>
+          <t>Stays INFERRED: no neighbour city holds a 2024 county copy (Everett stops at 2022, Mukilteo at 2019, Lynnwood publishes none), so there is no 2024 analogue of the 2022 byte-identity proof. Same definitive pin as 2020. Weather elimination (ASOS KPAE+KSEA+KBFI, criterion calibrated to 46/46 known Edmonds flight days; 2024-03-31..05-31): 18 of 62 days eliminated (29%, strongest of the four); longest feasible block Apr 16-24 (9 d). ELIMINATES ONLY - no surviving day is favoured. Per-day table: qc/imagery_date_evidence/weather/flyable_days.csv.</t>
         </is>
       </c>
       <c r="Q21" s="1" t="inlineStr">
@@ -14271,7 +14307,7 @@
       </c>
       <c r="S21" s="1" t="inlineStr">
         <is>
-          <t>https://weblink.edmondswa.gov/WebLink/DocView.aspx?id=1462454&amp;dbid=0&amp;repo=EdmondsWA</t>
+          <t>https://weblink.edmondswa.gov/WebLink/DocView.aspx?id=1462454&amp;dbid=0&amp;repo=Edmonds</t>
         </is>
       </c>
       <c r="T21" s="1" t="inlineStr">
@@ -14298,7 +14334,7 @@
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>City of Edmonds (source raster Ed_Aerial_2015.tif, 0.25 ftUS, LZW)</t>
+          <t>City of Edmonds (source raster Ed_Aerial_2015.tif, 0.25 ftUS EPSG:2285, LZW); content INFERRED = 2015 Western Washington Regional Orthophotography (King County lead, 88 participants; prime GeoTerra, Edmonds frames flown by Valley Air and GeoTerra)</t>
         </is>
       </c>
       <c r="D22" s="1" t="inlineStr">
@@ -14328,52 +14364,64 @@
       </c>
       <c r="I22" s="1" t="inlineStr">
         <is>
-          <t>7.62 (0.25 ftUS source) — vs 6.86 (0.225 ft, GeoTerra consortium spec) vs 12.19 (4.8 in, UFMP)</t>
+          <t>&lt;= 6.86 flown (MAX_GSD 0.225 ft 'as planned' for all 346 Edmonds frames; two cameras at two altitudes both back-compute to ~6.6-6.9 cm), delivered at the 0.25 ft = 7.62 cm tier (service pixelSizeX 0.07620015240030481 m = 0.250000 ftUS)</t>
         </is>
       </c>
       <c r="J22" s="1" t="inlineStr">
         <is>
-          <t>CONTESTED: 2015-04-08/09/17 (GeoTerra consortium photo centres) vs 2015-02-15..03-08 (King Pictometry) vs 2015-08-07 (UFMP '4.8 in')</t>
+          <t>2015-04-08 (n=135 photo centres in the city polygon; Valley Air, UltraCam X, 14:13-15:04 PDT) and 2015-04-17 (n=32; GeoTerra, UltraCam Xp, 12:54-13:55 PDT). CONTEST largely resolved: the King Pictometry leg is EXCLUDED by pixel comparison, the 'Aug 7 2015' leg is a DIFFERENT dataset (NAIP/HXIP 2015-08-07), leaving the consortium dates; attribution of Ed_Aerial_2015.tif to the consortium remains INFERRED and the UFMP's '4.8 in' figure is unexplained</t>
         </is>
       </c>
       <c r="K22" s="1" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2 flight days (window of 10 days) for the consortium product</t>
         </is>
       </c>
       <c r="L22" s="1" t="inlineStr">
         <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="M22" s="5" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
+          <t>MULTI - two days, two vendors, two cameras within the city (flightlines 16002-16011 Zone 16 / 13007-13015 Zone 13)</t>
+        </is>
+      </c>
+      <c r="M22" s="7" t="inlineStr">
+        <is>
+          <t>INFERRED</t>
         </is>
       </c>
       <c r="N22" s="1" t="inlineStr">
         <is>
-          <t>(see Contradictions sheet; three sources)</t>
+          <t>https://services.arcgis.com/Ej0PsM5Aw677QF1W/arcgis/rest/services/ORTHO_IMAGE15C_POINT_2574/FeatureServer/0/query</t>
         </is>
       </c>
       <c r="O22" s="1" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>{"FILENAME": "13007_57226", "FRAME": 57226, ... "UTC_TIME": "19:35:08", "MAX_GSD__f": 0.225, "USED": "YES", "VENDOR": "GeoTerra", "CAMERA": "UltraCam Xp", "SSN": 10411033, ... "FLIGHTLINE": "13007", "ACQ_DATE": 1429228800000} (photo-centre layer; in-polygon N=167; 'It is a reference for the raw image scans, it is not a index for tiled ortho imagery')</t>
         </is>
       </c>
       <c r="P22" s="1" t="inlineStr">
         <is>
-          <t>Included so the contest stops contaminating the held 2015_king_rgb.tif row. Likely explanation: the UFMP canopy-assessment imagery is a different dataset from the city basemap. Edmonds signed the 2015 consortium agreement 2015-06-23 ($3,696.21).</t>
+          <t>Photo-centre DAYS are MEASURED; binding them to Ed_Aerial_2015.tif is INFERRED via (a) 0.25 ftUS cell size matching the consortium tier, (b) CRS NAD83 SP WA North ftUS, (c) Edmonds named in GeoTerra's participant table and the consortium agreement signed 2015-06-23 ($3,696.21), (d) leaf-off/high-sun spec matching the tiles. NOTE: no Apr 9 frames exist over Edmonds (the catalogue's 'Apr 8/9/17' was wrong); one Mar 26 frame sits just outside the polygon. King leg excluded: CoE 2015 vs KingCo_Aerial_2015 LOD-20 tiles r=0.036-0.557 at 5 sites vs r=0.988-0.994 for the CoE-2017/King-2017 control. 'Aug 7 2015 / 4.8 in' (UFMP 2019 p.26) traces to the Davey Resource Group 2018 UTC Assessment which names 'USDA, Farm Service Agency' = NAIP 2015 (2015-08-07, 1 m = the same Hexagon flight as the HXIP 1-ft consortium product); '4.8 in' matches no known 2015 product. Phenology caveat from the project's own survey report: 'the need to begin immediate image acquisition due an earlier than normal bud break' - Apr 8/17 is late in a leaf-off window. Vendor/camera cross-validated at serial-number level against the Flight Subcontractor PDF (UCX 60418665 / UCXp 10411033).</t>
         </is>
       </c>
       <c r="Q22" s="1" t="inlineStr">
         <is>
-          <t>grid PUBLISHED (service); native PUBLISHED (source-raster XML)</t>
-        </is>
-      </c>
-      <c r="R22" s="1" t="inlineStr"/>
-      <c r="S22" s="1" t="inlineStr"/>
-      <c r="T22" s="1" t="inlineStr"/>
+          <t>grid MEASURED (live service); native MEASURED (index MAX_GSD) + PUBLISHED (tier)</t>
+        </is>
+      </c>
+      <c r="R22" s="1" t="inlineStr">
+        <is>
+          <t>2015-08-07 15:31 (UFMP/Davey 'August 7th, 2015' imagery = NAIP/HXIP 2015, NOT the city basemap)</t>
+        </is>
+      </c>
+      <c r="S22" s="1" t="inlineStr">
+        <is>
+          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2015/wa_fgdc_2015/47122/m_4712214_sw_10_1_20150807.txt</t>
+        </is>
+      </c>
+      <c r="T22" s="1" t="inlineStr">
+        <is>
+          <t>Time_Period_of_Content: Time_Period_Information: Single_Date/Time: Calendar_Date: 20150807 Currentness_Reference: Ground Condition</t>
+        </is>
+      </c>
       <c r="U22" s="1" t="inlineStr">
         <is>
           <t>context (not held)</t>
@@ -14393,7 +14441,7 @@
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>USDA FSA NAIP WA 2019 (DOQQ m_4712213/m_4712214; flown by Hexagon under the 2019 program)</t>
+          <t>USDA FSA NAIP WA 2019 (DOQQ m_4712213/m_4712214; the WA consortium 2019 1-ft flight carries the same date, i.e. the Hexagon flight)</t>
         </is>
       </c>
       <c r="D23" s="1" t="inlineStr">
@@ -14438,7 +14486,7 @@
       </c>
       <c r="L23" s="1" t="inlineStr">
         <is>
-          <t>single (all Edmonds DOQQs carry 20191011)</t>
+          <t>single (all Edmonds DOQQs carry 20191011; consortium flight-area IDATE '2019 -10-11' at the city centroid)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
@@ -14453,12 +14501,12 @@
       </c>
       <c r="O23" s="1" t="inlineStr">
         <is>
-          <t>Time_Period_of_Content: Time_Period_Information: Single_Date/Time: Calendar_Date: 20191011</t>
+          <t>Time_Period_of_Content: Time_Period_Information: Single_Date/Time: Calendar_Date: 20191011 Currentness_Reference: Ground Condition</t>
         </is>
       </c>
       <c r="P23" s="1" t="inlineStr">
         <is>
-          <t>OCTOBER — weakens the 'NAIP is leaf-on by spec' assumption. Corroborated by the WA consortium 2019 1-ft flight-area layer IDATE '2019 -10-11'.</t>
+          <t>OCTOBER. No NAIP metadata record (2015/2017/2021 Digital Coast) contains any leaf-on/leaf-off statement - only 'peak crop growing conditions'; the 'NAIP is leaf-on by spec' assumption has no documentary basis.</t>
         </is>
       </c>
       <c r="Q23" s="1" t="inlineStr">
@@ -14466,9 +14514,21 @@
           <t>grid/true MEASURED; effective MEASURED; native PUBLISHED</t>
         </is>
       </c>
-      <c r="R23" s="1" t="inlineStr"/>
-      <c r="S23" s="1" t="inlineStr"/>
-      <c r="T23" s="1" t="inlineStr"/>
+      <c r="R23" s="1" t="inlineStr">
+        <is>
+          <t>2019-10-11</t>
+        </is>
+      </c>
+      <c r="S23" s="1" t="inlineStr">
+        <is>
+          <t>https://services.arcgis.com/jsIt88o09Q0r1j8h/arcgis/rest/services/2019_Statewide_imagery_consortium_1_foot_flight_areas/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="T23" s="1" t="inlineStr">
+        <is>
+          <t>{"FID": 23, "IDATE": "2019 -10-11"} (stray space verbatim)</t>
+        </is>
+      </c>
       <c r="U23" s="1" t="inlineStr">
         <is>
           <t>held imagery</t>
@@ -14548,12 +14608,12 @@
       </c>
       <c r="O24" s="1" t="inlineStr">
         <is>
-          <t>m_4712214_ne_10_060_20231007.tif (date field of the DOQQ file name, ISO metadata)</t>
+          <t>&lt;gmd:title&gt; m_4712214_sw_10_060_20231007.tif (date field of the DOQQ file name in the ISO metadata record)</t>
         </is>
       </c>
       <c r="P24" s="1" t="inlineStr">
         <is>
-          <t>OCTOBER. Held bands 1-3 byte-identical to rgb_2023, band 4 to ir_2023 (DataLake_Issues).</t>
+          <t>OCTOBER. Held bands 1-3 byte-identical to rgb_2023, band 4 to ir_2023 (DataLake_Issues). Context: NAIP 2021 over Edmonds exists (all 8 QQs STAC datetime 2021-07-13, INFERRED from file names - the FGDC sidecars for quad 47122 are absent from the Azure mirror).</t>
         </is>
       </c>
       <c r="Q24" s="1" t="inlineStr">
@@ -14578,12 +14638,12 @@
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>~2016 (lidar)</t>
+          <t>2016 (lidar)</t>
         </is>
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
-          <t>USGS 3DEP HAG via Planetary Computer, reprojected by the project</t>
+          <t>USGS 3DEP HAG via Planetary Computer, reprojected by the project; underlying lidar = USGS_LPC_WA_Western_North_2016 (QSI for USGS/WADNR)</t>
         </is>
       </c>
       <c r="D25" s="1" t="inlineStr">
@@ -14618,12 +14678,12 @@
       </c>
       <c r="J25" s="1" t="inlineStr">
         <is>
-          <t>2016-03-17 to 2017-06-06 (USGS/WADNR lidar collection)</t>
+          <t>2016-03-17 to 2016-09-30 (Western Washington 3DEP NORTH AOI; all 46 tiles over the city are North-block)</t>
         </is>
       </c>
       <c r="K25" s="1" t="inlineStr">
         <is>
-          <t>window of 15 months</t>
+          <t>window of 198 days</t>
         </is>
       </c>
       <c r="L25" s="1" t="inlineStr">
@@ -14643,12 +14703,12 @@
       </c>
       <c r="O25" s="1" t="inlineStr">
         <is>
-          <t>(collection window per IMAGERY_FACTS 8.1, sourced from InPort 51853 — REFETCH NEEDED)</t>
+          <t>Time Frame 2016-03-17 - 2017-06-06 / North: March 17 - Sept 30, 2016 / South: March 17, 2016 - June 6, 2017</t>
         </is>
       </c>
       <c r="P25" s="1" t="inlineStr">
         <is>
-          <t>UNITS TRAP #4: grid is 1.0 m in EPSG:3857 = 67.2 cm true ground at 47.81N, not 1 m. Row included for completeness; excluded from the imagery count.</t>
+          <t>UNITS TRAP #4: grid is 1.0 m in EPSG:3857 = 67.2 cm true ground at 47.81N, not 1 m. Narrowed from 15 months (whole project) to the North window by point-in-polygon on NOAA's tile index (46/46 tiles /north/). Reference raster, excluded from the imagery count.</t>
         </is>
       </c>
       <c r="Q25" s="1" t="inlineStr">
@@ -14656,9 +14716,21 @@
           <t>grid/true MEASURED; native PUBLISHED</t>
         </is>
       </c>
-      <c r="R25" s="1" t="inlineStr"/>
-      <c r="S25" s="1" t="inlineStr"/>
-      <c r="T25" s="1" t="inlineStr"/>
+      <c r="R25" s="1" t="inlineStr">
+        <is>
+          <t>2016-03-30 (INFERRED from the tile filename prefix 20160330_USGS_LPC_WA_Western_North_2016_q47122G4405 - a FILE NAME; 3/30/16 is a flight day for all three contractors in QSI report Table 3)</t>
+        </is>
+      </c>
+      <c r="S25" s="1" t="inlineStr">
+        <is>
+          <t>https://noaa-nos-coastal-lidar-pds.s3.amazonaws.com/laz/geoid18/6331/tileindex_wa2016_west_wa_m6331.gpkg</t>
+        </is>
+      </c>
+      <c r="T25" s="1" t="inlineStr">
+        <is>
+          <t>20160330_USGS_LPC_WA_Western_North_2016_q47122G4405_LAS_2018.copc.laz</t>
+        </is>
+      </c>
       <c r="U25" s="1" t="inlineStr">
         <is>
           <t>reference raster</t>
@@ -14668,87 +14740,87 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>ccap_2016_hires_lc_snohfull.tif</t>
+          <t>PSLC_2005/ (47 laz tiles)</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>2016 (C-CAP ref)</t>
+          <t>2005 (lidar)</t>
         </is>
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t>NOAA OCM C-CAP hi-res land cover, Snohomish County 2016 (InPort 53263)</t>
+          <t>Puget Sound LiDAR Consortium 2005 North Puget Sound Lowlands (Terrapoint), InPort 50149</t>
         </is>
       </c>
       <c r="D26" s="1" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>point cloud</t>
         </is>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>metre</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>EPSG:26910</t>
+          <t>NAD83(HARN) UTM 10N, NAVD88 GEOID18</t>
         </is>
       </c>
       <c r="G26" s="1" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.25 pts/m2 stated (~0.17 cross-checked)</t>
         </is>
       </c>
       <c r="H26" s="1" t="inlineStr">
         <is>
-          <t>n/a (thematic)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I26" s="1" t="inlineStr">
         <is>
-          <t>100 (1 m product)</t>
+          <t>n/a (2 m nominal spacing)</t>
         </is>
       </c>
       <c r="J26" s="1" t="inlineStr">
         <is>
-          <t>NOT FOUND (source-imagery date; InPort 53263 returns 'Catalog Item Not Retrievable')</t>
+          <t>2005-02-27 (Edmonds sub-project, 11 sq mi)</t>
         </is>
       </c>
       <c r="K26" s="1" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>single day</t>
         </is>
       </c>
       <c r="L26" s="1" t="inlineStr">
         <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="M26" s="5" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
+          <t>single (sub-project row)</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="N26" s="1" t="inlineStr">
         <is>
-          <t>https://www.fisheries.noaa.gov/inport/item/53263</t>
+          <t>https://www.fisheries.noaa.gov/inport/item/50149</t>
         </is>
       </c>
       <c r="O26" s="1" t="inlineStr">
         <is>
-          <t>Catalog Item Not Retrievable</t>
+          <t>project, area (sq mi), date(s) collected, vert. acc (cm), horiz acc. (cm), RMSE (m) - ... - Edmonds, 11, 2/27/2005, 25, 60, 0.100 - Mt. Lake Terrace, 4, 7/15/2005-9/15/2005, 25, 60, 0.100 - Mukilteo, 16, 2/27/2005, 25, 60, 0.100</t>
         </is>
       </c>
       <c r="P26" s="1" t="inlineStr">
         <is>
-          <t>AGENT TARGET: Wayback copy of InPort 53263 / the .img sidecar metadata (wa_snohomish_co_ccap_hr_landcover20190314.img). Reference raster, not an imagery acquisition.</t>
+          <t>LEAF-OFF (late February). Record-internal inconsistency: Mt. Lake Terrace sub-project dates run past the record's own Time Frame end (2005-07-15). Held at D:/edmonds-pipeline/Imagery/PSLC_2005 and Full_Image/PSLC_2005 (IMAGERY_FACTS 8.2).</t>
         </is>
       </c>
       <c r="Q26" s="1" t="inlineStr">
         <is>
-          <t>grid/true MEASURED; native PUBLISHED</t>
+          <t>density PUBLISHED</t>
         </is>
       </c>
       <c r="R26" s="1" t="inlineStr"/>
@@ -14756,24 +14828,24 @@
       <c r="T26" s="1" t="inlineStr"/>
       <c r="U26" s="1" t="inlineStr">
         <is>
-          <t>reference raster</t>
+          <t>reference lidar</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>ccap_2021_hires_lc.tif</t>
+          <t>ccap_2016_hires_lc_snohfull.tif</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>2020-21 (C-CAP v2 ref)</t>
+          <t>2016 (C-CAP ref)</t>
         </is>
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t>NOAA OCM C-CAP hi-res v2 'Refined' (Ecopia extraction, NV5 refinement)</t>
+          <t>NOAA OCM C-CAP hi-res land cover, Snohomish County 2016 (InPort 53263 - record RECOVERED as an InPort XML export on coast.noaa.gov; fisheries.noaa.gov still 403)</t>
         </is>
       </c>
       <c r="D27" s="1" t="inlineStr">
@@ -14803,42 +14875,42 @@
       </c>
       <c r="I27" s="1" t="inlineStr">
         <is>
-          <t>100 (1 m extraction from &lt;=30 cm imagery)</t>
+          <t>100 (1 m product)</t>
         </is>
       </c>
       <c r="J27" s="1" t="inlineStr">
         <is>
-          <t>2020-2021 vintage (source imagery dates not stated per pixel)</t>
+          <t>summer 2016 (source imagery, stated as NAIP) - CONTESTED: no WA NAIP 2016 exists (Azure NAIP v002/wa/ holds 2011, 2013, 2015, 2017, 2019, 2021, 2023 only)</t>
         </is>
       </c>
       <c r="K27" s="1" t="inlineStr">
         <is>
-          <t>year range</t>
+          <t>season</t>
         </is>
       </c>
       <c r="L27" s="1" t="inlineStr">
         <is>
-          <t>multi (mosaic of vendor imagery)</t>
-        </is>
-      </c>
-      <c r="M27" s="5" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="N27" s="1" t="inlineStr">
         <is>
-          <t>(lineage XML cc_wa_puget_2021_ccap_v2_hires_landcover.xml — URL to be re-fetched)</t>
+          <t>https://chs.coast.noaa.gov/htdata/raster1/landcover/bulkdownload/hires/wa/WA_Snohomish_2016_lc.xml</t>
         </is>
       </c>
       <c r="O27" s="1" t="inlineStr">
         <is>
-          <t>Initial 1m spatial resolution feature extraction for Impervious, Water, and Canopy (tree and scrub/shrub) mapping was conducted by Ecopia AI</t>
+          <t>The timeframe for this metadata is summer 2016. These maps are developed utilizing high resolution National Agriculture Imagery Program (NAIP) imagery, and can be used to track changes in the landscape through time.</t>
         </is>
       </c>
       <c r="P27" s="1" t="inlineStr">
         <is>
-          <t>GATE: published date without fetched URL+quote -&gt; downgraded. Reference raster, not an imagery acquisition. Date of the underlying imagery is the agent question.</t>
+          <t>Candidate reconciliation (INFERENCE): the 'summer 2016' imagery is the HXIP Aug 11-12 2016 flight (the WA consortium product is itself branded 'NAIP_2016' on AGOL), or NOAA used NAIP 2015 (2015-08-07) and labelled the product 2016 - UNRESOLVED. Traps in the record: &lt;start-date-time&gt;2016-01-01 is a year placeholder; &lt;publish-date&gt;2019-03-14 is publication. Ancillary: NGS MLLW orthoimagery 2014 for shore classes. Reference raster.</t>
         </is>
       </c>
       <c r="Q27" s="1" t="inlineStr">
@@ -14855,8 +14927,317 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>ccap_2021_hires_lc.tif</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>2021 (C-CAP v2 ref)</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>NOAA OCM C-CAP hi-res v2 'Refined' Puget Sound 2021 (InPort 79723; Ecopia extraction, NV5 refinement)</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>metre</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:26910</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="H28" s="1" t="inlineStr">
+        <is>
+          <t>n/a (thematic)</t>
+        </is>
+      </c>
+      <c r="I28" s="1" t="inlineStr">
+        <is>
+          <t>100 (1 m extraction from '30cm or better' imagery)</t>
+        </is>
+      </c>
+      <c r="J28" s="1" t="inlineStr">
+        <is>
+          <t>2021 (year only; 'Acquisition date of the Aerial Imagery')</t>
+        </is>
+      </c>
+      <c r="K28" s="1" t="inlineStr">
+        <is>
+          <t>year only</t>
+        </is>
+      </c>
+      <c r="L28" s="1" t="inlineStr">
+        <is>
+          <t>multi (mosaic of vendor imagery)</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="N28" s="1" t="inlineStr">
+        <is>
+          <t>https://ocmgeodatastor1.blob.core.windows.net/ccap/bulk_download/C-CAP_High-Resolution_Data/Refined_C-CAP_High-Resolution_Land_Cover_Classification/CONUS/wa_puget_2021_ccap_v2_hires_landcover.xml</t>
+        </is>
+      </c>
+      <c r="O28" s="1" t="inlineStr">
+        <is>
+          <t>&lt;currentness-reference&gt;Acquisition date of the Aerial Imagery&lt;/currentness-reference&gt; ... &lt;time-frame-type&gt;Discrete&lt;/time-frame-type&gt; &lt;start-date-time&gt;2021&lt;/start-date-time&gt; ... Initial 1m spatial resolution feature extraction for Impervious, Water, and Canopy (tree and scrub/shrub) mapping was conducted by Ecopia AI</t>
+        </is>
+      </c>
+      <c r="P28" s="1" t="inlineStr">
+        <is>
+          <t>The record was created 2026-04-28 and may post-date the held clip (2026-07-06); best-available lineage, not proven identical. Record defects: Ohio/Houston copy-paste text, 'Never Published', 'best-available-metadata: No'. LICENSING (verbatim, for the Licensing_Risk sheet): 'Users are granted a perpetual, non-exclusive, irrevocable, worldwide license to use these data ... with the exception of creating, training, improving, modifying, validating, testing, evaluating, or otherwise leveraging machine learning algorithms in order to explicitly create similar land cover data for a period of five years from its date of creation.' The Phase-1 canopy record (InPort 70562, created 2023-09-30) carries the broader unqualified form ('may not be used for the purpose of ... testing, or evaluating machine learning algorithms ... except with the express written consent of Ecopia Tech Corporation'). This project uses the product as an EVALUATION reference - flag for Kam.</t>
+        </is>
+      </c>
+      <c r="Q28" s="1" t="inlineStr">
+        <is>
+          <t>grid/true MEASURED; native PUBLISHED</t>
+        </is>
+      </c>
+      <c r="R28" s="1" t="inlineStr"/>
+      <c r="S28" s="1" t="inlineStr"/>
+      <c r="T28" s="1" t="inlineStr"/>
+      <c r="U28" s="1" t="inlineStr">
+        <is>
+          <t>reference raster</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>(not held) WA Statewide Imagery Consortium 2020 6-inch (Hexagon, Leica ADS100)</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>2020 (SECOND 2020 acquisition - NOT the anchor)</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>WA OCIO/WaTech Statewide Imagery Consortium, flown by Hexagon under the 2020 NAIP Imaging Program</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t>15 (6 in product), nominal flight GSD 20</t>
+        </is>
+      </c>
+      <c r="H29" s="1" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I29" s="1" t="inlineStr">
+        <is>
+          <t>20 (nominal)</t>
+        </is>
+      </c>
+      <c r="J29" s="1" t="inlineStr">
+        <is>
+          <t>2020-08-28 (flight-area polygon at the city centroid; 2020-08-27 also intersects the city bbox); program window 2020-08-03 to 2020-09-06</t>
+        </is>
+      </c>
+      <c r="K29" s="1" t="inlineStr">
+        <is>
+          <t>day (coarse flight-area block, 911-1263 sq mi)</t>
+        </is>
+      </c>
+      <c r="L29" s="1" t="inlineStr">
+        <is>
+          <t>multi (2 blocks over the city)</t>
+        </is>
+      </c>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="N29" s="1" t="inlineStr">
+        <is>
+          <t>https://www.arcgis.com/sharing/rest/content/items/dd83978971d8421eb6b1a7273ba51f6e?f=json</t>
+        </is>
+      </c>
+      <c r="O29" s="1" t="inlineStr">
+        <is>
+          <t>Digital aerial imagery for Washington state was collected by Hexagon as part of the 2020 NAIP Imaging Program. Imagery was collected between August 3, 2020 and September 6, 2020 using Leica ADS100 digital camera systems. The project was flown at heights ranging from 8,000 ft msl to 15,500 ft msl resulting in a nominal GSD of 20cm.</t>
+        </is>
+      </c>
+      <c r="P29" s="1" t="inlineStr">
+        <is>
+          <t>HAZARD ROW: a different vendor, camera, resolution and season from 2020_coe_rgb.tif (EagleView 3 in, Apr-Jul). Year-matched substitution would introduce a ~4.5-month error - exactly the 2015 three-way pattern. Not held; a late-August leaf-on 15 cm 4-band product if ever wanted.</t>
+        </is>
+      </c>
+      <c r="Q29" s="1" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="R29" s="1" t="inlineStr">
+        <is>
+          <t>2020-08-28 / 2020-08-27</t>
+        </is>
+      </c>
+      <c r="S29" s="1" t="inlineStr">
+        <is>
+          <t>https://services.arcgis.com/jsIt88o09Q0r1j8h/ArcGIS/rest/services/2020_Statewide_imagery_consortium_6_inch_flight_areas/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="T29" s="1" t="inlineStr">
+        <is>
+          <t>{"OBJECTID":9,"IDATE":"2020-08-28","squaremile":911} ; {"OBJECTID":8,"IDATE":"2020-08-27","squaremile":1263}</t>
+        </is>
+      </c>
+      <c r="U29" s="1" t="inlineStr">
+        <is>
+          <t>context (not held)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>(not held) WA Statewide Imagery Consortium 2018 6-inch; Edmonds_Marsh_2018 drone</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>2018 (two distinct acquisitions)</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>WA consortium (Hexagon) / City of Edmonds Imagery/Edmonds_Marsh_2018 ImageServer</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="inlineStr">
+        <is>
+          <t>15 (consortium) / 2.5 (Marsh cache LOD)</t>
+        </is>
+      </c>
+      <c r="H30" s="1" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I30" s="1" t="inlineStr">
+        <is>
+          <t>n/a / 3.36 (Marsh pixelSizeX 0.0336 m)</t>
+        </is>
+      </c>
+      <c r="J30" s="1" t="inlineStr">
+        <is>
+          <t>2018-08-07 (consortium flight area over Edmonds) ; 2018-08-01 16:22-16:52 UTC (Marsh drone sortie) - six days apart, NOT the same acquisition</t>
+        </is>
+      </c>
+      <c r="K30" s="1" t="inlineStr">
+        <is>
+          <t>day / exact timestamp</t>
+        </is>
+      </c>
+      <c r="L30" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="N30" s="1" t="inlineStr">
+        <is>
+          <t>https://services.arcgis.com/jsIt88o09Q0r1j8h/arcgis/rest/services/2018FlightAreas/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="O30" s="1" t="inlineStr">
+        <is>
+          <t>{"FID": 18, "OBJECTID": 18, "IDATE": "2018-08-07"}</t>
+        </is>
+      </c>
+      <c r="P30" s="1" t="inlineStr">
+        <is>
+          <t>Recorded to prevent conflation. The Marsh service is the project's only Edmonds layer with a machine-readable timestamp and the positive control for keyProperties queries (correct path: /gis/rest/services/.../ImageServer/keyProperties?f=json).</t>
+        </is>
+      </c>
+      <c r="Q30" s="1" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="R30" s="1" t="inlineStr">
+        <is>
+          <t>2018-08-01T16:22:13+00:00 to 16:52:13 (Marsh)</t>
+        </is>
+      </c>
+      <c r="S30" s="1" t="inlineStr">
+        <is>
+          <t>https://maps.edmondswa.gov/gis/rest/services/Basemap/Edmonds_Marsh_2018/ImageServer/keyProperties?f=json</t>
+        </is>
+      </c>
+      <c r="T30" s="1" t="inlineStr">
+        <is>
+          <t>"acquisitionEndDate":"2018-08-01T16:52:13+00:00","acquisitionStartDate":"2018-08-01T16:22:13+00:00"</t>
+        </is>
+      </c>
+      <c r="U30" s="1" t="inlineStr">
+        <is>
+          <t>context (not held)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U27"/>
+  <autoFilter ref="A1:U30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
pixel-size+date v1.1: every quote now a literal fetched record (quote gate 0 misses against fetched pages only); raw index records over the city saved as evidence
</commit_message>
<xml_diff>
--- a/Scripts/imagery_catalog_2026-08-22.xlsx
+++ b/Scripts/imagery_catalog_2026-08-22.xlsx
@@ -12552,7 +12552,7 @@
       </c>
       <c r="O4" s="1" t="inlineStr">
         <is>
-          <t>2000-06-26 (callout label on the peach block containing cells t27r03, t27r04, t27r05, t28r04, t28r05). The live SDC page: 'Detailed photodate information is not available. A general overview at the township-level for data capture dates can interpolated from https://www5.kingcounty.gov/sdc/raster/ortho/images/ortho2000emergegeneralflightdate.jpg'</t>
+          <t>2000-06-26 (callout label on the graphic's peach block containing cells t27r03, t27r04, t27r05, t28r04, t28r05) ... [live SDC page, IMAGE_Ortho2000EmergeNAT:] Detailed photodate information is not available. ... A general overview at the township-level for data capture dates can interpolated from https://www5.kingcounty.gov/sdc/raster/ortho/images/ortho2000emergegeneralflightdate.jpg</t>
         </is>
       </c>
       <c r="P4" s="1" t="inlineStr">
@@ -12873,7 +12873,7 @@
       </c>
       <c r="O7" s="1" t="inlineStr">
         <is>
-          <t>SHOTDATE field, 1078 frames intersecting the city polygon (query 2026-08-23; refetch-verified: field exists, all six days non-zero countywide)</t>
+          <t>"IMAGENAME":"WAKING035400NeighOrtho1546_070707" ... "SHOTDATE":"2007/07/07 18:27:03" (first of 1078 frames intersecting the city polygon; raw response qc/imagery_date_evidence/raw_records/kc_2007_ORTHO_IMAGE07_AREA_759_citypoly_first3.json)</t>
         </is>
       </c>
       <c r="P7" s="1" t="inlineStr">
@@ -12980,7 +12980,7 @@
       </c>
       <c r="O8" s="1" t="inlineStr">
         <is>
-          <t>SHOTDATE/YYYYMMDD fields, 472 frames intersecting the city polygon (query 2026-08-23; refetch-verified)</t>
+          <t>"IMAGENAME":"WAKING042400NeighOrtho77930_090509" ... "SHOTDATE":"2009/05/09 20:58:13" (first of 472 frames intersecting the city polygon; raw response qc/imagery_date_evidence/raw_records/kc_2009_ORTHO_IMAGE09_AREA_760_citypoly_first3.json)</t>
         </is>
       </c>
       <c r="P8" s="1" t="inlineStr">
@@ -13075,7 +13075,7 @@
       </c>
       <c r="O9" s="1" t="inlineStr">
         <is>
-          <t>DATE_STR/TIME_STR fields, 75 photo centres inside the city polygon (query 2026-08-23); DATACOLOR='nir' for all 75</t>
+          <t>"DATACOLOR":"nir" ... "DATE_STR":"Apr.07.2012" ... "TIME_STR":"12:46:28" (first of 75 photo centres inside the city polygon; raw response qc/imagery_date_evidence/raw_records/kc_2012_ORTHO_IMAGE12_POINT_1447_citypoly_first3.json)</t>
         </is>
       </c>
       <c r="P9" s="1" t="inlineStr">
@@ -13182,7 +13182,7 @@
       </c>
       <c r="O10" s="1" t="inlineStr">
         <is>
-          <t>ShotDate/YYYYMMDD fields, 688 frames intersecting the city polygon (query 2026-08-23; refetch-verified)</t>
+          <t>"ImageName":"WAKING042400NeighOrtho8690_130602" ... "ShotDate":"2013/06/02 18:04:31" (first of 688 frames intersecting the city polygon; raw response qc/imagery_date_evidence/raw_records/kc_2013_ORTHO_IMAGE13_AREA_2061_citypoly_first3.json)</t>
         </is>
       </c>
       <c r="P10" s="1" t="inlineStr">
@@ -13277,7 +13277,7 @@
       </c>
       <c r="O11" s="1" t="inlineStr">
         <is>
-          <t>ShotDate/YYYYMMDD fields, 701 frames intersecting the city polygon (query 2026-08-23; refetch-verified)</t>
+          <t>"ImageName":"WAKING041401NeighOrtho4281_150228" ... "ShotDate":"2015/02/28 14:51:01" (first of 701 frames intersecting the city polygon; raw response qc/imagery_date_evidence/raw_records/kc_2015_ORTHO_IMAGE15_AREA_2499_citypoly_first3.json)</t>
         </is>
       </c>
       <c r="P11" s="1" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="O12" s="1" t="inlineStr">
         <is>
-          <t>ShotDate/YYYYMMDD fields, 710 frames intersecting the city polygon (query 2026-08-23; an independent re-query returned 695, all 15 missing on May 10 - residual geometry handling, same days)</t>
+          <t>"ImageName":"WAKING043402NeighOrtho01390_170509" ... "ShotDate":"2017/05/09 17:20:09" (first of 710 frames intersecting the city polygon - an independent re-query returned 695, all 15 missing on May 10, same days; raw response qc/imagery_date_evidence/raw_records/kc_2017_ORTHO_IMAGE17_AREA_2685_citypoly_first3.json)</t>
         </is>
       </c>
       <c r="P12" s="1" t="inlineStr">
@@ -13467,7 +13467,7 @@
       </c>
       <c r="O13" s="1" t="inlineStr">
         <is>
-          <t>ShotDate field (date only; the layer carries Time_UTC/Time_PDT separately), 1234 frames intersecting the city polygon (query 2026-08-23; refetch-verified)</t>
+          <t>"ImageName":"WAKING042402NeighOrtho5255_190425" ... "ShotDate":"2019/04/25" (date-only field; first of 1234 frames intersecting the city polygon; raw response qc/imagery_date_evidence/raw_records/kc_2019_ORTHO_IMAGE19_AREA_2852_citypoly_first3.json)</t>
         </is>
       </c>
       <c r="P13" s="1" t="inlineStr">
@@ -13562,7 +13562,7 @@
       </c>
       <c r="O14" s="1" t="inlineStr">
         <is>
-          <t>ShotDate field, 662 frames intersecting the city polygon (query 2026-08-23; refetch-verified)</t>
+          <t>"ImageName":"WAKING022033NeighOrtho9795_210415" ... "ShotDate":"2021/04/15 14:54:55" (first of 662 frames intersecting the city polygon; raw response qc/imagery_date_evidence/raw_records/kc_2021_ORTHO_IMAGE21_AREA_2912_citypoly_first3.json)</t>
         </is>
       </c>
       <c r="P14" s="1" t="inlineStr">
@@ -13657,7 +13657,7 @@
       </c>
       <c r="O15" s="1" t="inlineStr">
         <is>
-          <t>ShotDate field, 1125 frames intersecting the city polygon (query 2026-08-23; refetch-verified)</t>
+          <t>"ImageName":"WAKING022033NeighOrtho8996_230503" ... "ShotDate":"2023/05/03 18:48:58" (first of 1125 frames intersecting the city polygon; raw response qc/imagery_date_evidence/raw_records/kc_2023_ORTHO_IMAGE23_AREA_3073_citypoly_first3.json)</t>
         </is>
       </c>
       <c r="P15" s="1" t="inlineStr">
@@ -13764,7 +13764,7 @@
       </c>
       <c r="O16" s="1" t="inlineStr">
         <is>
-          <t>SDATE '08/11/2016 16:52' (SUNEL 31) / '08/12/2016 09:05' (SUNEL 34) / '08/12/2016 09:30' (SUNEL 37), THEMENAME hxip_m_4712213/4712214_*_10_15; city-centroid point query returns hxip_m_4712213_se2_10_15, SDATE '08/12/2016 09:30', SUNEL 37, ACCURACY '0.68m (ce 95%)'</t>
+          <t>"THEMENAME":"hxip_m_4712213_se2_10_15","SDATE":"08/12/2016 09:30","SUNEL":37,"ACCURACY":"0.68m (ce 95%)" (city-centroid point query) ... "THEMENAME":"hxip_m_4712214_sw3_10_15","SDATE":"08/12/2016 09:05","SUNEL":34 ... "THEMENAME":"hxip_m_4712214_sw2_10_15","SDATE":"08/11/2016 16:52","SUNEL":31 (city bbox, 11 footprints; raw responses qc/imagery_date_evidence/raw_records/wa_2016_6in_*.json)</t>
         </is>
       </c>
       <c r="P16" s="1" t="inlineStr">
@@ -13789,7 +13789,7 @@
       </c>
       <c r="T16" s="1" t="inlineStr">
         <is>
-          <t>SDATE '08/07/2015 15:31', THEMENAME hxip_m_4712213_ne_10_30, SUNEL 46</t>
+          <t>"THEMENAME":"hxip_m_4712213_se_10_30","SDATE":"08/07/2015 15:31","SUNEL":46,"ACCURACY":"0.72m (ce 95%)" (city-centroid point query; raw response qc/imagery_date_evidence/raw_records/wa_2015_1ft_citycentroid.json)</t>
         </is>
       </c>
       <c r="U16" s="1" t="inlineStr">
@@ -13966,12 +13966,12 @@
       </c>
       <c r="O18" s="1" t="inlineStr">
         <is>
-          <t>Identity MEASURED 2026-08-23: held 2017_coe_rgb.tif (2x boxcar-downsampled) vs 2017_king_rgb.tif over a 12x12 grid on the city polygon, 66 valid 512-px windows -&gt; r min 0.9568, p5 0.9786, median 0.9923, max 0.9966, MAE median 3.54 DN; live services 2017_Aerial_Cached vs KingCo_Aerial_2017 LOD-20 tiles at 5 sites r = 0.9876-0.9935. Identical vehicles in identical stalls and identical building relief displacement -&gt; same orthorectification, not merely the same flight.</t>
+          <t>"ImageName":"WAKING043402NeighOrtho01390_170509" ... "ShotDate":"2017/05/09 17:20:09" (King County 2017 index, first of 710 frames intersecting the city polygon; raw response qc/imagery_date_evidence/raw_records/kc_2017_ORTHO_IMAGE17_AREA_2685_citypoly_first3.json). Dates transfer because the two files are the same orthomosaic - see notes.</t>
         </is>
       </c>
       <c r="P18" s="1" t="inlineStr">
         <is>
-          <t>Retires the 8.5-month candidate window and the council-minutes line (2023-07-25 p.15, 'PlanIt Geo ... 2017 flyovers') as evidence - the 2019 UFMP was written by Davey Resource Group and its canopy work used Aug 2015 imagery; PlanIt Geo appears nowhere in it. No City of Edmonds document naming the 2017 vendor was found; attribution rests on measured pixel identity plus King County's published coverage statement (alt). Snohomish County's own 2017 product is a 1-ft HXIP flight (2017-08-15/21) and cannot be a 3-in source. Grid note: the held grid is exactly LOD 21, which King's tile endpoint does not serve (404 at L21) but Edmonds' does - consistent with a city-service export. Method detail: qc/imagery_date_evidence/coe2017_identity/.</t>
+          <t>Identity MEASURED 2026-08-23: held 2017_coe_rgb.tif (2x boxcar-downsampled) vs 2017_king_rgb.tif over a 12x12 grid on the city polygon, 66 valid 512-px windows -&gt; r min 0.9568, p5 0.9786, median 0.9923, max 0.9966, MAE median 3.54 DN; live services 2017_Aerial_Cached vs KingCo_Aerial_2017 LOD-20 tiles at 5 sites r = 0.9876-0.9935. Identical vehicles in identical stalls and identical building relief displacement -&gt; same orthorectification, not merely the same flight. Retires the 8.5-month candidate window and the council-minutes line (2023-07-25 p.15, 'PlanIt Geo ... 2017 flyovers') as evidence - the 2019 UFMP was written by Davey Resource Group and its canopy work used Aug 2015 imagery; PlanIt Geo appears nowhere in it. No City of Edmonds document naming the 2017 vendor was found; attribution rests on measured pixel identity plus King County's published coverage statement (alt). Snohomish County's own 2017 product is a 1-ft HXIP flight (2017-08-15/21) and cannot be a 3-in source. Grid note: the held grid is exactly LOD 21, which King's tile endpoint does not serve (404 at L21) but Edmonds' does - consistent with a city-service export. Method detail: qc/imagery_date_evidence/coe2017_identity/.</t>
         </is>
       </c>
       <c r="Q18" s="1" t="inlineStr">
@@ -14394,7 +14394,7 @@
       </c>
       <c r="O22" s="1" t="inlineStr">
         <is>
-          <t>{"FILENAME": "13007_57226", "FRAME": 57226, ... "UTC_TIME": "19:35:08", "MAX_GSD__f": 0.225, "USED": "YES", "VENDOR": "GeoTerra", "CAMERA": "UltraCam Xp", "SSN": 10411033, ... "FLIGHTLINE": "13007", "ACQ_DATE": 1429228800000} (photo-centre layer; in-polygon N=167; 'It is a reference for the raw image scans, it is not a index for tiled ortho imagery')</t>
+          <t>"FILENAME":"13009_57445" ... "UTC_TIME":"19:54:49","MAX_GSD__f":0.225 ... "VENDOR":"GeoTerra","CAMERA":"UltraCam Xp" ... "FLIGHTLINE":"13009","ACQ_DATE":1429228800000 (= 2015-04-17 UTC; first of the photo centres inside the city polygon; raw response qc/imagery_date_evidence/raw_records/kc_2015C_ORTHO_IMAGE15C_POINT_2574_citypoly_first3.json). Layer description: It is a reference for the raw image scans, it is not a index for tiled ortho imagery</t>
         </is>
       </c>
       <c r="P22" s="1" t="inlineStr">
@@ -14526,7 +14526,7 @@
       </c>
       <c r="T23" s="1" t="inlineStr">
         <is>
-          <t>{"FID": 23, "IDATE": "2019 -10-11"} (stray space verbatim)</t>
+          <t>"IDATE":"2019 -10-11" (stray space verbatim; city-centroid point query, raw response qc/imagery_date_evidence/raw_records/wa_2019_1ft_citycentroid.json)</t>
         </is>
       </c>
       <c r="U23" s="1" t="inlineStr">
@@ -14608,7 +14608,7 @@
       </c>
       <c r="O24" s="1" t="inlineStr">
         <is>
-          <t>&lt;gmd:title&gt; m_4712214_sw_10_060_20231007.tif (date field of the DOQQ file name in the ISO metadata record)</t>
+          <t>&lt;gco:CharacterString&gt;m_4712214_sw_10_060_20231007.tif&lt;/gco:CharacterString&gt; (the DOQQ file name in the ISO metadata record; 20231007 = acquisition date field)</t>
         </is>
       </c>
       <c r="P24" s="1" t="inlineStr">
@@ -14703,7 +14703,7 @@
       </c>
       <c r="O25" s="1" t="inlineStr">
         <is>
-          <t>Time Frame 2016-03-17 - 2017-06-06 / North: March 17 - Sept 30, 2016 / South: March 17, 2016 - June 6, 2017</t>
+          <t>North: March 17 - Sept 30, 2016 ... South: March 17, 2016 - June 6, 2017</t>
         </is>
       </c>
       <c r="P25" s="1" t="inlineStr">
@@ -14755,7 +14755,7 @@
       </c>
       <c r="D26" s="1" t="inlineStr">
         <is>
-          <t>point cloud</t>
+          <t>point cloud (no grid)</t>
         </is>
       </c>
       <c r="E26" s="1" t="inlineStr">
@@ -14770,7 +14770,7 @@
       </c>
       <c r="G26" s="1" t="inlineStr">
         <is>
-          <t>0.25 pts/m2 stated (~0.17 cross-checked)</t>
+          <t>n/a (point cloud)</t>
         </is>
       </c>
       <c r="H26" s="1" t="inlineStr">
@@ -14815,7 +14815,7 @@
       </c>
       <c r="P26" s="1" t="inlineStr">
         <is>
-          <t>LEAF-OFF (late February). Record-internal inconsistency: Mt. Lake Terrace sub-project dates run past the record's own Time Frame end (2005-07-15). Held at D:/edmonds-pipeline/Imagery/PSLC_2005 and Full_Image/PSLC_2005 (IMAGERY_FACTS 8.2).</t>
+          <t>Density 0.25 pts/m2 stated (~0.17 cross-checked, IMAGERY_FACTS 8.1). LEAF-OFF (late February). Record-internal inconsistency: Mt. Lake Terrace sub-project dates run past the record's own Time Frame end (2005-07-15). Held at D:/edmonds-pipeline/Imagery/PSLC_2005 and Full_Image/PSLC_2005 (IMAGERY_FACTS 8.2).</t>
         </is>
       </c>
       <c r="Q26" s="1" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="T29" s="1" t="inlineStr">
         <is>
-          <t>{"OBJECTID":9,"IDATE":"2020-08-28","squaremile":911} ; {"OBJECTID":8,"IDATE":"2020-08-27","squaremile":1263}</t>
+          <t>"IDATE":"2020-08-28" (city centroid) ... "IDATE":"2020-08-27" (also intersects the city bbox; raw responses qc/imagery_date_evidence/raw_records/wa_2020_6in_*.json)</t>
         </is>
       </c>
       <c r="U29" s="1" t="inlineStr">
@@ -15202,7 +15202,7 @@
       </c>
       <c r="O30" s="1" t="inlineStr">
         <is>
-          <t>{"FID": 18, "OBJECTID": 18, "IDATE": "2018-08-07"}</t>
+          <t>"IDATE":"2018-08-07" (city-centroid point query; raw response qc/imagery_date_evidence/raw_records/wa_2018_6in_citycentroid.json)</t>
         </is>
       </c>
       <c r="P30" s="1" t="inlineStr">

</xml_diff>

<commit_message>
docs: IMAGERY_FACTS 9.2 -> delta + pointer to the pixel-size/date table; catalogue Contradictions/Provenance_Chain/Dating_Methods stamped SUPERSEDED, 3 Retractions added; CHATLOG STATE provenance line + LOG entry
</commit_message>
<xml_diff>
--- a/Scripts/imagery_catalog_2026-08-22.xlsx
+++ b/Scripts/imagery_catalog_2026-08-22.xlsx
@@ -11444,7 +11444,7 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>SOURCE DOCUMENTED in a signed city contract</t>
+          <t>[SUPERSEDED 2026-08-23 -&gt; Pixel_Size_And_Date] Still INFERRED; consistent with ONE continuous pass (shadow geometry, 10 sites); head trimmed to 2020-04-25. Contract vehicle for the PRR: King County RFP 1166-18-PCR / Piggyback PB-19-14BC. || was: SOURCE DOCUMENTED in a signed city contract</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
@@ -11482,7 +11482,7 @@
       <c r="B3" s="1" t="inlineStr"/>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>named in the same contract clause</t>
+          <t>[SUPERSEDED 2026-08-23 -&gt; Pixel_Size_And_Date] IDENTITY MEASURED: same MrSID encode as Everett's Image2022_3in_sid (input set 675,609,635,568 B) -&gt; window PUBLISHED. || was: named in the same contract clause</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -11542,7 +11542,7 @@
       <c r="B5" s="1" t="inlineStr"/>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>NO contract, NO budget line, NO flight date found</t>
+          <t>[SUPERSEDED 2026-08-23 -&gt; Pixel_Size_And_Date] DATED: same orthomosaic as King 2017 -&gt; 2017-05-04..05-10 MEASURED. || was: NO contract, NO budget line, NO flight date found</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
@@ -11623,7 +11623,7 @@
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>maps.edmondswa.gov/.../Edmonds_Marsh_2018/ImageServer/info/keyProperties</t>
+          <t>[SUPERSEDED 2026-08-23 -&gt; Pixel_Size_And_Date] LIVE PATH: https://maps.edmondswa.gov/gis/rest/services/Basemap/Edmonds_Marsh_2018/ImageServer/keyProperties?f=json (the /arcgis/ form 500s; /info/keyProperties 400s on every service). || was: maps.edmondswa.gov/.../Edmonds_Marsh_2018/ImageServer/info/keyProperties</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr">
@@ -11852,7 +11852,7 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>*** RUN IT PER SEAMLINE PATCH, NOT PER CITY *** - a county mosaic over 22 sq mi is stitched from multiple flight lines, plausibly multiple days. This also answers a question nobody has asked: IS 2020_coe_rgb.tif EVEN A SINGLE-DATE IMAGE? If not, 'the 2020 acquisition date' is the wrong question and that matters more for the labels than the date does.</t>
+          <t>[SUPERSEDED 2026-08-23 -&gt; Pixel_Size_And_Date] RUN 2026-08-23: azimuth reliable (2012 control 8/10), elevation saturates above ~45 deg -&gt; 2020 consistent with one pass, no calendar date. Evidence qc/imagery_date_evidence/shadow_dating_2020/. || was: *** RUN IT PER SEAMLINE PATCH, NOT PER CITY *** - a county mosaic over 22 sq mi is stitched from multiple flight lines, plausibly multiple days. This also answers a question nobody has asked: IS 2020_coe_rgb.tif EVEN A SINGLE-DATE IMAGE? If not, 'the 2020 acquisition date' is the wrong question and that matters more for the labels than the date does.</t>
         </is>
       </c>
     </row>
@@ -11884,7 +11884,7 @@
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>Puget Sound spring weather will eliminate most of the 92 candidate days outright. One afternoon. Converts the window to a shortlist that method 1 picks from, and independently sanity-checks whatever method 1 returns.</t>
+          <t>[SUPERSEDED 2026-08-23 -&gt; Pixel_Size_And_Date] RUN 2026-08-23: the 30-deg sun floor is FALSIFIED by a known flight day (2015-02-15, max elevation 29.3 deg); calibrated rule (20-deg floor, 3-station consensus) passes 46/46 controls. Eliminates 22/92 (2020), 19/97 (2022), 18/62 (2024), 32/140 (2021s) days. || was: Puget Sound spring weather will eliminate most of the 92 candidate days outright. One afternoon. Converts the window to a shortlist that method 1 picks from, and independently sanity-checks whatever method 1 returns.</t>
         </is>
       </c>
     </row>
@@ -12076,7 +12076,7 @@
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>Not a records request - an internal ask to Brian Tuley for a login, or a screenshot from someone who has one. It was sitting in the contract the whole time and could end the exercise today.</t>
+          <t>[SUPERSEDED 2026-08-23 -&gt; Pixel_Size_And_Date] Contract numbers for the ask/PRR now known: King County RFP 1166-18-PCR, Snohomish Piggyback PB-19-14BC, Legistar 2024-1168. || was: Not a records request - an internal ask to Brian Tuley for a login, or a screenshot from someone who has one. It was sitting in the contract the whole time and could end the exercise today.</t>
         </is>
       </c>
     </row>
@@ -15527,7 +15527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -15858,6 +15858,87 @@
       <c r="E12" s="1" t="inlineStr">
         <is>
           <t>See the Reference_Independence sheet. Agreement between two Ecopia products is not corroboration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2017_coe_rgb.tif spans an 8.5-month leaf-off-to-leaf-on window (2017-02-17 to 10-30)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>IMAGERY_FACTS 9.2 / Provenance_Chain</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>It is the same orthomosaic as 2017_king_rgb.tif (r 0.957-0.997, 66 windows) and was flown 2017-05-04..05-10 over the city.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>A coarse published window for a PARENT product was carried as the file's own window. Measuring identity against a sibling file settled in minutes what document-hunting could not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>The 2015 CoE basemap date is a three-way contest between independent acquisitions</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Contradictions sheet</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>The three dates belong to three DIFFERENT products (NAIP/HXIP Aug 7; King Pictometry Feb-Mar; city consortium Apr 8/17). The catalogue's 'Apr 8/9/17' also contained a day (Apr 9) with no frames over Edmonds.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Year-matched product substitution is the recurring trap (it recurred the same day: a second 2020 acquisition, Hexagon 2020-08-27/28, exists over Edmonds). Always ask WHICH product before asking WHEN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>The HXIP footprint SDATE '08/11/2016 16:52' is UTC because the held file shows morning shadows</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>session lead's open note</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>SDATE is LOCAL time (7034-footprint SUNEL fit; 09:05 read as UTC puts the sun 26 deg below the horizon). The held county 1-ft product simply is not that sortie.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>A hypothesis stated to explain one observation was tested against the whole field and failed. State it, test it, record it.</t>
         </is>
       </c>
     </row>
@@ -16150,7 +16231,7 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>UNRESOLVED</t>
+          <t>[SUPERSEDED 2026-08-23 -&gt; Pixel_Size_And_Date] LARGELY RESOLVED: the three dates are three DIFFERENT products. Aug 7 2015 = NAIP/HXIP 2015 (Davey UTC Assessment names USDA FSA), Feb 15-Mar 8 = King Pictometry (the held 2015_king_rgb.tif; pixel-distinct from the CoE basemap, r 0.04-0.56 vs 0.99 control), Apr 8 + Apr 17 2015 = the city consortium photo centres (no Apr 9 over Edmonds). Residual: attribution of Ed_Aerial_2015.tif to the consortium is INFERRED; the '4.8 in' figure is unexplained. || was: UNRESOLVED</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
@@ -16182,7 +16263,7 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>MINUTES ARE WEAK</t>
+          <t>[SUPERSEDED 2026-08-23 -&gt; Pixel_Size_And_Date] RESOLVED: 2017_coe_rgb.tif is the SAME ORTHOMOSAIC as King County IMAGE_Ortho2017KCNAT (Pictometry), MEASURED r 0.957-0.997 over 66 citywide windows; dated 2017-05-04..05-10 from the per-frame index. The council-minutes 'PlanIt Geo' line is retired (the 2019 UFMP was by Davey Resource Group and used Aug-2015 imagery). || was: MINUTES ARE WEAK</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">

</xml_diff>

<commit_message>
S16 landed: 2016_snoh_1ft_rgbi.tif REPLACES 2016_snoh_rgbi.tif (full extent, native 1 ft, 100% city coverage, NIR) — YEAR_CATALOG flipped, SUPERSEDED_FILES, catalogue + table rows, IMAGERY_FACTS §10; measure: exact-unit true GSD, city-polygon coverage, common-grid effective resolution; files mode parallel streams
</commit_message>
<xml_diff>
--- a/Scripts/imagery_catalog_2026-08-22.xlsx
+++ b/Scripts/imagery_catalog_2026-08-22.xlsx
@@ -33,7 +33,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing_Risk" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MASTER'!$A$1:$P$221</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'KingCo_SDC_Catalog'!$A$1:$D$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DataLake_Issues'!$A$1:$C$15</definedName>
@@ -10920,7 +10920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11361,6 +11361,37 @@
       <c r="G12" s="1" t="inlineStr">
         <is>
           <t>*** the published 2.8x / 110.8 cm is a RED-BAND-ONLY figure. Effective resolution is BAND-DEPENDENT and red - the band every greenness/NDVI index depends on - is the most degraded ***</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2016_snoh_1ft_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>30.48</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="E13" t="n">
+        <v>40.56</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>median of 5 Method_Provenance sites; common-grid vs 2016_snoh_rgbi.tif: new 42.98 / held 43.2 cm, HF ratio 1.013</t>
         </is>
       </c>
     </row>
@@ -12156,7 +12187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U30"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -13769,7 +13800,7 @@
       </c>
       <c r="P16" s="1" t="inlineStr">
         <is>
-          <t>Held file = export of the county service (window means identical to exportImage) and pixel-DISTINCT from Aerial_2015 and Aerial_2017 (MEASURED). SDATE is LOCAL clock time: a 7034-footprint fit of published SUNEL vs pvlib gives RMSE 6.9 deg for UTC-7 vs 55.6 for UTC, and 09:05 read as UTC puts the sun 26 deg below the horizon. The county gdb is HXIP_2016_SNOHOMISH.gdb (the 'HXIP_2015' tokens in the lineage are a stale parent-folder / dataset-name carry-over, not 2015 imagery); the 2015-08-07 flight is excluded three ways (pixel comparison, afternoon vs morning shadows, lineage). 6-in coverage reached Edmonds because it lies inside the Valtus/Hexagon 'Seattle' UAC polygon, not via a county buy-up. The Geocortex blurb 'acquired in August 2016 as part of a Washington Statewide Imagery consortium. Pixel size of the raster is 6 inch' sits on a layer titled '2017 Aerial Photos' and contradicts the county's 1-ft tiles - CONTESTED, month-level corroboration only. Both Aug 11 and Aug 12 2016 were flyable at all three ASOS stations (Aug 11 morning marine stratus at KPAE only). C-CAP 2016 Snohomish (InPort 53263) says its source imagery is 'NAIP ... summer 2016' but no WA NAIP 2016 exists - most plausibly this HXIP flight. Held file is a study-area CROP (lon -122.404..-122.316, lat 47.783..47.828).</t>
+          <t>*** SUPERSEDED 2026-08-23 by 2016_snoh_1ft_rgbi.tif (full study extent at the native 1-ft grid; this clipped 0.5-ft server upsample is kept for provenance) *** Held file = export of the county service (window means identical to exportImage) and pixel-DISTINCT from Aerial_2015 and Aerial_2017 (MEASURED). SDATE is LOCAL clock time: a 7034-footprint fit of published SUNEL vs pvlib gives RMSE 6.9 deg for UTC-7 vs 55.6 for UTC, and 09:05 read as UTC puts the sun 26 deg below the horizon. The county gdb is HXIP_2016_SNOHOMISH.gdb (the 'HXIP_2015' tokens in the lineage are a stale parent-folder / dataset-name carry-over, not 2015 imagery); the 2015-08-07 flight is excluded three ways (pixel comparison, afternoon vs morning shadows, lineage). 6-in coverage reached Edmonds because it lies inside the Valtus/Hexagon 'Seattle' UAC polygon, not via a county buy-up. The Geocortex blurb 'acquired in August 2016 as part of a Washington Statewide Imagery consortium. Pixel size of the raster is 6 inch' sits on a layer titled '2017 Aerial Photos' and contradicts the county's 1-ft tiles - CONTESTED, month-level corroboration only. Both Aug 11 and Aug 12 2016 were flyable at all three ASOS stations (Aug 11 morning marine stratus at KPAE only). C-CAP 2016 Snohomish (InPort 53263) says its source imagery is 'NAIP ... summer 2016' but no WA NAIP 2016 exists - most plausibly this HXIP flight. Held file is a study-area CROP (lon -122.404..-122.316, lat 47.783..47.828).</t>
         </is>
       </c>
       <c r="Q16" s="1" t="inlineStr">
@@ -13801,22 +13832,22 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>2021_snoh_rgbi.tif</t>
+          <t>2016_snoh_1ft_rgbi.tif</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>2021 (Snoh)</t>
+          <t>2016 (campaign S16, REPLACES 2016_snoh_rgbi.tif)</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>HXIP via Snohomish County Imagery/Aerial_2021 ImageServer (mosaic gdb HXIP_2021_SNOHOMISH.gdb - a Hexagon delivery, not EagleView)</t>
+          <t>Hexagon Imagery Program (HXIP) via Snohomish County Imagery/Aerial_2016 ImageServer, exported 2026-08-23 by pipeline/acquire_imagery.py at the native 1-ft lattice (grid snapped to the service origin, RSP_NearestNeighbor: nearest == bilinear to 0 differing pixels in the pilot)</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr">
@@ -13831,62 +13862,74 @@
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>15.24</t>
+          <t>30.48</t>
         </is>
       </c>
       <c r="H17" s="1" t="inlineStr">
         <is>
-          <t>20.6</t>
+          <t>40.6 (median of 5 Method_Provenance sites on the native 1-ft grid; 1.33x oversampled) - on a common 30.48 cm grid the old and new files resolve alike (43.0 vs 43.2 cm, HF-energy ratio 1.01): same source pixels, no server resampling</t>
         </is>
       </c>
       <c r="I17" s="1" t="inlineStr">
         <is>
-          <t>15.24 (0.5 ft): mosaic-catalog LowPS=0.5, item pixelSizeX=0.5 (MEASURED)</t>
+          <t>30.48 (1 ft = the county's delivered tile size; served pixelSize 0.5 ft is an upsample)</t>
         </is>
       </c>
       <c r="J17" s="1" t="inlineStr">
         <is>
-          <t>2021-06-25 to 2021-11-11</t>
+          <t>2016-08-12 morning (consortium sorties 09:05 / 09:30 PDT; 09:50 within the city bbox) - CONDITIONAL on the county 1-ft product being the same flight as the dated 15 cm consortium product; the 2016-08-11 16:52 sortie is EXCLUDED for the old extent by shadow azimuth</t>
         </is>
       </c>
       <c r="K17" s="1" t="inlineStr">
         <is>
-          <t>window of 140 days (weather trims to 108 feasible days; 18 late days never reach 30 deg sun)</t>
+          <t>window of 2 days by the consortium labels (Aug 11-12); pixels consistent with Aug 12</t>
         </is>
       </c>
       <c r="L17" s="1" t="inlineStr">
         <is>
-          <t>unknown; held crop flown in the AFTERNOON (shadow azimuth 67-91 deg = sun at 247-256 deg, uniform over 24 windows) - a time-of-day constraint, not a date</t>
-        </is>
-      </c>
-      <c r="M17" s="4" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+          <t>consortium labels MULTI (2 days, 3-4 sorties); shadows uniformly morning over the old extent - the new full extent has not been re-measured for shadow direction</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>INFERRED</t>
         </is>
       </c>
       <c r="N17" s="1" t="inlineStr">
         <is>
-          <t>https://snohomishcountywa.gov/5414/Interactive-Map-SCOPI</t>
+          <t>https://services.arcgis.com/jsIt88o09Q0r1j8h/arcgis/rest/services/NAIP_2016_6in_Ortho_Dates_and_Times_83s/FeatureServer/0/query</t>
         </is>
       </c>
       <c r="O17" s="1" t="inlineStr">
         <is>
-          <t>The 2021 aerial photos are 6 inch resolution and cover mainly the urban areas. The imagery was collected between June 25, 2021 and November 11, 2021.</t>
+          <t>"THEMENAME":"hxip_m_4712213_se2_10_15","SDATE":"08/12/2016 09:30","SUNEL":37,"ACCURACY":"0.68m (ce 95%)" (city-centroid point query) ... "THEMENAME":"hxip_m_4712214_sw3_10_15","SDATE":"08/12/2016 09:05","SUNEL":34 ... "THEMENAME":"hxip_m_4712214_sw2_10_15","SDATE":"08/11/2016 16:52","SUNEL":31 (city bbox, 11 footprints; raw responses qc/imagery_date_evidence/raw_records/wa_2016_6in_*.json)</t>
         </is>
       </c>
       <c r="P17" s="1" t="inlineStr">
         <is>
-          <t>CLOSED LEADS: no WA consortium flight-date layer exists for 2021 or later (all 68 WAGeoservices services + 225 items enumerated; series ends 2020); the mosaic-catalog schema has no date field at all; WA NAIP 2021 does not cover quad 47122 (eastern WA only), so no NAIP ride-along date. Remaining route: the Hexagon flight log via Snohomish County DoIT, or the consortium contact (Joanne Markert, WA OCIO). Weather elimination (ASOS KPAE+KSEA+KBFI, criterion calibrated to 46/46 known Edmonds flight days; 2021-06-25..11-11): 32 of 140 days eliminated; longest feasible blocks Jul 22-Aug 6, Jul 2-15, Aug 9-19. ELIMINATES ONLY - no surviving day is favoured. Per-day table: qc/imagery_date_evidence/weather/flyable_days.csv.</t>
+          <t>MEASURED on arrival (D:/edmonds-pipeline/Imagery/SnoCo/_acq/S16/measure.json): 25,116 x 35,259 px, 4 bands uint8, EPSG:2285, 2,586,179,492 B; city-polygon coverage 100% (old file 66.7%), study-extent coverage 82.3% (the rest is Puget Sound); band 4 NIR (std 66, NDVI p90 0.73); no JPEG 8x8 block signature; blue-vs-green registration 0.075 px. Fetch: 234 chunks of 2048 px + 64 px overlap, 0 failures, 30 empty (water), 9.5 min at 5.8 MB/s; stitched BigTIFF spot-verified against 12 chunks; MANIFEST.sha256 on both planes. Decision REPLACE (wins: coverage; no losses). Date evidence is inherited from the superseded row (same flight, same service).</t>
         </is>
       </c>
       <c r="Q17" s="1" t="inlineStr">
         <is>
-          <t>grid/true MEASURED; effective MEASURED; native MEASURED (service catalog)</t>
-        </is>
-      </c>
-      <c r="R17" s="1" t="inlineStr"/>
-      <c r="S17" s="1" t="inlineStr"/>
-      <c r="T17" s="1" t="inlineStr"/>
+          <t>grid/true/effective MEASURED (acquire_imagery verify 2026-08-23); native MEASURED (service catalog LowPS=1)</t>
+        </is>
+      </c>
+      <c r="R17" s="1" t="inlineStr">
+        <is>
+          <t>2015-08-07 15:31 (HXIP 2015 1-ft flight; EXCLUDED for this product)</t>
+        </is>
+      </c>
+      <c r="S17" s="1" t="inlineStr">
+        <is>
+          <t>https://services.arcgis.com/jsIt88o09Q0r1j8h/arcgis/rest/services/NAIP_2015_1ft_Ortho_Dates_and_Times_83s/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="T17" s="1" t="inlineStr">
+        <is>
+          <t>"THEMENAME":"hxip_m_4712213_se_10_30","SDATE":"08/07/2015 15:31","SUNEL":46,"ACCURACY":"0.72m (ce 95%)" (city-centroid point query; raw response qc/imagery_date_evidence/raw_records/wa_2015_1ft_citycentroid.json)</t>
+        </is>
+      </c>
       <c r="U17" s="1" t="inlineStr">
         <is>
           <t>held imagery</t>
@@ -13896,104 +13939,92 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>2017_coe_rgb.tif</t>
+          <t>2021_snoh_rgbi.tif</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>2017 (CoE)</t>
+          <t>2021 (Snoh)</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>City of Edmonds Basemap/2017_Aerial_Cached (source raster 2017_Aerial.tif, 0.25 ftUS EPSG:2285, JPEG); CONTENT = King County IMAGE_Ortho2017KCNAT (Pictometry International, 3-in 'Neighborhood' tier covering southwestern Snohomish County) - MEASURED identity</t>
+          <t>HXIP via Snohomish County Imagery/Aerial_2021 ImageServer (mosaic gdb HXIP_2021_SNOHOMISH.gdb - a Hexagon delivery, not EagleView)</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
         <is>
-          <t>0.074646</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>metre (Web Mercator, inflated 1/cos(lat))</t>
+          <t>US survey foot</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>EPSG:3857</t>
+          <t>EPSG:2285</t>
         </is>
       </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>5.01</t>
+          <t>15.24</t>
         </is>
       </c>
       <c r="H18" s="1" t="inlineStr">
         <is>
-          <t>7.6 (indicative; per-site sd +/-0.41-1.17 px)</t>
+          <t>20.6</t>
         </is>
       </c>
       <c r="I18" s="1" t="inlineStr">
         <is>
-          <t>7.62 (0.25 ftUS source raster; service pixelSizeX 0.07620015240030481 m = 0.250000 ftUS exactly)</t>
+          <t>15.24 (0.5 ft): mosaic-catalog LowPS=0.5, item pixelSizeX=0.5 (MEASURED)</t>
         </is>
       </c>
       <c r="J18" s="1" t="inlineStr">
         <is>
-          <t>2017-05-04 to 2017-05-10 (5 days over the city: May 4 n=16, May 6 90, May 8 48, May 9 192, May 10 364) - transferred from the King County per-frame index because the two files are the SAME ORTHOMOSAIC</t>
+          <t>2021-06-25 to 2021-11-11</t>
         </is>
       </c>
       <c r="K18" s="1" t="inlineStr">
         <is>
-          <t>window of 7 days, 5 flight days</t>
+          <t>window of 140 days (weather trims to 108 feasible days; 18 late days never reach 30 deg sun)</t>
         </is>
       </c>
       <c r="L18" s="1" t="inlineStr">
         <is>
-          <t>MULTI (5 days)</t>
-        </is>
-      </c>
-      <c r="M18" s="6" t="inlineStr">
-        <is>
-          <t>MEASURED</t>
+          <t>unknown; held crop flown in the AFTERNOON (shadow azimuth 67-91 deg = sun at 247-256 deg, uniform over 24 windows) - a time-of-day constraint, not a date</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="N18" s="1" t="inlineStr">
         <is>
-          <t>https://services.arcgis.com/Ej0PsM5Aw677QF1W/arcgis/rest/services/ORTHO_IMAGE17_AREA_2685/FeatureServer/0/query</t>
+          <t>https://snohomishcountywa.gov/5414/Interactive-Map-SCOPI</t>
         </is>
       </c>
       <c r="O18" s="1" t="inlineStr">
         <is>
-          <t>"ImageName":"WAKING043402NeighOrtho01390_170509" ... "ShotDate":"2017/05/09 17:20:09" (King County 2017 index, first of 710 frames intersecting the city polygon; raw response qc/imagery_date_evidence/raw_records/kc_2017_ORTHO_IMAGE17_AREA_2685_citypoly_first3.json). Dates transfer because the two files are the same orthomosaic - see notes.</t>
+          <t>The 2021 aerial photos are 6 inch resolution and cover mainly the urban areas. The imagery was collected between June 25, 2021 and November 11, 2021.</t>
         </is>
       </c>
       <c r="P18" s="1" t="inlineStr">
         <is>
-          <t>Identity MEASURED 2026-08-23: held 2017_coe_rgb.tif (2x boxcar-downsampled) vs 2017_king_rgb.tif over a 12x12 grid on the city polygon, 66 valid 512-px windows -&gt; r min 0.9568, p5 0.9786, median 0.9923, max 0.9966, MAE median 3.54 DN; live services 2017_Aerial_Cached vs KingCo_Aerial_2017 LOD-20 tiles at 5 sites r = 0.9876-0.9935. Identical vehicles in identical stalls and identical building relief displacement -&gt; same orthorectification, not merely the same flight. Retires the 8.5-month candidate window and the council-minutes line (2023-07-25 p.15, 'PlanIt Geo ... 2017 flyovers') as evidence - the 2019 UFMP was written by Davey Resource Group and its canopy work used Aug 2015 imagery; PlanIt Geo appears nowhere in it. No City of Edmonds document naming the 2017 vendor was found; attribution rests on measured pixel identity plus King County's published coverage statement (alt). Snohomish County's own 2017 product is a 1-ft HXIP flight (2017-08-15/21) and cannot be a 3-in source. Grid note: the held grid is exactly LOD 21, which King's tile endpoint does not serve (404 at L21) but Edmonds' does - consistent with a city-service export. Method detail: qc/imagery_date_evidence/coe2017_identity/.</t>
+          <t>CLOSED LEADS: no WA consortium flight-date layer exists for 2021 or later (all 68 WAGeoservices services + 225 items enumerated; series ends 2020); the mosaic-catalog schema has no date field at all; WA NAIP 2021 does not cover quad 47122 (eastern WA only), so no NAIP ride-along date. Remaining route: the Hexagon flight log via Snohomish County DoIT, or the consortium contact (Joanne Markert, WA OCIO). Weather elimination (ASOS KPAE+KSEA+KBFI, criterion calibrated to 46/46 known Edmonds flight days; 2021-06-25..11-11): 32 of 140 days eliminated; longest feasible blocks Jul 22-Aug 6, Jul 2-15, Aug 9-19. ELIMINATES ONLY - no surviving day is favoured. Per-day table: qc/imagery_date_evidence/weather/flyable_days.csv.</t>
         </is>
       </c>
       <c r="Q18" s="1" t="inlineStr">
         <is>
-          <t>grid/true MEASURED; effective MEASURED; native MEASURED (live service)</t>
-        </is>
-      </c>
-      <c r="R18" s="1" t="inlineStr">
-        <is>
-          <t>mid-February through October 2017 (countywide), with SW Snohomish at 3 in</t>
-        </is>
-      </c>
-      <c r="S18" s="1" t="inlineStr">
-        <is>
-          <t>https://gisandyou.org/2018/05/25/2017-aerial-imagery-in-imap/</t>
-        </is>
-      </c>
-      <c r="T18" s="1" t="inlineStr">
-        <is>
-          <t>The imagery was captured by Pictometry International Corp. from mid-February through October of 2017. The original photos have a resolution of 3 inches per pixel ("Neighborhood" scale in Pictometry terminology) over urbanized, western King County ... Also covered at the Neighborhood resolution level in the 2017 imagery are southwestern Snohomish County</t>
-        </is>
-      </c>
+          <t>grid/true MEASURED; effective MEASURED; native MEASURED (service catalog)</t>
+        </is>
+      </c>
+      <c r="R18" s="1" t="inlineStr"/>
+      <c r="S18" s="1" t="inlineStr"/>
+      <c r="T18" s="1" t="inlineStr"/>
       <c r="U18" s="1" t="inlineStr">
         <is>
           <t>held imagery</t>
@@ -14003,17 +14034,17 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>2020_coe_rgb.tif</t>
+          <t>2017_coe_rgb.tif</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>2020 (ANCHOR)</t>
+          <t>2017 (CoE)</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>City of Edmonds Basemap/2020_Aerial_Cached (MrSID/MG4 mosaic, GeoExpress 10.0.1.5035, input GeoTIFF set 665,235,977,256 B); source = Snohomish County 2020 EagleView/Pictometry regional project WASNOH20_3in per the 2021 ILA; product identity corroborated by Everett's copy ('Aerial Photos 2020 Pictometry Mosiac 3 inch resolution urban areas', 0.25 ftUS)</t>
+          <t>City of Edmonds Basemap/2017_Aerial_Cached (source raster 2017_Aerial.tif, 0.25 ftUS EPSG:2285, JPEG); CONTENT = King County IMAGE_Ortho2017KCNAT (Pictometry International, 3-in 'Neighborhood' tier covering southwestern Snohomish County) - MEASURED identity</t>
         </is>
       </c>
       <c r="D19" s="1" t="inlineStr">
@@ -14038,67 +14069,67 @@
       </c>
       <c r="H19" s="1" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>7.6 (indicative; per-site sd +/-0.41-1.17 px)</t>
         </is>
       </c>
       <c r="I19" s="1" t="inlineStr">
         <is>
-          <t>7.62 (0.25 ftUS; county Aerial_2020 LowCellSize 0.25, dimResol 0.250000 ftUS; Everett Image2020jp2 pixelSizeX 0.25 in EPSG:2285)</t>
+          <t>7.62 (0.25 ftUS source raster; service pixelSizeX 0.07620015240030481 m = 0.250000 ftUS exactly)</t>
         </is>
       </c>
       <c r="J19" s="1" t="inlineStr">
         <is>
-          <t>2020-04-13 to 2020-07-13 (county window; the single published window is the UNION of the 3-in urban and 9-in rural sub-projects - unlike 2022/2024 the county did not publish them separately). Shadow solar geometry excludes the head: 2020-04-25 to 07-13 survive (80 of 92 days)</t>
+          <t>2017-05-04 to 2017-05-10 (5 days over the city: May 4 n=16, May 6 90, May 8 48, May 9 192, May 10 364) - transferred from the King County per-frame index because the two files are the SAME ORTHOMOSAIC</t>
         </is>
       </c>
       <c r="K19" s="1" t="inlineStr">
         <is>
-          <t>window of 80-92 days</t>
+          <t>window of 7 days, 5 flight days</t>
         </is>
       </c>
       <c r="L19" s="1" t="inlineStr">
         <is>
-          <t>CONSISTENT WITH ONE CONTINUOUS PASS, single date NOT PROVEN: 10 QC-passing sites of 34 on a ~850 m city-wide grid give sun azimuths 120.8-192.5 deg = local times ~10:22-13:39 PDT straddling solar noon, increasing monotonically east-to-west (az vs lon r=-0.75, p=0.013; permutation p=0.026) - the signature of successive flight lines in one pass, not of day-blocks. Not excluded: several dates each flown at the same time of day.</t>
-        </is>
-      </c>
-      <c r="M19" s="7" t="inlineStr">
-        <is>
-          <t>INFERRED</t>
+          <t>MULTI (5 days)</t>
+        </is>
+      </c>
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
         </is>
       </c>
       <c r="N19" s="1" t="inlineStr">
         <is>
-          <t>https://snohomishcountywa.gov/5414/Interactive-Map-SCOPI</t>
+          <t>https://services.arcgis.com/Ej0PsM5Aw677QF1W/arcgis/rest/services/ORTHO_IMAGE17_AREA_2685/FeatureServer/0/query</t>
         </is>
       </c>
       <c r="O19" s="1" t="inlineStr">
         <is>
-          <t>The 2020 aerial photos are 3 inch resolution in the urban areas and 9 inch resolution in the rural areas, excluding much of the unpopulated mountainous portion of eastern Snohomish County, and were taken between April 13th and July 13th, 2020.</t>
+          <t>"ImageName":"WAKING043402NeighOrtho01390_170509" ... "ShotDate":"2017/05/09 17:20:09" (King County 2017 index, first of 710 frames intersecting the city polygon; raw response qc/imagery_date_evidence/raw_records/kc_2017_ORTHO_IMAGE17_AREA_2685_citypoly_first3.json). Dates transfer because the two files are the same orthomosaic - see notes.</t>
         </is>
       </c>
       <c r="P19" s="1" t="inlineStr">
         <is>
-          <t>ILA 2021 (Laserfiche id 1462454, repo=Edmonds) Work Order p.14: 'Upon completion of the 2020, 2022 and 2024 EagleView regional aerial imagery acquisition projects ... County will provide Edmonds with orthogonal imagery for Edmonds's identified area of interest'. Contract vehicle for a records request: King County RFP 1166-18-PCR (EagleView Technology Corp) via Snohomish County Piggyback PB-19-14BC (Legistar matter 2024-1168). DEFINITIVE PIN = EagleView flight log / photo-centre index via Snohomish County DoIT (Viggo Forde), or a CONNECTExplorer capture-date screenshot (Edmonds holds up to ten accounts under the ILA). City keyProperties (correct endpoint &lt;ImageServer&gt;/keyProperties?f=json; /info/keyProperties 400s on this server, positive control Edmonds_Marsh_2018 returns acquisitionStartDate 2018-08-01T16:22:13+00:00 / End 16:52:13) carry NO date: IMAGE__MODIFICATIONS 'COMPRESSED EMBEDDED MASKED MOSAICKED' - a validated null. Everett's 2020 copy is JPEG2000 and also carries no date; no 2020 MrSID twin with a surviving date was found. A per-frame index CANNOT exist on the county service (mosaic catalog = two whole-project items WASNOH20_3in / WASNOH20_9in). HAZARD: a SECOND 2020 acquisition covers Edmonds - the WA consortium 6-in Hexagon/ADS100 flight of 2020-08-27/28 (program window 2020-08-03..09-06) - DO NOT borrow its date (see context row). Shadow dating (qc/imagery_date_evidence/shadow_dating_2020/): azimuth is reliable (2012 control 8/10 in-window), elevation reads LOW and saturates above ~45 deg, so 2020 elevations are lower bounds - hence no calendar date. 2020 ortho co-registered to 2012 within &lt;=1.5 WM m. Weather elimination (ASOS KPAE+KSEA+KBFI, criterion calibrated to 46/46 known Edmonds flight days; 2020-04-13..07-13): 22 of 92 days eliminated; longest feasible blocks May 7-15 (9 d), Apr 13-17, May 26-30, Jun 1-5, Jun 22-26. ELIMINATES ONLY - no surviving day is favoured. Per-day table: qc/imagery_date_evidence/weather/flyable_days.csv.</t>
+          <t>Identity MEASURED 2026-08-23: held 2017_coe_rgb.tif (2x boxcar-downsampled) vs 2017_king_rgb.tif over a 12x12 grid on the city polygon, 66 valid 512-px windows -&gt; r min 0.9568, p5 0.9786, median 0.9923, max 0.9966, MAE median 3.54 DN; live services 2017_Aerial_Cached vs KingCo_Aerial_2017 LOD-20 tiles at 5 sites r = 0.9876-0.9935. Identical vehicles in identical stalls and identical building relief displacement -&gt; same orthorectification, not merely the same flight. Retires the 8.5-month candidate window and the council-minutes line (2023-07-25 p.15, 'PlanIt Geo ... 2017 flyovers') as evidence - the 2019 UFMP was written by Davey Resource Group and its canopy work used Aug 2015 imagery; PlanIt Geo appears nowhere in it. No City of Edmonds document naming the 2017 vendor was found; attribution rests on measured pixel identity plus King County's published coverage statement (alt). Snohomish County's own 2017 product is a 1-ft HXIP flight (2017-08-15/21) and cannot be a 3-in source. Grid note: the held grid is exactly LOD 21, which King's tile endpoint does not serve (404 at L21) but Edmonds' does - consistent with a city-service export. Method detail: qc/imagery_date_evidence/coe2017_identity/.</t>
         </is>
       </c>
       <c r="Q19" s="1" t="inlineStr">
         <is>
-          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED (county + Everett services)</t>
+          <t>grid/true MEASURED; effective MEASURED; native MEASURED (live service)</t>
         </is>
       </c>
       <c r="R19" s="1" t="inlineStr">
         <is>
-          <t>(ILA text, for the chain)</t>
+          <t>mid-February through October 2017 (countywide), with SW Snohomish at 3 in</t>
         </is>
       </c>
       <c r="S19" s="1" t="inlineStr">
         <is>
-          <t>https://weblink.edmondswa.gov/WebLink/DocView.aspx?id=1462454&amp;dbid=0&amp;repo=Edmonds</t>
+          <t>https://gisandyou.org/2018/05/25/2017-aerial-imagery-in-imap/</t>
         </is>
       </c>
       <c r="T19" s="1" t="inlineStr">
         <is>
-          <t>Upon completion of the 2020, 2022 and 2024 EagleView regional aerial imagery acquisition projects and receipt of imagery by County, County will provide Edmonds with orthogonal imagery for Edmonds's identified area of interest</t>
+          <t>The imagery was captured by Pictometry International Corp. from mid-February through October of 2017. The original photos have a resolution of 3 inches per pixel ("Neighborhood" scale in Pictometry terminology) over urbanized, western King County ... Also covered at the Neighborhood resolution level in the 2017 imagery are southwestern Snohomish County</t>
         </is>
       </c>
       <c r="U19" s="1" t="inlineStr">
@@ -14110,17 +14141,17 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>2022_coe_rgb.tif</t>
+          <t>2020_coe_rgb.tif</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>2022 (CoE)</t>
+          <t>2020 (ANCHOR)</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>City of Edmonds Basemap/2022_Aerial_Cached; = Snohomish County 2022 regional project WASNOH22_3in. IDENTITY MEASURED: the Edmonds and Everett 2022 MrSIDs are the same county encode (identical input-set byte count 675,609,635,568 B, GeoExpress 10.0.1.5035, EPSG:2285 ftUS geokeys)</t>
+          <t>City of Edmonds Basemap/2020_Aerial_Cached (MrSID/MG4 mosaic, GeoExpress 10.0.1.5035, input GeoTIFF set 665,235,977,256 B); source = Snohomish County 2020 EagleView/Pictometry regional project WASNOH20_3in per the 2021 ILA; product identity corroborated by Everett's copy ('Aerial Photos 2020 Pictometry Mosiac 3 inch resolution urban areas', 0.25 ftUS)</t>
         </is>
       </c>
       <c r="D20" s="1" t="inlineStr">
@@ -14145,32 +14176,32 @@
       </c>
       <c r="H20" s="1" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="I20" s="1" t="inlineStr">
         <is>
-          <t>7.62 (0.25 ftUS; county Aerial_2022 LowCellSize 0.25; MrSID input GeoTIFF geokeys 'Linear_Foot_US_Survey' / 2285)</t>
+          <t>7.62 (0.25 ftUS; county Aerial_2020 LowCellSize 0.25, dimResol 0.250000 ftUS; Everett Image2020jp2 pixelSizeX 0.25 in EPSG:2285)</t>
         </is>
       </c>
       <c r="J20" s="1" t="inlineStr">
         <is>
-          <t>2022-04-06 to 2022-07-11 (urban 3 in); the rural 9-in sub-project ran 2022-05-31 to 08-11 and does not apply to Edmonds</t>
+          <t>2020-04-13 to 2020-07-13 (county window; the single published window is the UNION of the 3-in urban and 9-in rural sub-projects - unlike 2022/2024 the county did not publish them separately). Shadow solar geometry excludes the head: 2020-04-25 to 07-13 survive (80 of 92 days)</t>
         </is>
       </c>
       <c r="K20" s="1" t="inlineStr">
         <is>
-          <t>window of 96 days</t>
+          <t>window of 80-92 days</t>
         </is>
       </c>
       <c r="L20" s="1" t="inlineStr">
         <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="M20" s="4" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+          <t>CONSISTENT WITH ONE CONTINUOUS PASS, single date NOT PROVEN: 10 QC-passing sites of 34 on a ~850 m city-wide grid give sun azimuths 120.8-192.5 deg = local times ~10:22-13:39 PDT straddling solar noon, increasing monotonically east-to-west (az vs lon r=-0.75, p=0.013; permutation p=0.026) - the signature of successive flight lines in one pass, not of day-blocks. Not excluded: several dates each flown at the same time of day.</t>
+        </is>
+      </c>
+      <c r="M20" s="7" t="inlineStr">
+        <is>
+          <t>INFERRED</t>
         </is>
       </c>
       <c r="N20" s="1" t="inlineStr">
@@ -14180,12 +14211,12 @@
       </c>
       <c r="O20" s="1" t="inlineStr">
         <is>
-          <t>The 2022 3 inch resolution aerial photos in the urban areas, were captured between April 6, 2022 and July, 11 2022. The 2022 9 inch resolution aerial photos in the rural areas, were captured between May, 31 2022 and August, 11 2022.</t>
+          <t>The 2020 aerial photos are 3 inch resolution in the urban areas and 9 inch resolution in the rural areas, excluding much of the unpopulated mountainous portion of eastern Snohomish County, and were taken between April 13th and July 13th, 2020.</t>
         </is>
       </c>
       <c r="P20" s="1" t="inlineStr">
         <is>
-          <t>Upgraded INFERRED -&gt; PUBLISHED 2026-08-23: the window is published for a product whose identity with the held file is now measured (byte-count identity of the input set with Everett's Image2022_3in_sid, 'Aerial Photos 2022 Pictometry Mosaic 3 inch resolution urban areas'), not only contractual. Same definitive pin as 2020 (one PRR covers 2020/2022/2024). Weather elimination (ASOS KPAE+KSEA+KBFI, criterion calibrated to 46/46 known Edmonds flight days; 2022-04-06..07-11): 19 of 97 days eliminated (weakest of the four windows - a settled spring); longest feasible block May 16-28 (13 d). ELIMINATES ONLY - no surviving day is favoured. Per-day table: qc/imagery_date_evidence/weather/flyable_days.csv.</t>
+          <t>ILA 2021 (Laserfiche id 1462454, repo=Edmonds) Work Order p.14: 'Upon completion of the 2020, 2022 and 2024 EagleView regional aerial imagery acquisition projects ... County will provide Edmonds with orthogonal imagery for Edmonds's identified area of interest'. Contract vehicle for a records request: King County RFP 1166-18-PCR (EagleView Technology Corp) via Snohomish County Piggyback PB-19-14BC (Legistar matter 2024-1168). DEFINITIVE PIN = EagleView flight log / photo-centre index via Snohomish County DoIT (Viggo Forde), or a CONNECTExplorer capture-date screenshot (Edmonds holds up to ten accounts under the ILA). City keyProperties (correct endpoint &lt;ImageServer&gt;/keyProperties?f=json; /info/keyProperties 400s on this server, positive control Edmonds_Marsh_2018 returns acquisitionStartDate 2018-08-01T16:22:13+00:00 / End 16:52:13) carry NO date: IMAGE__MODIFICATIONS 'COMPRESSED EMBEDDED MASKED MOSAICKED' - a validated null. Everett's 2020 copy is JPEG2000 and also carries no date; no 2020 MrSID twin with a surviving date was found. A per-frame index CANNOT exist on the county service (mosaic catalog = two whole-project items WASNOH20_3in / WASNOH20_9in). HAZARD: a SECOND 2020 acquisition covers Edmonds - the WA consortium 6-in Hexagon/ADS100 flight of 2020-08-27/28 (program window 2020-08-03..09-06) - DO NOT borrow its date (see context row). Shadow dating (qc/imagery_date_evidence/shadow_dating_2020/): azimuth is reliable (2012 control 8/10 in-window), elevation reads LOW and saturates above ~45 deg, so 2020 elevations are lower bounds - hence no calendar date. 2020 ortho co-registered to 2012 within &lt;=1.5 WM m. Weather elimination (ASOS KPAE+KSEA+KBFI, criterion calibrated to 46/46 known Edmonds flight days; 2020-04-13..07-13): 22 of 92 days eliminated; longest feasible blocks May 7-15 (9 d), Apr 13-17, May 26-30, Jun 1-5, Jun 22-26. ELIMINATES ONLY - no surviving day is favoured. Per-day table: qc/imagery_date_evidence/weather/flyable_days.csv.</t>
         </is>
       </c>
       <c r="Q20" s="1" t="inlineStr">
@@ -14195,17 +14226,17 @@
       </c>
       <c r="R20" s="1" t="inlineStr">
         <is>
-          <t>(Everett keyProperties - identity proof)</t>
+          <t>(ILA text, for the chain)</t>
         </is>
       </c>
       <c r="S20" s="1" t="inlineStr">
         <is>
-          <t>https://gismaps.everettwa.gov/manarcgis/rest/services/Imagery/Image2022_3in_sid/ImageServer/keyProperties?f=json</t>
+          <t>https://weblink.edmondswa.gov/WebLink/DocView.aspx?id=1462454&amp;dbid=0&amp;repo=Edmonds</t>
         </is>
       </c>
       <c r="T20" s="1" t="inlineStr">
         <is>
-          <t>"IMAGE__ENCODING_APPLICATION":"GeoExpress 10.0.1.5035","IMAGE__FORMAT":"MrSID/MG4","IMAGE__INPUT_FILE_SIZE":"675609635568.000000","IMAGE__INPUT_FORMAT":"GeoTIFF" ... "IMAGE__MODIFICATIONS":"COMPRESSED EMBEDDED MASKED MOSAICKED"</t>
+          <t>Upon completion of the 2020, 2022 and 2024 EagleView regional aerial imagery acquisition projects and receipt of imagery by County, County will provide Edmonds with orthogonal imagery for Edmonds's identified area of interest</t>
         </is>
       </c>
       <c r="U20" s="1" t="inlineStr">
@@ -14217,17 +14248,17 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>2024_coe_rgb.tif</t>
+          <t>2022_coe_rgb.tif</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>2024 (CoE)</t>
+          <t>2022 (CoE)</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>City of Edmonds Basemap/2024_Aerial_Cached (MapServer over Edmonds2024.sid - no ImageServer, so no keyProperties resource exists); source = Snohomish County 2024 regional project WASNOH24_3in per the 2021 ILA</t>
+          <t>City of Edmonds Basemap/2022_Aerial_Cached; = Snohomish County 2022 regional project WASNOH22_3in. IDENTITY MEASURED: the Edmonds and Everett 2022 MrSIDs are the same county encode (identical input-set byte count 675,609,635,568 B, GeoExpress 10.0.1.5035, EPSG:2285 ftUS geokeys)</t>
         </is>
       </c>
       <c r="D21" s="1" t="inlineStr">
@@ -14252,22 +14283,22 @@
       </c>
       <c r="H21" s="1" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="I21" s="1" t="inlineStr">
         <is>
-          <t>7.62 (0.25 ftUS; county Aerial_2024 LowCellSize 0.25)</t>
+          <t>7.62 (0.25 ftUS; county Aerial_2022 LowCellSize 0.25; MrSID input GeoTIFF geokeys 'Linear_Foot_US_Survey' / 2285)</t>
         </is>
       </c>
       <c r="J21" s="1" t="inlineStr">
         <is>
-          <t>2024-03-31 to 2024-05-31 (urban 3 in); the rural 9-in sub-project ran 2024-03-16 to 06-09</t>
+          <t>2022-04-06 to 2022-07-11 (urban 3 in); the rural 9-in sub-project ran 2022-05-31 to 08-11 and does not apply to Edmonds</t>
         </is>
       </c>
       <c r="K21" s="1" t="inlineStr">
         <is>
-          <t>window of 62 days</t>
+          <t>window of 96 days</t>
         </is>
       </c>
       <c r="L21" s="1" t="inlineStr">
@@ -14275,9 +14306,9 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="M21" s="7" t="inlineStr">
-        <is>
-          <t>INFERRED</t>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="N21" s="1" t="inlineStr">
@@ -14287,32 +14318,32 @@
       </c>
       <c r="O21" s="1" t="inlineStr">
         <is>
-          <t>The 2024 3 inch resolution aerial photos in the urban areas, were captured between March 31, 2024 and May, 31 2024. The 2024 9 inch resolution aerial photos in the rural areas, were captured between March, 16 2024 and June, 9 2024.</t>
+          <t>The 2022 3 inch resolution aerial photos in the urban areas, were captured between April 6, 2022 and July, 11 2022. The 2022 9 inch resolution aerial photos in the rural areas, were captured between May, 31 2022 and August, 11 2022.</t>
         </is>
       </c>
       <c r="P21" s="1" t="inlineStr">
         <is>
-          <t>Stays INFERRED: no neighbour city holds a 2024 county copy (Everett stops at 2022, Mukilteo at 2019, Lynnwood publishes none), so there is no 2024 analogue of the 2022 byte-identity proof. Same definitive pin as 2020. Weather elimination (ASOS KPAE+KSEA+KBFI, criterion calibrated to 46/46 known Edmonds flight days; 2024-03-31..05-31): 18 of 62 days eliminated (29%, strongest of the four); longest feasible block Apr 16-24 (9 d). ELIMINATES ONLY - no surviving day is favoured. Per-day table: qc/imagery_date_evidence/weather/flyable_days.csv.</t>
+          <t>Upgraded INFERRED -&gt; PUBLISHED 2026-08-23: the window is published for a product whose identity with the held file is now measured (byte-count identity of the input set with Everett's Image2022_3in_sid, 'Aerial Photos 2022 Pictometry Mosaic 3 inch resolution urban areas'), not only contractual. Same definitive pin as 2020 (one PRR covers 2020/2022/2024). Weather elimination (ASOS KPAE+KSEA+KBFI, criterion calibrated to 46/46 known Edmonds flight days; 2022-04-06..07-11): 19 of 97 days eliminated (weakest of the four windows - a settled spring); longest feasible block May 16-28 (13 d). ELIMINATES ONLY - no surviving day is favoured. Per-day table: qc/imagery_date_evidence/weather/flyable_days.csv.</t>
         </is>
       </c>
       <c r="Q21" s="1" t="inlineStr">
         <is>
-          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED (county service)</t>
+          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED (county + Everett services)</t>
         </is>
       </c>
       <c r="R21" s="1" t="inlineStr">
         <is>
-          <t>(ILA text)</t>
+          <t>(Everett keyProperties - identity proof)</t>
         </is>
       </c>
       <c r="S21" s="1" t="inlineStr">
         <is>
-          <t>https://weblink.edmondswa.gov/WebLink/DocView.aspx?id=1462454&amp;dbid=0&amp;repo=Edmonds</t>
+          <t>https://gismaps.everettwa.gov/manarcgis/rest/services/Imagery/Image2022_3in_sid/ImageServer/keyProperties?f=json</t>
         </is>
       </c>
       <c r="T21" s="1" t="inlineStr">
         <is>
-          <t>Upon completion of the 2020, 2022 and 2024 EagleView regional aerial imagery acquisition projects ...</t>
+          <t>"IMAGE__ENCODING_APPLICATION":"GeoExpress 10.0.1.5035","IMAGE__FORMAT":"MrSID/MG4","IMAGE__INPUT_FILE_SIZE":"675609635568.000000","IMAGE__INPUT_FORMAT":"GeoTIFF" ... "IMAGE__MODIFICATIONS":"COMPRESSED EMBEDDED MASKED MOSAICKED"</t>
         </is>
       </c>
       <c r="U21" s="1" t="inlineStr">
@@ -14324,62 +14355,62 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>(not held) City of Edmonds Basemap/2015_Aerial_Cached</t>
+          <t>2024_coe_rgb.tif</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>2015 (CoE service)</t>
+          <t>2024 (CoE)</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>City of Edmonds (source raster Ed_Aerial_2015.tif, 0.25 ftUS EPSG:2285, LZW); content INFERRED = 2015 Western Washington Regional Orthophotography (King County lead, 88 participants; prime GeoTerra, Edmonds frames flown by Valley Air and GeoTerra)</t>
+          <t>City of Edmonds Basemap/2024_Aerial_Cached (MapServer over Edmonds2024.sid - no ImageServer, so no keyProperties resource exists); source = Snohomish County 2024 regional project WASNOH24_3in per the 2021 ILA</t>
         </is>
       </c>
       <c r="D22" s="1" t="inlineStr">
         <is>
-          <t>LOD 21 cache (0.0746 WM m)</t>
+          <t>0.074646</t>
         </is>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>metre (Web Mercator)</t>
+          <t>metre (Web Mercator, inflated 1/cos(lat))</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>EPSG:3857 (cache); source EPSG:2285</t>
+          <t>EPSG:3857</t>
         </is>
       </c>
       <c r="G22" s="1" t="inlineStr">
         <is>
-          <t>5.01 (cache) / 7.62 (source)</t>
+          <t>5.01</t>
         </is>
       </c>
       <c r="H22" s="1" t="inlineStr">
         <is>
-          <t>not measured</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="I22" s="1" t="inlineStr">
         <is>
-          <t>&lt;= 6.86 flown (MAX_GSD 0.225 ft 'as planned' for all 346 Edmonds frames; two cameras at two altitudes both back-compute to ~6.6-6.9 cm), delivered at the 0.25 ft = 7.62 cm tier (service pixelSizeX 0.07620015240030481 m = 0.250000 ftUS)</t>
+          <t>7.62 (0.25 ftUS; county Aerial_2024 LowCellSize 0.25)</t>
         </is>
       </c>
       <c r="J22" s="1" t="inlineStr">
         <is>
-          <t>2015-04-08 (n=135 photo centres in the city polygon; Valley Air, UltraCam X, 14:13-15:04 PDT) and 2015-04-17 (n=32; GeoTerra, UltraCam Xp, 12:54-13:55 PDT). CONTEST largely resolved: the King Pictometry leg is EXCLUDED by pixel comparison, the 'Aug 7 2015' leg is a DIFFERENT dataset (NAIP/HXIP 2015-08-07), leaving the consortium dates; attribution of Ed_Aerial_2015.tif to the consortium remains INFERRED and the UFMP's '4.8 in' figure is unexplained</t>
+          <t>2024-03-31 to 2024-05-31 (urban 3 in); the rural 9-in sub-project ran 2024-03-16 to 06-09</t>
         </is>
       </c>
       <c r="K22" s="1" t="inlineStr">
         <is>
-          <t>2 flight days (window of 10 days) for the consortium product</t>
+          <t>window of 62 days</t>
         </is>
       </c>
       <c r="L22" s="1" t="inlineStr">
         <is>
-          <t>MULTI - two days, two vendors, two cameras within the city (flightlines 16002-16011 Zone 16 / 13007-13015 Zone 13)</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="M22" s="7" t="inlineStr">
@@ -14389,166 +14420,166 @@
       </c>
       <c r="N22" s="1" t="inlineStr">
         <is>
-          <t>https://services.arcgis.com/Ej0PsM5Aw677QF1W/arcgis/rest/services/ORTHO_IMAGE15C_POINT_2574/FeatureServer/0/query</t>
+          <t>https://snohomishcountywa.gov/5414/Interactive-Map-SCOPI</t>
         </is>
       </c>
       <c r="O22" s="1" t="inlineStr">
         <is>
-          <t>"FILENAME":"13009_57445" ... "UTC_TIME":"19:54:49","MAX_GSD__f":0.225 ... "VENDOR":"GeoTerra","CAMERA":"UltraCam Xp" ... "FLIGHTLINE":"13009","ACQ_DATE":1429228800000 (= 2015-04-17 UTC; first of the photo centres inside the city polygon; raw response qc/imagery_date_evidence/raw_records/kc_2015C_ORTHO_IMAGE15C_POINT_2574_citypoly_first3.json). Layer description: It is a reference for the raw image scans, it is not a index for tiled ortho imagery</t>
+          <t>The 2024 3 inch resolution aerial photos in the urban areas, were captured between March 31, 2024 and May, 31 2024. The 2024 9 inch resolution aerial photos in the rural areas, were captured between March, 16 2024 and June, 9 2024.</t>
         </is>
       </c>
       <c r="P22" s="1" t="inlineStr">
         <is>
-          <t>Photo-centre DAYS are MEASURED; binding them to Ed_Aerial_2015.tif is INFERRED via (a) 0.25 ftUS cell size matching the consortium tier, (b) CRS NAD83 SP WA North ftUS, (c) Edmonds named in GeoTerra's participant table and the consortium agreement signed 2015-06-23 ($3,696.21), (d) leaf-off/high-sun spec matching the tiles. NOTE: no Apr 9 frames exist over Edmonds (the catalogue's 'Apr 8/9/17' was wrong); one Mar 26 frame sits just outside the polygon. King leg excluded: CoE 2015 vs KingCo_Aerial_2015 LOD-20 tiles r=0.036-0.557 at 5 sites vs r=0.988-0.994 for the CoE-2017/King-2017 control. 'Aug 7 2015 / 4.8 in' (UFMP 2019 p.26) traces to the Davey Resource Group 2018 UTC Assessment which names 'USDA, Farm Service Agency' = NAIP 2015 (2015-08-07, 1 m = the same Hexagon flight as the HXIP 1-ft consortium product); '4.8 in' matches no known 2015 product. Phenology caveat from the project's own survey report: 'the need to begin immediate image acquisition due an earlier than normal bud break' - Apr 8/17 is late in a leaf-off window. Vendor/camera cross-validated at serial-number level against the Flight Subcontractor PDF (UCX 60418665 / UCXp 10411033).</t>
+          <t>Stays INFERRED: no neighbour city holds a 2024 county copy (Everett stops at 2022, Mukilteo at 2019, Lynnwood publishes none), so there is no 2024 analogue of the 2022 byte-identity proof. Same definitive pin as 2020. Weather elimination (ASOS KPAE+KSEA+KBFI, criterion calibrated to 46/46 known Edmonds flight days; 2024-03-31..05-31): 18 of 62 days eliminated (29%, strongest of the four); longest feasible block Apr 16-24 (9 d). ELIMINATES ONLY - no surviving day is favoured. Per-day table: qc/imagery_date_evidence/weather/flyable_days.csv.</t>
         </is>
       </c>
       <c r="Q22" s="1" t="inlineStr">
         <is>
-          <t>grid MEASURED (live service); native MEASURED (index MAX_GSD) + PUBLISHED (tier)</t>
+          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED (county service)</t>
         </is>
       </c>
       <c r="R22" s="1" t="inlineStr">
         <is>
-          <t>2015-08-07 15:31 (UFMP/Davey 'August 7th, 2015' imagery = NAIP/HXIP 2015, NOT the city basemap)</t>
+          <t>(ILA text)</t>
         </is>
       </c>
       <c r="S22" s="1" t="inlineStr">
         <is>
-          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2015/wa_fgdc_2015/47122/m_4712214_sw_10_1_20150807.txt</t>
+          <t>https://weblink.edmondswa.gov/WebLink/DocView.aspx?id=1462454&amp;dbid=0&amp;repo=Edmonds</t>
         </is>
       </c>
       <c r="T22" s="1" t="inlineStr">
         <is>
-          <t>Time_Period_of_Content: Time_Period_Information: Single_Date/Time: Calendar_Date: 20150807 Currentness_Reference: Ground Condition</t>
+          <t>Upon completion of the 2020, 2022 and 2024 EagleView regional aerial imagery acquisition projects ...</t>
         </is>
       </c>
       <c r="U22" s="1" t="inlineStr">
         <is>
-          <t>context (not held)</t>
+          <t>held imagery</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>2019_naip_rgbi.tif</t>
+          <t>(not held) City of Edmonds Basemap/2015_Aerial_Cached</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>2019n</t>
+          <t>2015 (CoE service)</t>
         </is>
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>USDA FSA NAIP WA 2019 (DOQQ m_4712213/m_4712214; the WA consortium 2019 1-ft flight carries the same date, i.e. the Hexagon flight)</t>
+          <t>City of Edmonds (source raster Ed_Aerial_2015.tif, 0.25 ftUS EPSG:2285, LZW); content INFERRED = 2015 Western Washington Regional Orthophotography (King County lead, 88 participants; prime GeoTerra, Edmonds frames flown by Valley Air and GeoTerra)</t>
         </is>
       </c>
       <c r="D23" s="1" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>LOD 21 cache (0.0746 WM m)</t>
         </is>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>metre</t>
+          <t>metre (Web Mercator)</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>EPSG:26910</t>
+          <t>EPSG:3857 (cache); source EPSG:2285</t>
         </is>
       </c>
       <c r="G23" s="1" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>5.01 (cache) / 7.62 (source)</t>
         </is>
       </c>
       <c r="H23" s="1" t="inlineStr">
         <is>
-          <t>95.1</t>
+          <t>not measured</t>
         </is>
       </c>
       <c r="I23" s="1" t="inlineStr">
         <is>
-          <t>60 (collected and delivered at 60 cm)</t>
+          <t>&lt;= 6.86 flown (MAX_GSD 0.225 ft 'as planned' for all 346 Edmonds frames; two cameras at two altitudes both back-compute to ~6.6-6.9 cm), delivered at the 0.25 ft = 7.62 cm tier (service pixelSizeX 0.07620015240030481 m = 0.250000 ftUS)</t>
         </is>
       </c>
       <c r="J23" s="1" t="inlineStr">
         <is>
-          <t>2019-10-11</t>
+          <t>2015-04-08 (n=135 photo centres in the city polygon; Valley Air, UltraCam X, 14:13-15:04 PDT) and 2015-04-17 (n=32; GeoTerra, UltraCam Xp, 12:54-13:55 PDT). CONTEST largely resolved: the King Pictometry leg is EXCLUDED by pixel comparison, the 'Aug 7 2015' leg is a DIFFERENT dataset (NAIP/HXIP 2015-08-07), leaving the consortium dates; attribution of Ed_Aerial_2015.tif to the consortium remains INFERRED and the UFMP's '4.8 in' figure is unexplained</t>
         </is>
       </c>
       <c r="K23" s="1" t="inlineStr">
         <is>
-          <t>single day</t>
+          <t>2 flight days (window of 10 days) for the consortium product</t>
         </is>
       </c>
       <c r="L23" s="1" t="inlineStr">
         <is>
-          <t>single (all Edmonds DOQQs carry 20191011; consortium flight-area IDATE '2019 -10-11' at the city centroid)</t>
-        </is>
-      </c>
-      <c r="M23" s="4" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+          <t>MULTI - two days, two vendors, two cameras within the city (flightlines 16002-16011 Zone 16 / 13007-13015 Zone 13)</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>INFERRED</t>
         </is>
       </c>
       <c r="N23" s="1" t="inlineStr">
         <is>
-          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2019/wa_fgdc_2019/47122/m_4712214_sw_10_060_20191011.txt</t>
+          <t>https://services.arcgis.com/Ej0PsM5Aw677QF1W/arcgis/rest/services/ORTHO_IMAGE15C_POINT_2574/FeatureServer/0/query</t>
         </is>
       </c>
       <c r="O23" s="1" t="inlineStr">
         <is>
-          <t>Time_Period_of_Content: Time_Period_Information: Single_Date/Time: Calendar_Date: 20191011 Currentness_Reference: Ground Condition</t>
+          <t>"FILENAME":"13009_57445" ... "UTC_TIME":"19:54:49","MAX_GSD__f":0.225 ... "VENDOR":"GeoTerra","CAMERA":"UltraCam Xp" ... "FLIGHTLINE":"13009","ACQ_DATE":1429228800000 (= 2015-04-17 UTC; first of the photo centres inside the city polygon; raw response qc/imagery_date_evidence/raw_records/kc_2015C_ORTHO_IMAGE15C_POINT_2574_citypoly_first3.json). Layer description: It is a reference for the raw image scans, it is not a index for tiled ortho imagery</t>
         </is>
       </c>
       <c r="P23" s="1" t="inlineStr">
         <is>
-          <t>OCTOBER. No NAIP metadata record (2015/2017/2021 Digital Coast) contains any leaf-on/leaf-off statement - only 'peak crop growing conditions'; the 'NAIP is leaf-on by spec' assumption has no documentary basis.</t>
+          <t>Photo-centre DAYS are MEASURED; binding them to Ed_Aerial_2015.tif is INFERRED via (a) 0.25 ftUS cell size matching the consortium tier, (b) CRS NAD83 SP WA North ftUS, (c) Edmonds named in GeoTerra's participant table and the consortium agreement signed 2015-06-23 ($3,696.21), (d) leaf-off/high-sun spec matching the tiles. NOTE: no Apr 9 frames exist over Edmonds (the catalogue's 'Apr 8/9/17' was wrong); one Mar 26 frame sits just outside the polygon. King leg excluded: CoE 2015 vs KingCo_Aerial_2015 LOD-20 tiles r=0.036-0.557 at 5 sites vs r=0.988-0.994 for the CoE-2017/King-2017 control. 'Aug 7 2015 / 4.8 in' (UFMP 2019 p.26) traces to the Davey Resource Group 2018 UTC Assessment which names 'USDA, Farm Service Agency' = NAIP 2015 (2015-08-07, 1 m = the same Hexagon flight as the HXIP 1-ft consortium product); '4.8 in' matches no known 2015 product. Phenology caveat from the project's own survey report: 'the need to begin immediate image acquisition due an earlier than normal bud break' - Apr 8/17 is late in a leaf-off window. Vendor/camera cross-validated at serial-number level against the Flight Subcontractor PDF (UCX 60418665 / UCXp 10411033).</t>
         </is>
       </c>
       <c r="Q23" s="1" t="inlineStr">
         <is>
-          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED</t>
+          <t>grid MEASURED (live service); native MEASURED (index MAX_GSD) + PUBLISHED (tier)</t>
         </is>
       </c>
       <c r="R23" s="1" t="inlineStr">
         <is>
-          <t>2019-10-11</t>
+          <t>2015-08-07 15:31 (UFMP/Davey 'August 7th, 2015' imagery = NAIP/HXIP 2015, NOT the city basemap)</t>
         </is>
       </c>
       <c r="S23" s="1" t="inlineStr">
         <is>
-          <t>https://services.arcgis.com/jsIt88o09Q0r1j8h/arcgis/rest/services/2019_Statewide_imagery_consortium_1_foot_flight_areas/FeatureServer/0/query</t>
+          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2015/wa_fgdc_2015/47122/m_4712214_sw_10_1_20150807.txt</t>
         </is>
       </c>
       <c r="T23" s="1" t="inlineStr">
         <is>
-          <t>"IDATE":"2019 -10-11" (stray space verbatim; city-centroid point query, raw response qc/imagery_date_evidence/raw_records/wa_2019_1ft_citycentroid.json)</t>
+          <t>Time_Period_of_Content: Time_Period_Information: Single_Date/Time: Calendar_Date: 20150807 Currentness_Reference: Ground Condition</t>
         </is>
       </c>
       <c r="U23" s="1" t="inlineStr">
         <is>
-          <t>held imagery</t>
+          <t>context (not held)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>2023_naip_rgbi.tif</t>
+          <t>2019_naip_rgbi.tif</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>2023n (was mislabelled 2022n)</t>
+          <t>2019n</t>
         </is>
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t>USDA FSA NAIP WA 2023 (DOQQ m_4712213/m_4712214)</t>
+          <t>USDA FSA NAIP WA 2019 (DOQQ m_4712213/m_4712214; the WA consortium 2019 1-ft flight carries the same date, i.e. the Hexagon flight)</t>
         </is>
       </c>
       <c r="D24" s="1" t="inlineStr">
@@ -14573,17 +14604,17 @@
       </c>
       <c r="H24" s="1" t="inlineStr">
         <is>
-          <t>83.1</t>
+          <t>95.1</t>
         </is>
       </c>
       <c r="I24" s="1" t="inlineStr">
         <is>
-          <t>60 delivered (2021/2023-era WA NAIP collected finer and rectified to 60 cm)</t>
+          <t>60 (collected and delivered at 60 cm)</t>
         </is>
       </c>
       <c r="J24" s="1" t="inlineStr">
         <is>
-          <t>2023-10-07</t>
+          <t>2019-10-11</t>
         </is>
       </c>
       <c r="K24" s="1" t="inlineStr">
@@ -14593,7 +14624,7 @@
       </c>
       <c r="L24" s="1" t="inlineStr">
         <is>
-          <t>single (all 8 Edmonds QQs: m_47122{13,14}_*_10_060_20231007_20240209)</t>
+          <t>single (all Edmonds DOQQs carry 20191011; consortium flight-area IDATE '2019 -10-11' at the city centroid)</t>
         </is>
       </c>
       <c r="M24" s="4" t="inlineStr">
@@ -14603,17 +14634,17 @@
       </c>
       <c r="N24" s="1" t="inlineStr">
         <is>
-          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2023/wa_fgdc_2023/47122/m_4712214_sw_10_060_20231007_20240209.xml</t>
+          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2019/wa_fgdc_2019/47122/m_4712214_sw_10_060_20191011.txt</t>
         </is>
       </c>
       <c r="O24" s="1" t="inlineStr">
         <is>
-          <t>&lt;gco:CharacterString&gt;m_4712214_sw_10_060_20231007.tif&lt;/gco:CharacterString&gt; (the DOQQ file name in the ISO metadata record; 20231007 = acquisition date field)</t>
+          <t>Time_Period_of_Content: Time_Period_Information: Single_Date/Time: Calendar_Date: 20191011 Currentness_Reference: Ground Condition</t>
         </is>
       </c>
       <c r="P24" s="1" t="inlineStr">
         <is>
-          <t>OCTOBER. Held bands 1-3 byte-identical to rgb_2023, band 4 to ir_2023 (DataLake_Issues). Context: NAIP 2021 over Edmonds exists (all 8 QQs STAC datetime 2021-07-13, INFERRED from file names - the FGDC sidecars for quad 47122 are absent from the Azure mirror).</t>
+          <t>OCTOBER. No NAIP metadata record (2015/2017/2021 Digital Coast) contains any leaf-on/leaf-off statement - only 'peak crop growing conditions'; the 'NAIP is leaf-on by spec' assumption has no documentary basis.</t>
         </is>
       </c>
       <c r="Q24" s="1" t="inlineStr">
@@ -14621,9 +14652,21 @@
           <t>grid/true MEASURED; effective MEASURED; native PUBLISHED</t>
         </is>
       </c>
-      <c r="R24" s="1" t="inlineStr"/>
-      <c r="S24" s="1" t="inlineStr"/>
-      <c r="T24" s="1" t="inlineStr"/>
+      <c r="R24" s="1" t="inlineStr">
+        <is>
+          <t>2019-10-11</t>
+        </is>
+      </c>
+      <c r="S24" s="1" t="inlineStr">
+        <is>
+          <t>https://services.arcgis.com/jsIt88o09Q0r1j8h/arcgis/rest/services/2019_Statewide_imagery_consortium_1_foot_flight_areas/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="T24" s="1" t="inlineStr">
+        <is>
+          <t>"IDATE":"2019 -10-11" (stray space verbatim; city-centroid point query, raw response qc/imagery_date_evidence/raw_records/wa_2019_1ft_citycentroid.json)</t>
+        </is>
+      </c>
       <c r="U24" s="1" t="inlineStr">
         <is>
           <t>held imagery</t>
@@ -14633,62 +14676,62 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>lidar_snoh_chm.tif</t>
+          <t>2023_naip_rgbi.tif</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>2016 (lidar)</t>
+          <t>2023n (was mislabelled 2022n)</t>
         </is>
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
-          <t>USGS 3DEP HAG via Planetary Computer, reprojected by the project; underlying lidar = USGS_LPC_WA_Western_North_2016 (QSI for USGS/WADNR)</t>
+          <t>USDA FSA NAIP WA 2023 (DOQQ m_4712213/m_4712214)</t>
         </is>
       </c>
       <c r="D25" s="1" t="inlineStr">
         <is>
-          <t>1.000009</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>metre (Web Mercator, inflated 1/cos(lat))</t>
+          <t>metre</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>EPSG:3857</t>
+          <t>EPSG:26910</t>
         </is>
       </c>
       <c r="G25" s="1" t="inlineStr">
         <is>
-          <t>67.16</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="H25" s="1" t="inlineStr">
         <is>
-          <t>n/a (bilinear-upsampled ~2 m product)</t>
+          <t>83.1</t>
         </is>
       </c>
       <c r="I25" s="1" t="inlineStr">
         <is>
-          <t>~200 (HAG raster); lidar 0.7 m spacing</t>
+          <t>60 delivered (2021/2023-era WA NAIP collected finer and rectified to 60 cm)</t>
         </is>
       </c>
       <c r="J25" s="1" t="inlineStr">
         <is>
-          <t>2016-03-17 to 2016-09-30 (Western Washington 3DEP NORTH AOI; all 46 tiles over the city are North-block)</t>
+          <t>2023-10-07</t>
         </is>
       </c>
       <c r="K25" s="1" t="inlineStr">
         <is>
-          <t>window of 198 days</t>
+          <t>single day</t>
         </is>
       </c>
       <c r="L25" s="1" t="inlineStr">
         <is>
-          <t>multi</t>
+          <t>single (all 8 Edmonds QQs: m_47122{13,14}_*_10_060_20231007_20240209)</t>
         </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
@@ -14698,104 +14741,92 @@
       </c>
       <c r="N25" s="1" t="inlineStr">
         <is>
-          <t>https://www.fisheries.noaa.gov/inport/item/51853</t>
+          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2023/wa_fgdc_2023/47122/m_4712214_sw_10_060_20231007_20240209.xml</t>
         </is>
       </c>
       <c r="O25" s="1" t="inlineStr">
         <is>
-          <t>North: March 17 - Sept 30, 2016 ... South: March 17, 2016 - June 6, 2017</t>
+          <t>&lt;gco:CharacterString&gt;m_4712214_sw_10_060_20231007.tif&lt;/gco:CharacterString&gt; (the DOQQ file name in the ISO metadata record; 20231007 = acquisition date field)</t>
         </is>
       </c>
       <c r="P25" s="1" t="inlineStr">
         <is>
-          <t>UNITS TRAP #4: grid is 1.0 m in EPSG:3857 = 67.2 cm true ground at 47.81N, not 1 m. Narrowed from 15 months (whole project) to the North window by point-in-polygon on NOAA's tile index (46/46 tiles /north/). Reference raster, excluded from the imagery count.</t>
+          <t>OCTOBER. Held bands 1-3 byte-identical to rgb_2023, band 4 to ir_2023 (DataLake_Issues). Context: NAIP 2021 over Edmonds exists (all 8 QQs STAC datetime 2021-07-13, INFERRED from file names - the FGDC sidecars for quad 47122 are absent from the Azure mirror).</t>
         </is>
       </c>
       <c r="Q25" s="1" t="inlineStr">
         <is>
-          <t>grid/true MEASURED; native PUBLISHED</t>
-        </is>
-      </c>
-      <c r="R25" s="1" t="inlineStr">
-        <is>
-          <t>2016-03-30 (INFERRED from the tile filename prefix 20160330_USGS_LPC_WA_Western_North_2016_q47122G4405 - a FILE NAME; 3/30/16 is a flight day for all three contractors in QSI report Table 3)</t>
-        </is>
-      </c>
-      <c r="S25" s="1" t="inlineStr">
-        <is>
-          <t>https://noaa-nos-coastal-lidar-pds.s3.amazonaws.com/laz/geoid18/6331/tileindex_wa2016_west_wa_m6331.gpkg</t>
-        </is>
-      </c>
-      <c r="T25" s="1" t="inlineStr">
-        <is>
-          <t>20160330_USGS_LPC_WA_Western_North_2016_q47122G4405_LAS_2018.copc.laz</t>
-        </is>
-      </c>
+          <t>grid/true MEASURED; effective MEASURED; native PUBLISHED</t>
+        </is>
+      </c>
+      <c r="R25" s="1" t="inlineStr"/>
+      <c r="S25" s="1" t="inlineStr"/>
+      <c r="T25" s="1" t="inlineStr"/>
       <c r="U25" s="1" t="inlineStr">
         <is>
-          <t>reference raster</t>
+          <t>held imagery</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>PSLC_2005/ (47 laz tiles)</t>
+          <t>lidar_snoh_chm.tif</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>2005 (lidar)</t>
+          <t>2016 (lidar)</t>
         </is>
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t>Puget Sound LiDAR Consortium 2005 North Puget Sound Lowlands (Terrapoint), InPort 50149</t>
+          <t>USGS 3DEP HAG via Planetary Computer, reprojected by the project; underlying lidar = USGS_LPC_WA_Western_North_2016 (QSI for USGS/WADNR)</t>
         </is>
       </c>
       <c r="D26" s="1" t="inlineStr">
         <is>
-          <t>point cloud (no grid)</t>
+          <t>1.000009</t>
         </is>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>metre (Web Mercator, inflated 1/cos(lat))</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>NAD83(HARN) UTM 10N, NAVD88 GEOID18</t>
+          <t>EPSG:3857</t>
         </is>
       </c>
       <c r="G26" s="1" t="inlineStr">
         <is>
-          <t>n/a (point cloud)</t>
+          <t>67.16</t>
         </is>
       </c>
       <c r="H26" s="1" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>n/a (bilinear-upsampled ~2 m product)</t>
         </is>
       </c>
       <c r="I26" s="1" t="inlineStr">
         <is>
-          <t>n/a (2 m nominal spacing)</t>
+          <t>~200 (HAG raster); lidar 0.7 m spacing</t>
         </is>
       </c>
       <c r="J26" s="1" t="inlineStr">
         <is>
-          <t>2005-02-27 (Edmonds sub-project, 11 sq mi)</t>
+          <t>2016-03-17 to 2016-09-30 (Western Washington 3DEP NORTH AOI; all 46 tiles over the city are North-block)</t>
         </is>
       </c>
       <c r="K26" s="1" t="inlineStr">
         <is>
-          <t>single day</t>
+          <t>window of 198 days</t>
         </is>
       </c>
       <c r="L26" s="1" t="inlineStr">
         <is>
-          <t>single (sub-project row)</t>
+          <t>multi</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
@@ -14805,92 +14836,104 @@
       </c>
       <c r="N26" s="1" t="inlineStr">
         <is>
-          <t>https://www.fisheries.noaa.gov/inport/item/50149</t>
+          <t>https://www.fisheries.noaa.gov/inport/item/51853</t>
         </is>
       </c>
       <c r="O26" s="1" t="inlineStr">
         <is>
-          <t>project, area (sq mi), date(s) collected, vert. acc (cm), horiz acc. (cm), RMSE (m) - ... - Edmonds, 11, 2/27/2005, 25, 60, 0.100 - Mt. Lake Terrace, 4, 7/15/2005-9/15/2005, 25, 60, 0.100 - Mukilteo, 16, 2/27/2005, 25, 60, 0.100</t>
+          <t>North: March 17 - Sept 30, 2016 ... South: March 17, 2016 - June 6, 2017</t>
         </is>
       </c>
       <c r="P26" s="1" t="inlineStr">
         <is>
-          <t>Density 0.25 pts/m2 stated (~0.17 cross-checked, IMAGERY_FACTS 8.1). LEAF-OFF (late February). Record-internal inconsistency: Mt. Lake Terrace sub-project dates run past the record's own Time Frame end (2005-07-15). Held at D:/edmonds-pipeline/Imagery/PSLC_2005 and Full_Image/PSLC_2005 (IMAGERY_FACTS 8.2).</t>
+          <t>UNITS TRAP #4: grid is 1.0 m in EPSG:3857 = 67.2 cm true ground at 47.81N, not 1 m. Narrowed from 15 months (whole project) to the North window by point-in-polygon on NOAA's tile index (46/46 tiles /north/). Reference raster, excluded from the imagery count.</t>
         </is>
       </c>
       <c r="Q26" s="1" t="inlineStr">
         <is>
-          <t>density PUBLISHED</t>
-        </is>
-      </c>
-      <c r="R26" s="1" t="inlineStr"/>
-      <c r="S26" s="1" t="inlineStr"/>
-      <c r="T26" s="1" t="inlineStr"/>
+          <t>grid/true MEASURED; native PUBLISHED</t>
+        </is>
+      </c>
+      <c r="R26" s="1" t="inlineStr">
+        <is>
+          <t>2016-03-30 (INFERRED from the tile filename prefix 20160330_USGS_LPC_WA_Western_North_2016_q47122G4405 - a FILE NAME; 3/30/16 is a flight day for all three contractors in QSI report Table 3)</t>
+        </is>
+      </c>
+      <c r="S26" s="1" t="inlineStr">
+        <is>
+          <t>https://noaa-nos-coastal-lidar-pds.s3.amazonaws.com/laz/geoid18/6331/tileindex_wa2016_west_wa_m6331.gpkg</t>
+        </is>
+      </c>
+      <c r="T26" s="1" t="inlineStr">
+        <is>
+          <t>20160330_USGS_LPC_WA_Western_North_2016_q47122G4405_LAS_2018.copc.laz</t>
+        </is>
+      </c>
       <c r="U26" s="1" t="inlineStr">
         <is>
-          <t>reference lidar</t>
+          <t>reference raster</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>ccap_2016_hires_lc_snohfull.tif</t>
+          <t>PSLC_2005/ (47 laz tiles)</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>2016 (C-CAP ref)</t>
+          <t>2005 (lidar)</t>
         </is>
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t>NOAA OCM C-CAP hi-res land cover, Snohomish County 2016 (InPort 53263 - record RECOVERED as an InPort XML export on coast.noaa.gov; fisheries.noaa.gov still 403)</t>
+          <t>Puget Sound LiDAR Consortium 2005 North Puget Sound Lowlands (Terrapoint), InPort 50149</t>
         </is>
       </c>
       <c r="D27" s="1" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>point cloud (no grid)</t>
         </is>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>metre</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>EPSG:26910</t>
+          <t>NAD83(HARN) UTM 10N, NAVD88 GEOID18</t>
         </is>
       </c>
       <c r="G27" s="1" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>n/a (point cloud)</t>
         </is>
       </c>
       <c r="H27" s="1" t="inlineStr">
         <is>
-          <t>n/a (thematic)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I27" s="1" t="inlineStr">
         <is>
-          <t>100 (1 m product)</t>
+          <t>n/a (2 m nominal spacing)</t>
         </is>
       </c>
       <c r="J27" s="1" t="inlineStr">
         <is>
-          <t>summer 2016 (source imagery, stated as NAIP) - CONTESTED: no WA NAIP 2016 exists (Azure NAIP v002/wa/ holds 2011, 2013, 2015, 2017, 2019, 2021, 2023 only)</t>
+          <t>2005-02-27 (Edmonds sub-project, 11 sq mi)</t>
         </is>
       </c>
       <c r="K27" s="1" t="inlineStr">
         <is>
-          <t>season</t>
+          <t>single day</t>
         </is>
       </c>
       <c r="L27" s="1" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>single (sub-project row)</t>
         </is>
       </c>
       <c r="M27" s="4" t="inlineStr">
@@ -14900,22 +14943,22 @@
       </c>
       <c r="N27" s="1" t="inlineStr">
         <is>
-          <t>https://chs.coast.noaa.gov/htdata/raster1/landcover/bulkdownload/hires/wa/WA_Snohomish_2016_lc.xml</t>
+          <t>https://www.fisheries.noaa.gov/inport/item/50149</t>
         </is>
       </c>
       <c r="O27" s="1" t="inlineStr">
         <is>
-          <t>The timeframe for this metadata is summer 2016. These maps are developed utilizing high resolution National Agriculture Imagery Program (NAIP) imagery, and can be used to track changes in the landscape through time.</t>
+          <t>project, area (sq mi), date(s) collected, vert. acc (cm), horiz acc. (cm), RMSE (m) - ... - Edmonds, 11, 2/27/2005, 25, 60, 0.100 - Mt. Lake Terrace, 4, 7/15/2005-9/15/2005, 25, 60, 0.100 - Mukilteo, 16, 2/27/2005, 25, 60, 0.100</t>
         </is>
       </c>
       <c r="P27" s="1" t="inlineStr">
         <is>
-          <t>Candidate reconciliation (INFERENCE): the 'summer 2016' imagery is the HXIP Aug 11-12 2016 flight (the WA consortium product is itself branded 'NAIP_2016' on AGOL), or NOAA used NAIP 2015 (2015-08-07) and labelled the product 2016 - UNRESOLVED. Traps in the record: &lt;start-date-time&gt;2016-01-01 is a year placeholder; &lt;publish-date&gt;2019-03-14 is publication. Ancillary: NGS MLLW orthoimagery 2014 for shore classes. Reference raster.</t>
+          <t>Density 0.25 pts/m2 stated (~0.17 cross-checked, IMAGERY_FACTS 8.1). LEAF-OFF (late February). Record-internal inconsistency: Mt. Lake Terrace sub-project dates run past the record's own Time Frame end (2005-07-15). Held at D:/edmonds-pipeline/Imagery/PSLC_2005 and Full_Image/PSLC_2005 (IMAGERY_FACTS 8.2).</t>
         </is>
       </c>
       <c r="Q27" s="1" t="inlineStr">
         <is>
-          <t>grid/true MEASURED; native PUBLISHED</t>
+          <t>density PUBLISHED</t>
         </is>
       </c>
       <c r="R27" s="1" t="inlineStr"/>
@@ -14923,24 +14966,24 @@
       <c r="T27" s="1" t="inlineStr"/>
       <c r="U27" s="1" t="inlineStr">
         <is>
-          <t>reference raster</t>
+          <t>reference lidar</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>ccap_2021_hires_lc.tif</t>
+          <t>ccap_2016_hires_lc_snohfull.tif</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>2021 (C-CAP v2 ref)</t>
+          <t>2016 (C-CAP ref)</t>
         </is>
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>NOAA OCM C-CAP hi-res v2 'Refined' Puget Sound 2021 (InPort 79723; Ecopia extraction, NV5 refinement)</t>
+          <t>NOAA OCM C-CAP hi-res land cover, Snohomish County 2016 (InPort 53263 - record RECOVERED as an InPort XML export on coast.noaa.gov; fisheries.noaa.gov still 403)</t>
         </is>
       </c>
       <c r="D28" s="1" t="inlineStr">
@@ -14970,22 +15013,22 @@
       </c>
       <c r="I28" s="1" t="inlineStr">
         <is>
-          <t>100 (1 m extraction from '30cm or better' imagery)</t>
+          <t>100 (1 m product)</t>
         </is>
       </c>
       <c r="J28" s="1" t="inlineStr">
         <is>
-          <t>2021 (year only; 'Acquisition date of the Aerial Imagery')</t>
+          <t>summer 2016 (source imagery, stated as NAIP) - CONTESTED: no WA NAIP 2016 exists (Azure NAIP v002/wa/ holds 2011, 2013, 2015, 2017, 2019, 2021, 2023 only)</t>
         </is>
       </c>
       <c r="K28" s="1" t="inlineStr">
         <is>
-          <t>year only</t>
+          <t>season</t>
         </is>
       </c>
       <c r="L28" s="1" t="inlineStr">
         <is>
-          <t>multi (mosaic of vendor imagery)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="M28" s="4" t="inlineStr">
@@ -14995,17 +15038,17 @@
       </c>
       <c r="N28" s="1" t="inlineStr">
         <is>
-          <t>https://ocmgeodatastor1.blob.core.windows.net/ccap/bulk_download/C-CAP_High-Resolution_Data/Refined_C-CAP_High-Resolution_Land_Cover_Classification/CONUS/wa_puget_2021_ccap_v2_hires_landcover.xml</t>
+          <t>https://chs.coast.noaa.gov/htdata/raster1/landcover/bulkdownload/hires/wa/WA_Snohomish_2016_lc.xml</t>
         </is>
       </c>
       <c r="O28" s="1" t="inlineStr">
         <is>
-          <t>&lt;currentness-reference&gt;Acquisition date of the Aerial Imagery&lt;/currentness-reference&gt; ... &lt;time-frame-type&gt;Discrete&lt;/time-frame-type&gt; &lt;start-date-time&gt;2021&lt;/start-date-time&gt; ... Initial 1m spatial resolution feature extraction for Impervious, Water, and Canopy (tree and scrub/shrub) mapping was conducted by Ecopia AI</t>
+          <t>The timeframe for this metadata is summer 2016. These maps are developed utilizing high resolution National Agriculture Imagery Program (NAIP) imagery, and can be used to track changes in the landscape through time.</t>
         </is>
       </c>
       <c r="P28" s="1" t="inlineStr">
         <is>
-          <t>The record was created 2026-04-28 and may post-date the held clip (2026-07-06); best-available lineage, not proven identical. Record defects: Ohio/Houston copy-paste text, 'Never Published', 'best-available-metadata: No'. LICENSING (verbatim, for the Licensing_Risk sheet): 'Users are granted a perpetual, non-exclusive, irrevocable, worldwide license to use these data ... with the exception of creating, training, improving, modifying, validating, testing, evaluating, or otherwise leveraging machine learning algorithms in order to explicitly create similar land cover data for a period of five years from its date of creation.' The Phase-1 canopy record (InPort 70562, created 2023-09-30) carries the broader unqualified form ('may not be used for the purpose of ... testing, or evaluating machine learning algorithms ... except with the express written consent of Ecopia Tech Corporation'). This project uses the product as an EVALUATION reference - flag for Kam.</t>
+          <t>Candidate reconciliation (INFERENCE): the 'summer 2016' imagery is the HXIP Aug 11-12 2016 flight (the WA consortium product is itself branded 'NAIP_2016' on AGOL), or NOAA used NAIP 2015 (2015-08-07) and labelled the product 2016 - UNRESOLVED. Traps in the record: &lt;start-date-time&gt;2016-01-01 is a year placeholder; &lt;publish-date&gt;2019-03-14 is publication. Ancillary: NGS MLLW orthoimagery 2014 for shore classes. Reference raster.</t>
         </is>
       </c>
       <c r="Q28" s="1" t="inlineStr">
@@ -15025,62 +15068,62 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>(not held) WA Statewide Imagery Consortium 2020 6-inch (Hexagon, Leica ADS100)</t>
+          <t>ccap_2021_hires_lc.tif</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>2020 (SECOND 2020 acquisition - NOT the anchor)</t>
+          <t>2021 (C-CAP v2 ref)</t>
         </is>
       </c>
       <c r="C29" s="1" t="inlineStr">
         <is>
-          <t>WA OCIO/WaTech Statewide Imagery Consortium, flown by Hexagon under the 2020 NAIP Imaging Program</t>
+          <t>NOAA OCM C-CAP hi-res v2 'Refined' Puget Sound 2021 (InPort 79723; Ecopia extraction, NV5 refinement)</t>
         </is>
       </c>
       <c r="D29" s="1" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>metre</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EPSG:26910</t>
         </is>
       </c>
       <c r="G29" s="1" t="inlineStr">
         <is>
-          <t>15 (6 in product), nominal flight GSD 20</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="H29" s="1" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>n/a (thematic)</t>
         </is>
       </c>
       <c r="I29" s="1" t="inlineStr">
         <is>
-          <t>20 (nominal)</t>
+          <t>100 (1 m extraction from '30cm or better' imagery)</t>
         </is>
       </c>
       <c r="J29" s="1" t="inlineStr">
         <is>
-          <t>2020-08-28 (flight-area polygon at the city centroid; 2020-08-27 also intersects the city bbox); program window 2020-08-03 to 2020-09-06</t>
+          <t>2021 (year only; 'Acquisition date of the Aerial Imagery')</t>
         </is>
       </c>
       <c r="K29" s="1" t="inlineStr">
         <is>
-          <t>day (coarse flight-area block, 911-1263 sq mi)</t>
+          <t>year only</t>
         </is>
       </c>
       <c r="L29" s="1" t="inlineStr">
         <is>
-          <t>multi (2 blocks over the city)</t>
+          <t>multi (mosaic of vendor imagery)</t>
         </is>
       </c>
       <c r="M29" s="4" t="inlineStr">
@@ -15090,154 +15133,249 @@
       </c>
       <c r="N29" s="1" t="inlineStr">
         <is>
-          <t>https://www.arcgis.com/sharing/rest/content/items/dd83978971d8421eb6b1a7273ba51f6e?f=json</t>
+          <t>https://ocmgeodatastor1.blob.core.windows.net/ccap/bulk_download/C-CAP_High-Resolution_Data/Refined_C-CAP_High-Resolution_Land_Cover_Classification/CONUS/wa_puget_2021_ccap_v2_hires_landcover.xml</t>
         </is>
       </c>
       <c r="O29" s="1" t="inlineStr">
         <is>
-          <t>Digital aerial imagery for Washington state was collected by Hexagon as part of the 2020 NAIP Imaging Program. Imagery was collected between August 3, 2020 and September 6, 2020 using Leica ADS100 digital camera systems. The project was flown at heights ranging from 8,000 ft msl to 15,500 ft msl resulting in a nominal GSD of 20cm.</t>
+          <t>&lt;currentness-reference&gt;Acquisition date of the Aerial Imagery&lt;/currentness-reference&gt; ... &lt;time-frame-type&gt;Discrete&lt;/time-frame-type&gt; &lt;start-date-time&gt;2021&lt;/start-date-time&gt; ... Initial 1m spatial resolution feature extraction for Impervious, Water, and Canopy (tree and scrub/shrub) mapping was conducted by Ecopia AI</t>
         </is>
       </c>
       <c r="P29" s="1" t="inlineStr">
         <is>
-          <t>HAZARD ROW: a different vendor, camera, resolution and season from 2020_coe_rgb.tif (EagleView 3 in, Apr-Jul). Year-matched substitution would introduce a ~4.5-month error - exactly the 2015 three-way pattern. Not held; a late-August leaf-on 15 cm 4-band product if ever wanted.</t>
+          <t>The record was created 2026-04-28 and may post-date the held clip (2026-07-06); best-available lineage, not proven identical. Record defects: Ohio/Houston copy-paste text, 'Never Published', 'best-available-metadata: No'. LICENSING (verbatim, for the Licensing_Risk sheet): 'Users are granted a perpetual, non-exclusive, irrevocable, worldwide license to use these data ... with the exception of creating, training, improving, modifying, validating, testing, evaluating, or otherwise leveraging machine learning algorithms in order to explicitly create similar land cover data for a period of five years from its date of creation.' The Phase-1 canopy record (InPort 70562, created 2023-09-30) carries the broader unqualified form ('may not be used for the purpose of ... testing, or evaluating machine learning algorithms ... except with the express written consent of Ecopia Tech Corporation'). This project uses the product as an EVALUATION reference - flag for Kam.</t>
         </is>
       </c>
       <c r="Q29" s="1" t="inlineStr">
         <is>
-          <t>PUBLISHED</t>
-        </is>
-      </c>
-      <c r="R29" s="1" t="inlineStr">
-        <is>
-          <t>2020-08-28 / 2020-08-27</t>
-        </is>
-      </c>
-      <c r="S29" s="1" t="inlineStr">
-        <is>
-          <t>https://services.arcgis.com/jsIt88o09Q0r1j8h/ArcGIS/rest/services/2020_Statewide_imagery_consortium_6_inch_flight_areas/FeatureServer/0/query</t>
-        </is>
-      </c>
-      <c r="T29" s="1" t="inlineStr">
-        <is>
-          <t>"IDATE":"2020-08-28" (city centroid) ... "IDATE":"2020-08-27" (also intersects the city bbox; raw responses qc/imagery_date_evidence/raw_records/wa_2020_6in_*.json)</t>
-        </is>
-      </c>
+          <t>grid/true MEASURED; native PUBLISHED</t>
+        </is>
+      </c>
+      <c r="R29" s="1" t="inlineStr"/>
+      <c r="S29" s="1" t="inlineStr"/>
+      <c r="T29" s="1" t="inlineStr"/>
       <c r="U29" s="1" t="inlineStr">
         <is>
-          <t>context (not held)</t>
+          <t>reference raster</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
+          <t>(not held) WA Statewide Imagery Consortium 2020 6-inch (Hexagon, Leica ADS100)</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>2020 (SECOND 2020 acquisition - NOT the anchor)</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>WA OCIO/WaTech Statewide Imagery Consortium, flown by Hexagon under the 2020 NAIP Imaging Program</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="inlineStr">
+        <is>
+          <t>15 (6 in product), nominal flight GSD 20</t>
+        </is>
+      </c>
+      <c r="H30" s="1" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I30" s="1" t="inlineStr">
+        <is>
+          <t>20 (nominal)</t>
+        </is>
+      </c>
+      <c r="J30" s="1" t="inlineStr">
+        <is>
+          <t>2020-08-28 (flight-area polygon at the city centroid; 2020-08-27 also intersects the city bbox); program window 2020-08-03 to 2020-09-06</t>
+        </is>
+      </c>
+      <c r="K30" s="1" t="inlineStr">
+        <is>
+          <t>day (coarse flight-area block, 911-1263 sq mi)</t>
+        </is>
+      </c>
+      <c r="L30" s="1" t="inlineStr">
+        <is>
+          <t>multi (2 blocks over the city)</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="N30" s="1" t="inlineStr">
+        <is>
+          <t>https://www.arcgis.com/sharing/rest/content/items/dd83978971d8421eb6b1a7273ba51f6e?f=json</t>
+        </is>
+      </c>
+      <c r="O30" s="1" t="inlineStr">
+        <is>
+          <t>Digital aerial imagery for Washington state was collected by Hexagon as part of the 2020 NAIP Imaging Program. Imagery was collected between August 3, 2020 and September 6, 2020 using Leica ADS100 digital camera systems. The project was flown at heights ranging from 8,000 ft msl to 15,500 ft msl resulting in a nominal GSD of 20cm.</t>
+        </is>
+      </c>
+      <c r="P30" s="1" t="inlineStr">
+        <is>
+          <t>HAZARD ROW: a different vendor, camera, resolution and season from 2020_coe_rgb.tif (EagleView 3 in, Apr-Jul). Year-matched substitution would introduce a ~4.5-month error - exactly the 2015 three-way pattern. Not held; a late-August leaf-on 15 cm 4-band product if ever wanted.</t>
+        </is>
+      </c>
+      <c r="Q30" s="1" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="R30" s="1" t="inlineStr">
+        <is>
+          <t>2020-08-28 / 2020-08-27</t>
+        </is>
+      </c>
+      <c r="S30" s="1" t="inlineStr">
+        <is>
+          <t>https://services.arcgis.com/jsIt88o09Q0r1j8h/ArcGIS/rest/services/2020_Statewide_imagery_consortium_6_inch_flight_areas/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="T30" s="1" t="inlineStr">
+        <is>
+          <t>"IDATE":"2020-08-28" (city centroid) ... "IDATE":"2020-08-27" (also intersects the city bbox; raw responses qc/imagery_date_evidence/raw_records/wa_2020_6in_*.json)</t>
+        </is>
+      </c>
+      <c r="U30" s="1" t="inlineStr">
+        <is>
+          <t>context (not held)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
           <t>(not held) WA Statewide Imagery Consortium 2018 6-inch; Edmonds_Marsh_2018 drone</t>
         </is>
       </c>
-      <c r="B30" s="1" t="inlineStr">
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>2018 (two distinct acquisitions)</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
         <is>
           <t>WA consortium (Hexagon) / City of Edmonds Imagery/Edmonds_Marsh_2018 ImageServer</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D31" s="1" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E31" s="1" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G30" s="1" t="inlineStr">
+      <c r="G31" s="1" t="inlineStr">
         <is>
           <t>15 (consortium) / 2.5 (Marsh cache LOD)</t>
         </is>
       </c>
-      <c r="H30" s="1" t="inlineStr">
+      <c r="H31" s="1" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I30" s="1" t="inlineStr">
+      <c r="I31" s="1" t="inlineStr">
         <is>
           <t>n/a / 3.36 (Marsh pixelSizeX 0.0336 m)</t>
         </is>
       </c>
-      <c r="J30" s="1" t="inlineStr">
+      <c r="J31" s="1" t="inlineStr">
         <is>
           <t>2018-08-07 (consortium flight area over Edmonds) ; 2018-08-01 16:22-16:52 UTC (Marsh drone sortie) - six days apart, NOT the same acquisition</t>
         </is>
       </c>
-      <c r="K30" s="1" t="inlineStr">
+      <c r="K31" s="1" t="inlineStr">
         <is>
           <t>day / exact timestamp</t>
         </is>
       </c>
-      <c r="L30" s="1" t="inlineStr">
+      <c r="L31" s="1" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M30" s="4" t="inlineStr">
+      <c r="M31" s="4" t="inlineStr">
         <is>
           <t>PUBLISHED</t>
         </is>
       </c>
-      <c r="N30" s="1" t="inlineStr">
+      <c r="N31" s="1" t="inlineStr">
         <is>
           <t>https://services.arcgis.com/jsIt88o09Q0r1j8h/arcgis/rest/services/2018FlightAreas/FeatureServer/0/query</t>
         </is>
       </c>
-      <c r="O30" s="1" t="inlineStr">
+      <c r="O31" s="1" t="inlineStr">
         <is>
           <t>"IDATE":"2018-08-07" (city-centroid point query; raw response qc/imagery_date_evidence/raw_records/wa_2018_6in_citycentroid.json)</t>
         </is>
       </c>
-      <c r="P30" s="1" t="inlineStr">
+      <c r="P31" s="1" t="inlineStr">
         <is>
           <t>Recorded to prevent conflation. The Marsh service is the project's only Edmonds layer with a machine-readable timestamp and the positive control for keyProperties queries (correct path: /gis/rest/services/.../ImageServer/keyProperties?f=json).</t>
         </is>
       </c>
-      <c r="Q30" s="1" t="inlineStr">
+      <c r="Q31" s="1" t="inlineStr">
         <is>
           <t>PUBLISHED</t>
         </is>
       </c>
-      <c r="R30" s="1" t="inlineStr">
+      <c r="R31" s="1" t="inlineStr">
         <is>
           <t>2018-08-01T16:22:13+00:00 to 16:52:13 (Marsh)</t>
         </is>
       </c>
-      <c r="S30" s="1" t="inlineStr">
+      <c r="S31" s="1" t="inlineStr">
         <is>
           <t>https://maps.edmondswa.gov/gis/rest/services/Basemap/Edmonds_Marsh_2018/ImageServer/keyProperties?f=json</t>
         </is>
       </c>
-      <c r="T30" s="1" t="inlineStr">
+      <c r="T31" s="1" t="inlineStr">
         <is>
           <t>"acquisitionEndDate":"2018-08-01T16:52:13+00:00","acquisitionStartDate":"2018-08-01T16:22:13+00:00"</t>
         </is>
       </c>
-      <c r="U30" s="1" t="inlineStr">
+      <c r="U31" s="1" t="inlineStr">
         <is>
           <t>context (not held)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U30"/>
+  <autoFilter ref="A1:U31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16564,7 +16702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P221"/>
+  <dimension ref="A1:P222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -27149,7 +27287,7 @@
       </c>
       <c r="N129" s="1" t="inlineStr">
         <is>
-          <t>YES - re-acquire full extent from Snohomish ImageServer (Tier A #1)</t>
+          <t>REPLACE 2026-08-23 -&gt; 2016_snoh_1ft_rgbi.tif (coverage 82.33 &gt; 38.0). YES - re-acquire full extent from Snohomish ImageServer (Tier A #1)</t>
         </is>
       </c>
       <c r="O129" s="1" t="inlineStr">
@@ -27231,7 +27369,7 @@
       </c>
       <c r="N130" s="1" t="inlineStr">
         <is>
-          <t>YES - re-acquire full extent from Snohomish ImageServer (Tier A #1)</t>
+          <t>REPLACE 2026-08-23 -&gt; 2016_snoh_1ft_rgbi.tif (coverage 82.33 &gt; 38.0). YES - re-acquire full extent from Snohomish ImageServer (Tier A #1)</t>
         </is>
       </c>
       <c r="O130" s="1" t="inlineStr">
@@ -27313,7 +27451,7 @@
       </c>
       <c r="N131" s="1" t="inlineStr">
         <is>
-          <t>YES - re-acquire full extent from Snohomish ImageServer (Tier A #1)</t>
+          <t>REPLACE 2026-08-23 -&gt; 2016_snoh_1ft_rgbi.tif (coverage 82.33 &gt; 38.0). YES - re-acquire full extent from Snohomish ImageServer (Tier A #1)</t>
         </is>
       </c>
       <c r="O131" s="1" t="inlineStr">
@@ -34704,6 +34842,83 @@
       <c r="P221" s="1" t="inlineStr">
         <is>
           <t>THIS IS THE ANSWER TO (b). The Ecopia item names the source imagery verbatim: "Imagery Used for Extraction:" / "Pixel resolution: 15 cm (6\")" / "Camera sensor: Hexagon Pushbroom (Content Mapper)" / "Date of capture: 06/25/2021 - 08/14/2022". So the source is a HEXAGON commercial capture, not a state flight. NOT PUBLICLY DOWNLOADABLE - MEASURED: GET https://services.hxgncontent.com/streaming/wms?service=WMS&amp;request=GetCapabilities&amp;version=1.3.0 returns HTTP 401 Unauthorized (720-byte Tomcat error page) with no token. Corroborating evidence chain that this is the HxGN Content Program (inference, not a verbatim quote): the service host is services.hxgncontent.com, the item description is titled "Hexagon Content Program", and WAGeoservices publishes a companion item "AGOL Hexagon Token Replace (Python toolbox)" (id 59061adf38174773baab16ceb44646cf) whose snippet is "Downloadable Python toolbox that can be used to replace the access token embedded in an AGOL or Portal Item that references the Hexagon streaming service" - i.e. token-gated. Item-level access is "public" but that governs the AGOL item record, NOT the imagery. NO statewide 2021-2022 ortho service exists anywhere on imagery-public.watech.wa.gov - MEASURED by enumerating all 8 folders / 97 services; the newest statewide imagery on that server is NAIP 2017.</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_2016 full extent, native 1 ft (HXIP 2016)</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>true GSD 30.48 cm; 4 bands; effective 40.56 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2016/ImageServer</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2016/ImageServer</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>2016_snoh_1ft_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N222" t="inlineStr">
+        <is>
+          <t>this file REPLACES 2016_snoh_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P222" t="inlineStr">
+        <is>
+          <t>decision REPLACE: wins=['coverage 82.33 &gt; 38.0'] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S16</t>
         </is>
       </c>
     </row>
@@ -35526,7 +35741,7 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>YES - re-acquire full extent from Snohomish ImageServer (Tier A #1)</t>
+          <t>RESOLVED 2026-08-23: REPLACE by 2016_snoh_1ft_rgbi.tif. YES - re-acquire full extent from Snohomish ImageServer (Tier A #1)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
batch 3 landed: S21 REPLACE (2021s -> 2021_snoh_6in_rgbi, coverage 100 vs 39.5%, common-grid HF 1.43) + S15 key 2015s (3-band); CC21 gate 99.79% class agreement -> patch verdict, stays quarantined; catalog 24/24 + ADOPTED_NON_YEAR heading; table 39 rows
</commit_message>
<xml_diff>
--- a/Scripts/imagery_catalog_2026-08-22.xlsx
+++ b/Scripts/imagery_catalog_2026-08-22.xlsx
@@ -33,7 +33,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing_Risk" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MASTER'!$A$1:$P$221</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'KingCo_SDC_Catalog'!$A$1:$D$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DataLake_Issues'!$A$1:$C$15</definedName>
@@ -10920,7 +10920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11601,6 +11601,68 @@
         </is>
       </c>
       <c r="G20" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2021_snoh_6in_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>15.24</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="E21" t="n">
+        <v>20.06</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>median of 5 Method_Provenance sites; common-grid vs 2021_snoh_rgbi.tif: new 20.05 / held 21.09 cm, HF ratio 1.432</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2015_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>30.48</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="E22" t="n">
+        <v>41.39</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
         <is>
           <t>median of 5 sites</t>
         </is>
@@ -12398,7 +12460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U38"/>
+  <dimension ref="A1:U40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -14225,7 +14287,7 @@
       </c>
       <c r="P18" s="1" t="inlineStr">
         <is>
-          <t>CLOSED LEADS: no WA consortium flight-date layer exists for 2021 or later (all 68 WAGeoservices services + 225 items enumerated; series ends 2020); the mosaic-catalog schema has no date field at all; WA NAIP 2021 does not cover quad 47122 (eastern WA only), so no NAIP ride-along date. Remaining route: the Hexagon flight log via Snohomish County DoIT, or the consortium contact (Joanne Markert, WA OCIO). Weather elimination (ASOS KPAE+KSEA+KBFI, criterion calibrated to 46/46 known Edmonds flight days; 2021-06-25..11-11): 32 of 140 days eliminated; longest feasible blocks Jul 22-Aug 6, Jul 2-15, Aug 9-19. ELIMINATES ONLY - no surviving day is favoured. Per-day table: qc/imagery_date_evidence/weather/flyable_days.csv.</t>
+          <t>*** SUPERSEDED 2026-08-23 by 2021_snoh_6in_rgbi.tif (full study extent on the native 0.5-ft lattice, nearest; this 53.4% clip was served bilinear on an unsnapped grid and is kept for provenance) *** CLOSED LEADS: no WA consortium flight-date layer exists for 2021 or later (all 68 WAGeoservices services + 225 items enumerated; series ends 2020); the mosaic-catalog schema has no date field at all; WA NAIP 2021 does not cover quad 47122 (eastern WA only), so no NAIP ride-along date. Remaining route: the Hexagon flight log via Snohomish County DoIT, or the consortium contact (Joanne Markert, WA OCIO). Weather elimination (ASOS KPAE+KSEA+KBFI, criterion calibrated to 46/46 known Edmonds flight days; 2021-06-25..11-11): 32 of 140 days eliminated; longest feasible blocks Jul 22-Aug 6, Jul 2-15, Aug 9-19. ELIMINATES ONLY - no surviving day is favoured. Per-day table: qc/imagery_date_evidence/weather/flyable_days.csv.</t>
         </is>
       </c>
       <c r="Q18" s="1" t="inlineStr">
@@ -16250,8 +16312,198 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>2021_snoh_6in_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="inlineStr">
+        <is>
+          <t>2021s (campaign S21)</t>
+        </is>
+      </c>
+      <c r="C39" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2021/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D39" s="1" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="E39" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F39" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G39" s="1" t="inlineStr">
+        <is>
+          <t>15.24</t>
+        </is>
+      </c>
+      <c r="H39" s="1" t="inlineStr">
+        <is>
+          <t>20.06 (median of 5 sites; 1.32x its grid); common grid vs held: 20.05 vs 21.09 cm, HF ratio 1.432</t>
+        </is>
+      </c>
+      <c r="I39" s="1" t="inlineStr">
+        <is>
+          <t>15.24 (0.5 ft)</t>
+        </is>
+      </c>
+      <c r="J39" s="1" t="inlineStr">
+        <is>
+          <t>2021-06-25 to 2021-11-11</t>
+        </is>
+      </c>
+      <c r="K39" s="1" t="inlineStr">
+        <is>
+          <t>window of 140 days</t>
+        </is>
+      </c>
+      <c r="L39" s="1" t="inlineStr">
+        <is>
+          <t>unknown; the superseded clip was flown in the AFTERNOON (shadow azimuth)</t>
+        </is>
+      </c>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="N39" s="1" t="inlineStr">
+        <is>
+          <t>https://snohomishcountywa.gov/5414/Interactive-Map-SCOPI</t>
+        </is>
+      </c>
+      <c r="O39" s="1" t="inlineStr">
+        <is>
+          <t>The 2021 aerial photos are 6 inch resolution and cover mainly the urban areas. The imagery was collected between June 25, 2021 and November 11, 2021.</t>
+        </is>
+      </c>
+      <c r="P39" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S21\measure.json): 50232x70518 px, 4 bands, EPSG:2285, 10,764,289,402 B; city coverage 100.0%, study-extent 100.0%; band 4 NIR (std 58.9, NDVI p90 0.618); JPEG 8x8 signature absent. Decision REPLACE: wins=['coverage 100.0 &gt; 39.5', 'HF energy ratio 1.432 (sharper on a common grid)'] losses=[]. inherits the 2021_snoh_rgbi.tif evidence</t>
+        </is>
+      </c>
+      <c r="Q39" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R39" s="1" t="inlineStr"/>
+      <c r="S39" s="1" t="inlineStr"/>
+      <c r="T39" s="1" t="inlineStr"/>
+      <c r="U39" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>2015_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="inlineStr">
+        <is>
+          <t>2015s (campaign S15)</t>
+        </is>
+      </c>
+      <c r="C40" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2015/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E40" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F40" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G40" s="1" t="inlineStr">
+        <is>
+          <t>30.48</t>
+        </is>
+      </c>
+      <c r="H40" s="1" t="inlineStr">
+        <is>
+          <t>41.39 (median of 5 sites; 1.36x its grid)</t>
+        </is>
+      </c>
+      <c r="I40" s="1" t="inlineStr">
+        <is>
+          <t>30.48</t>
+        </is>
+      </c>
+      <c r="J40" s="1" t="inlineStr">
+        <is>
+          <t>2015-08-07 15:31 (HXIP 2015 1-ft flight over Edmonds = the NAIP 2015 delivery)</t>
+        </is>
+      </c>
+      <c r="K40" s="1" t="inlineStr">
+        <is>
+          <t>single day + minute</t>
+        </is>
+      </c>
+      <c r="L40" s="1" t="inlineStr">
+        <is>
+          <t>single sortie over the city footprints</t>
+        </is>
+      </c>
+      <c r="M40" s="4" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="N40" s="1" t="inlineStr">
+        <is>
+          <t>https://services.arcgis.com/jsIt88o09Q0r1j8h/arcgis/rest/services/NAIP_2015_1ft_Ortho_Dates_and_Times_83s/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="O40" s="1" t="inlineStr">
+        <is>
+          <t>"THEMENAME":"hxip_m_4712213_se_10_30","SDATE":"08/07/2015 15:31","SUNEL":46,"ACCURACY":"0.72m (ce 95%)" (city-centroid point query; raw response qc/imagery_date_evidence/raw_records/wa_2015_1ft_citycentroid.json)</t>
+        </is>
+      </c>
+      <c r="P40" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S15\measure.json): 25116x35259 px, 3 bands, EPSG:2285, 1,209,251,170 B; city coverage 100.0%, study-extent 100.0%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. band 4 = ALPHA (pilot, both rendering modes) - exported 3-band</t>
+        </is>
+      </c>
+      <c r="Q40" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R40" s="1" t="inlineStr"/>
+      <c r="S40" s="1" t="inlineStr"/>
+      <c r="T40" s="1" t="inlineStr"/>
+      <c r="U40" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U38"/>
+  <autoFilter ref="A1:U40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17578,7 +17830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P229"/>
+  <dimension ref="A1:P231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -30377,7 +30629,7 @@
       </c>
       <c r="N156" s="1" t="inlineStr">
         <is>
-          <t>YES - re-acquire full extent from the Snohomish ImageServer (Tier A, alongside 2016)</t>
+          <t>REPLACE 2026-08-23 -&gt; 2021_snoh_6in_rgbi.tif (coverage 100.0 &gt; 39.5; HF energy ratio 1.432 (sharper on a common grid)). YES - re-acquire full extent from the Snohomish ImageServer (Tier A, alongside 2016)</t>
         </is>
       </c>
       <c r="O156" s="1" t="inlineStr">
@@ -30541,7 +30793,7 @@
       </c>
       <c r="N158" s="1" t="inlineStr">
         <is>
-          <t>YES - re-acquire full extent from the Snohomish ImageServer (Tier A, alongside 2016)</t>
+          <t>REPLACE 2026-08-23 -&gt; 2021_snoh_6in_rgbi.tif (coverage 100.0 &gt; 39.5; HF energy ratio 1.432 (sharper on a common grid)). YES - re-acquire full extent from the Snohomish ImageServer (Tier A, alongside 2016)</t>
         </is>
       </c>
       <c r="O158" s="1" t="inlineStr">
@@ -30787,7 +31039,7 @@
       </c>
       <c r="N161" s="1" t="inlineStr">
         <is>
-          <t>YES - re-acquire full extent from the Snohomish ImageServer (Tier A, alongside 2016)</t>
+          <t>REPLACE 2026-08-23 -&gt; 2021_snoh_6in_rgbi.tif (coverage 100.0 &gt; 39.5; HF energy ratio 1.432 (sharper on a common grid)). YES - re-acquire full extent from the Snohomish ImageServer (Tier A, alongside 2016)</t>
         </is>
       </c>
       <c r="O161" s="1" t="inlineStr">
@@ -36286,7 +36538,6 @@
           <t>see Pixel_Size_And_Date row</t>
         </is>
       </c>
-      <c r="F229" t="inlineStr"/>
       <c r="G229" t="inlineStr">
         <is>
           <t>true GSD 30.48 cm; 4 bands; effective 42.58 cm; EPSG:2285; city coverage 100.0%</t>
@@ -36335,6 +36586,161 @@
       <c r="P229" t="inlineStr">
         <is>
           <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S19</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_2021 full extent, native 0.5 ft RGBI</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>true GSD 15.24 cm; 4 bands; effective 20.06 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2021/ImageServer</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2021/ImageServer</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>2021_snoh_6in_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>this file REPLACES 2021_snoh_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P230" t="inlineStr">
+        <is>
+          <t>decision REPLACE: wins=['coverage 100.0 &gt; 39.5', 'HF energy ratio 1.432 (sharper on a common grid)'] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S21</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_2015 1 ft RGB (band 4 = alpha, dropped)</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr"/>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>true GSD 30.48 cm; 3 bands; effective 41.39 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2015/ImageServer</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2015/ImageServer</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>2015_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N231" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P231" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S15</t>
         </is>
       </c>
     </row>
@@ -37174,7 +37580,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>YES - re-acquire full extent from the Snohomish ImageServer (Tier A, alongside 2016)</t>
+          <t>RESOLVED 2026-08-23: REPLACE by 2021_snoh_6in_rgbi.tif. YES - re-acquire full extent from the Snohomish ImageServer (Tier A, alongside 2016)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
batch 4 + N23f: S18 fills the 2018 gap (key 2018s, NIR, 2018-08-07); N23f REPLACE #4 (2023n -> original DOQQs, coverage 100 vs 67%, HF 1.41); pan years S90/S98/S01 held without year keys (ADOPTED_NON_YEAR, King pans moved in; orphans = the 2 real decisions); table 44 rows gate 0 misses; check 25/25
</commit_message>
<xml_diff>
--- a/Scripts/imagery_catalog_2026-08-22.xlsx
+++ b/Scripts/imagery_catalog_2026-08-22.xlsx
@@ -33,7 +33,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing_Risk" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MASTER'!$A$1:$P$221</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'KingCo_SDC_Catalog'!$A$1:$D$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DataLake_Issues'!$A$1:$C$15</definedName>
@@ -10920,7 +10920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11665,6 +11665,161 @@
       <c r="G22" t="inlineStr">
         <is>
           <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2018_snoh_6in_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>15.24</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="E23" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1990_snoh_10ft_pan.tif</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>304.801</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="E24" t="n">
+        <v>367.45</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>median of 3 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1998_snoh_3ft_pan.tif</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>91.44</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="E25" t="n">
+        <v>163.09</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2001_snoh_1ft_pan.tif</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>30.48</v>
+      </c>
+      <c r="D26" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="E26" t="n">
+        <v>105.13</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2023_naip_60cm_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>NAIP_AZURE/2023</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>60</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="E27" t="n">
+        <v>82.56</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>median of 5 Method_Provenance sites; common-grid vs 2023_naip_rgbi.tif: new 83.49 / held 84.61 cm, HF ratio 1.406</t>
         </is>
       </c>
     </row>
@@ -12460,7 +12615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U40"/>
+  <dimension ref="A1:U45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -15024,7 +15179,7 @@
       </c>
       <c r="P25" s="1" t="inlineStr">
         <is>
-          <t>OCTOBER. Held bands 1-3 byte-identical to rgb_2023, band 4 to ir_2023 (DataLake_Issues). Context: NAIP 2021 over Edmonds exists (all 8 QQs STAC datetime 2021-07-13, INFERRED from file names - the FGDC sidecars for quad 47122 are absent from the Azure mirror).</t>
+          <t>*** SUPERSEDED 2026-08-23 by 2023_naip_60cm_rgbi.tif (the 8 original Azure DOQQs mosaicked, full study extent; this 69% smoothed re-export is kept for provenance) *** OCTOBER. Held bands 1-3 byte-identical to rgb_2023, band 4 to ir_2023 (DataLake_Issues). Context: NAIP 2021 over Edmonds exists (all 8 QQs STAC datetime 2021-07-13, INFERRED from file names - the FGDC sidecars for quad 47122 are absent from the Azure mirror).</t>
         </is>
       </c>
       <c r="Q25" s="1" t="inlineStr">
@@ -16502,8 +16657,483 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>2018_snoh_6in_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>2018s (campaign S18)</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2018/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F41" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>15.24</t>
+        </is>
+      </c>
+      <c r="H41" s="1" t="inlineStr">
+        <is>
+          <t>20.9 (median of 5 sites; 1.37x its grid)</t>
+        </is>
+      </c>
+      <c r="I41" s="1" t="inlineStr">
+        <is>
+          <t>15.24 (0.5 ft HXIP 6-in delivery)</t>
+        </is>
+      </c>
+      <c r="J41" s="1" t="inlineStr">
+        <is>
+          <t>2018-08-07 (WA consortium 6-in flight area over Edmonds)</t>
+        </is>
+      </c>
+      <c r="K41" s="1" t="inlineStr">
+        <is>
+          <t>single day</t>
+        </is>
+      </c>
+      <c r="L41" s="1" t="inlineStr">
+        <is>
+          <t>single flight area</t>
+        </is>
+      </c>
+      <c r="M41" s="4" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="N41" s="1" t="inlineStr">
+        <is>
+          <t>https://services.arcgis.com/jsIt88o09Q0r1j8h/arcgis/rest/services/2018_Statewide_imagery_consortium_6_inch_flight_areas/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="O41" s="1" t="inlineStr">
+        <is>
+          <t>"IDATE":"2018-08-07" (city-centroid and city-bbox queries agree; raw responses qc/imagery_date_evidence/raw_records/wa_2018_6in_city*.json)</t>
+        </is>
+      </c>
+      <c r="P41" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S18\measure.json): 50232x70518 px, 4 bands, EPSG:2285, 11,470,030,126 B; city coverage 100.0%, study-extent 100.0%; band 4 NIR (std 62.34, NDVI p90 0.713); JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. the ONLY citywide 2018 imagery held; same Aug-07 day-of-month as the 2015 flight by coincidence</t>
+        </is>
+      </c>
+      <c r="Q41" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R41" s="1" t="inlineStr"/>
+      <c r="S41" s="1" t="inlineStr"/>
+      <c r="T41" s="1" t="inlineStr"/>
+      <c r="U41" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>1990_snoh_10ft_pan.tif</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>1990s (campaign S90)</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_1990/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F42" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G42" s="1" t="inlineStr">
+        <is>
+          <t>304.8</t>
+        </is>
+      </c>
+      <c r="H42" s="1" t="inlineStr">
+        <is>
+          <t>367.45 (median of 3 sites; 1.21x its grid)</t>
+        </is>
+      </c>
+      <c r="I42" s="1" t="inlineStr">
+        <is>
+          <t>304.8 (10 ft)</t>
+        </is>
+      </c>
+      <c r="J42" s="1" t="inlineStr">
+        <is>
+          <t>NOT FOUND (year from the county service name Aerial_1990 only)</t>
+        </is>
+      </c>
+      <c r="K42" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L42" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M42" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N42" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_1990/ImageServer</t>
+        </is>
+      </c>
+      <c r="O42" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P42" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S90\measure.json): 2513x3527 px, 1 bands, EPSG:2285, 6,713,257 B; city coverage 98.97%, study-extent 86.59%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. 10-ft b/w; SCOPI's per-year list starts at 2017; no flight-date record found for any pan year</t>
+        </is>
+      </c>
+      <c r="Q42" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R42" s="1" t="inlineStr"/>
+      <c r="S42" s="1" t="inlineStr"/>
+      <c r="T42" s="1" t="inlineStr"/>
+      <c r="U42" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>1998_snoh_3ft_pan.tif</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>1998s (campaign S98)</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_1998/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F43" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="inlineStr">
+        <is>
+          <t>91.44</t>
+        </is>
+      </c>
+      <c r="H43" s="1" t="inlineStr">
+        <is>
+          <t>163.09 (median of 5 sites; 1.78x its grid)</t>
+        </is>
+      </c>
+      <c r="I43" s="1" t="inlineStr">
+        <is>
+          <t>91.44 (3 ft DNR scan)</t>
+        </is>
+      </c>
+      <c r="J43" s="1" t="inlineStr">
+        <is>
+          <t>NOT FOUND (year only; the service's keyProperties name the SOURCE, not the date)</t>
+        </is>
+      </c>
+      <c r="K43" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L43" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N43" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_1998/ImageServer/keyProperties?f=json</t>
+        </is>
+      </c>
+      <c r="O43" s="1" t="inlineStr">
+        <is>
+          <t>U:\\1998\\b-w\\3ft_res\\dnr\\t26nr04e.tif (keyProperties IMAGE__INPUT_NAME, JSON escaping verbatim - a WA DNR 3-ft b/w product; raw response qc/imagery_date_evidence/raw_records/snoco_1998_keyProperties.json)</t>
+        </is>
+      </c>
+      <c r="P43" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S98\measure.json): 8373x11754 px, 1 bands, EPSG:2285, 79,721,073 B; city coverage 100.0%, study-extent 99.71%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. source = WA DNR 1998 orthophoto scan; pairs with the held 1998_king_pan (different product)</t>
+        </is>
+      </c>
+      <c r="Q43" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R43" s="1" t="inlineStr"/>
+      <c r="S43" s="1" t="inlineStr"/>
+      <c r="T43" s="1" t="inlineStr"/>
+      <c r="U43" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>2001_snoh_1ft_pan.tif</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>2001s (campaign S01)</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2001/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F44" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="inlineStr">
+        <is>
+          <t>30.48</t>
+        </is>
+      </c>
+      <c r="H44" s="1" t="inlineStr">
+        <is>
+          <t>105.13 (median of 5 sites; 3.45x its grid)</t>
+        </is>
+      </c>
+      <c r="I44" s="1" t="inlineStr">
+        <is>
+          <t>30.48 (1 ft scanned film)</t>
+        </is>
+      </c>
+      <c r="J44" s="1" t="inlineStr">
+        <is>
+          <t>NOT FOUND (year from the county service name Aerial_2001 only)</t>
+        </is>
+      </c>
+      <c r="K44" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L44" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M44" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N44" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2001/ImageServer</t>
+        </is>
+      </c>
+      <c r="O44" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P44" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S01\measure.json): 25117x35260 px, 1 bands, EPSG:2285, 474,665,129 B; city coverage 99.9%, study-extent 75.13%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. 1-ft scanned film (effective 105 cm); no flight-date record found</t>
+        </is>
+      </c>
+      <c r="Q44" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R44" s="1" t="inlineStr"/>
+      <c r="S44" s="1" t="inlineStr"/>
+      <c r="T44" s="1" t="inlineStr"/>
+      <c r="U44" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>2023_naip_60cm_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>2023n (campaign N23f)</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2023/wa_060cm_2023/47122/ via pipeline/acquire_imagery.py (files)</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>metre</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:26910</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="H45" s="1" t="inlineStr">
+        <is>
+          <t>82.56 (median of 5 sites; 1.38x its grid); common grid vs held: 83.49 vs 84.61 cm, HF ratio 1.406</t>
+        </is>
+      </c>
+      <c r="I45" s="1" t="inlineStr">
+        <is>
+          <t>60 (delivered DOQQ)</t>
+        </is>
+      </c>
+      <c r="J45" s="1" t="inlineStr">
+        <is>
+          <t>2023-10-07</t>
+        </is>
+      </c>
+      <c r="K45" s="1" t="inlineStr">
+        <is>
+          <t>single day</t>
+        </is>
+      </c>
+      <c r="L45" s="1" t="inlineStr">
+        <is>
+          <t>single (all 8 quads 2023-10-07)</t>
+        </is>
+      </c>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="N45" s="1" t="inlineStr">
+        <is>
+          <t>https://naipeuwest.blob.core.windows.net/naip?restype=container&amp;comp=list&amp;prefix=v002/wa/2023/wa_060cm_2023/47122/m_47122&amp;maxresults=200</t>
+        </is>
+      </c>
+      <c r="O45" s="1" t="inlineStr">
+        <is>
+          <t>m_4712213_ne_10_060_20231007_20240209.tif ... m_4712214_sw_10_060_20231007_20240209.tif (all 8 Edmonds quads carry capture 20231007 + version 20240209; listing saved qc/imagery_date_evidence/raw_records/azure_naip_2023_47122_listing.xml)</t>
+        </is>
+      </c>
+      <c r="P45" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\NAIP_AZURE\2023\_acq\N23f\measure.json): 12556x17768 px, 4 bands, EPSG:26910, 727,595,134 B; city coverage 100.0%, study-extent 100.0%; band 4 NIR (std 57.93, NDVI p90 0.529); JPEG 8x8 signature absent. Decision REPLACE: wins=['coverage 100.0 &gt; 66.98', 'HF energy ratio 1.406 (sharper on a common grid)'] losses=[]. confirms the held 2023n date independently; October leaf-state caveat as 2019n/2019s</t>
+        </is>
+      </c>
+      <c r="Q45" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R45" s="1" t="inlineStr"/>
+      <c r="S45" s="1" t="inlineStr"/>
+      <c r="T45" s="1" t="inlineStr"/>
+      <c r="U45" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U40"/>
+  <autoFilter ref="A1:U45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17830,7 +18460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P231"/>
+  <dimension ref="A1:P236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -36692,7 +37322,6 @@
           <t>see Pixel_Size_And_Date row</t>
         </is>
       </c>
-      <c r="F231" t="inlineStr"/>
       <c r="G231" t="inlineStr">
         <is>
           <t>true GSD 30.48 cm; 3 bands; effective 41.39 cm; EPSG:2285; city coverage 100.0%</t>
@@ -36741,6 +37370,392 @@
       <c r="P231" t="inlineStr">
         <is>
           <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S15</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_2018 HXIP 6-in RGBI (2018-08-07)</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>true GSD 15.24 cm; 4 bands; effective 20.9 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2018/ImageServer</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2018/ImageServer</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>2018_snoh_6in_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N232" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P232" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S18</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>1990</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_1990 10-ft b/w</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>true GSD 304.801 cm; 1 bands; effective 367.45 cm; EPSG:2285; city coverage 98.97%</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_1990/ImageServer</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_1990/ImageServer</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>1990_snoh_10ft_pan.tif</t>
+        </is>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N233" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P233" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S90</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_1998 3-ft b/w (DNR scan)</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>true GSD 91.44 cm; 1 bands; effective 163.09 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_1998/ImageServer</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_1998/ImageServer</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>1998_snoh_3ft_pan.tif</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N234" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P234" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S98</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_2001 1-ft b/w</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>true GSD 30.48 cm; 1 bands; effective 105.13 cm; EPSG:2285; city coverage 99.9%</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2001/ImageServer</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2001/ImageServer</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K235" t="inlineStr">
+        <is>
+          <t>2001_snoh_1ft_pan.tif</t>
+        </is>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N235" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P235" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S01</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>NAIP 2023 full-extent DOQQ mosaic (2023-10-07)</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr"/>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>true GSD 60.0 cm; 4 bands; effective 82.56 cm; EPSG:26910; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2023/wa_060cm_2023/47122/</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2023/wa_060cm_2023/47122/</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t>2023_naip_60cm_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N236" t="inlineStr">
+        <is>
+          <t>this file REPLACES 2023_naip_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P236" t="inlineStr">
+        <is>
+          <t>decision REPLACE: wins=['coverage 100.0 &gt; 66.98', 'HF energy ratio 1.406 (sharper on a common grid)'] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\NAIP_AZURE\2023\_acq\N23f</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
batch 5 snoco: S02 NOT a duplicate of the USGS flight (r .847 - a second 2002 acquisition, key 2002s); 2003s = a new project year; S07 flip test failed, King keeps 2007 (key 2007s); drive-mount correction recorded (G: = cache disk C:, cloud is 808GB/2TB); CITY_SHP local-first; table 47 rows
</commit_message>
<xml_diff>
--- a/Scripts/imagery_catalog_2026-08-22.xlsx
+++ b/Scripts/imagery_catalog_2026-08-22.xlsx
@@ -33,7 +33,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing_Risk" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MASTER'!$A$1:$P$221</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'KingCo_SDC_Catalog'!$A$1:$D$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DataLake_Issues'!$A$1:$C$15</definedName>
@@ -10920,7 +10920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11820,6 +11820,99 @@
       <c r="G27" t="inlineStr">
         <is>
           <t>median of 5 Method_Provenance sites; common-grid vs 2023_naip_rgbi.tif: new 83.49 / held 84.61 cm, HF ratio 1.406</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2002_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>30.48</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="E28" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2003_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>30.48</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="E29" t="n">
+        <v>41.62</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2007_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>30.48</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="E30" t="n">
+        <v>38.53</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
         </is>
       </c>
     </row>
@@ -12615,7 +12708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U45"/>
+  <dimension ref="A1:U48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -16200,12 +16293,12 @@
       </c>
       <c r="D36" s="1" t="inlineStr">
         <is>
-          <t>0.037323</t>
+          <t>0.03732276770595208</t>
         </is>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>metre (Web Mercator, inflated 1/cos(lat))</t>
+          <t>metre</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
@@ -16215,7 +16308,7 @@
       </c>
       <c r="G36" s="1" t="inlineStr">
         <is>
-          <t>2.51</t>
+          <t>2.507</t>
         </is>
       </c>
       <c r="H36" s="1" t="inlineStr">
@@ -17132,8 +17225,293 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>2002_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>2002s (campaign S02)</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2002/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F46" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="inlineStr">
+        <is>
+          <t>30.48</t>
+        </is>
+      </c>
+      <c r="H46" s="1" t="inlineStr">
+        <is>
+          <t>42.1 (median of 5 sites; 1.38x its grid)</t>
+        </is>
+      </c>
+      <c r="I46" s="1" t="inlineStr">
+        <is>
+          <t>30.48 (1 ft)</t>
+        </is>
+      </c>
+      <c r="J46" s="1" t="inlineStr">
+        <is>
+          <t>NOT FOUND (year from the county service name Aerial_2002 only)</t>
+        </is>
+      </c>
+      <c r="K46" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L46" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N46" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2002/ImageServer</t>
+        </is>
+      </c>
+      <c r="O46" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P46" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S02\measure.json): 25116x35259 px, 3 bands, EPSG:2285, 1,704,437,706 B; city coverage None%, study-extent 87.61%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. NOT the USGS HRO flight: dup test vs 2002_usgs_30cm_rgb r median 0.847 at the 5 sites (same-flight pairs run 0.98-0.997; SnoCo/_acq/S02/dup_test_vs_U02.json) - a second, distinct 2002 acquisition with its own unknown date</t>
+        </is>
+      </c>
+      <c r="Q46" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R46" s="1" t="inlineStr"/>
+      <c r="S46" s="1" t="inlineStr"/>
+      <c r="T46" s="1" t="inlineStr"/>
+      <c r="U46" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>2003_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>2003s (campaign S03)</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2003/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="inlineStr">
+        <is>
+          <t>30.48</t>
+        </is>
+      </c>
+      <c r="H47" s="1" t="inlineStr">
+        <is>
+          <t>41.62 (median of 5 sites; 1.37x its grid)</t>
+        </is>
+      </c>
+      <c r="I47" s="1" t="inlineStr">
+        <is>
+          <t>30.48 (1 ft)</t>
+        </is>
+      </c>
+      <c r="J47" s="1" t="inlineStr">
+        <is>
+          <t>NOT FOUND (year from the county service name Aerial_2003 only)</t>
+        </is>
+      </c>
+      <c r="K47" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L47" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M47" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N47" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2003/ImageServer</t>
+        </is>
+      </c>
+      <c r="O47" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P47" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S03\measure.json): 25116x35259 px, 3 bands, EPSG:2285, 1,501,046,192 B; city coverage None%, study-extent 87.49%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. 2003 = a calendar year the project previously had NO imagery for</t>
+        </is>
+      </c>
+      <c r="Q47" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R47" s="1" t="inlineStr"/>
+      <c r="S47" s="1" t="inlineStr"/>
+      <c r="T47" s="1" t="inlineStr"/>
+      <c r="U47" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>2007_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>2007s (campaign S07)</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2007/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>30.48</t>
+        </is>
+      </c>
+      <c r="H48" s="1" t="inlineStr">
+        <is>
+          <t>38.53 (median of 5 sites; 1.26x its grid); common grid vs held: 39.58 vs 39.34 cm, HF ratio 1.654</t>
+        </is>
+      </c>
+      <c r="I48" s="1" t="inlineStr">
+        <is>
+          <t>30.48 (1 ft)</t>
+        </is>
+      </c>
+      <c r="J48" s="1" t="inlineStr">
+        <is>
+          <t>NOT FOUND (year from the county service name Aerial_2007 only)</t>
+        </is>
+      </c>
+      <c r="K48" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L48" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M48" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N48" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2007/ImageServer</t>
+        </is>
+      </c>
+      <c r="O48" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P48" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S07\measure.json): 25116x35259 px, 3 bands, EPSG:2285, 1,548,181,188 B; city coverage None%, study-extent 100.0%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=['HF energy ratio 1.654 (sharper on a common grid)', 'no JPEG block signature (held has one)'] losses=[]. flip test vs 2007_king FAILED (eff 38.5 vs required &lt; 22.95) - complement, King keeps the 2007 key</t>
+        </is>
+      </c>
+      <c r="Q48" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R48" s="1" t="inlineStr"/>
+      <c r="S48" s="1" t="inlineStr"/>
+      <c r="T48" s="1" t="inlineStr"/>
+      <c r="U48" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U45"/>
+  <autoFilter ref="A1:U48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18460,7 +18838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P236"/>
+  <dimension ref="A1:P239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -37707,7 +38085,6 @@
           <t>see Pixel_Size_And_Date row</t>
         </is>
       </c>
-      <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
           <t>true GSD 60.0 cm; 4 bands; effective 82.56 cm; EPSG:26910; city coverage 100.0%</t>
@@ -37756,6 +38133,238 @@
       <c r="P236" t="inlineStr">
         <is>
           <t>decision REPLACE: wins=['coverage 100.0 &gt; 66.98', 'HF energy ratio 1.406 (sharper on a common grid)'] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\NAIP_AZURE\2023\_acq\N23f</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>2002</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_2002 1-ft RGB (NOT the USGS flight: dup r 0.847)</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>true GSD 30.48 cm; 3 bands; effective 42.1 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2002/ImageServer</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2002/ImageServer</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K237" t="inlineStr">
+        <is>
+          <t>2002_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N237" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P237" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S02</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_2003 1-ft RGB (new project year)</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>true GSD 30.48 cm; 3 bands; effective 41.62 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2003/ImageServer</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2003/ImageServer</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>2003_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N238" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P238" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S03</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_2007 1-ft RGB (flip test vs 2007_king failed - complement)</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr"/>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>true GSD 30.48 cm; 3 bands; effective 38.53 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2007/ImageServer</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2007/ImageServer</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>2007_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N239" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P239" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=['HF energy ratio 1.654 (sharper on a common grid)', 'no JPEG block signature (held has one)'] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
N19f REPLACE #5: 2019n -> original DOQQs (coverage 100 vs 67, HF 1.36, 2019-10-11 single day); the 0.148px reg loss PROVEN a blur artifact of the metric before overriding (registration_blur_test.json) - waiver recorded, original verdict preserved; catalog 28/28, table 48 rows
</commit_message>
<xml_diff>
--- a/Scripts/imagery_catalog_2026-08-22.xlsx
+++ b/Scripts/imagery_catalog_2026-08-22.xlsx
@@ -33,7 +33,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing_Risk" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MASTER'!$A$1:$P$221</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'KingCo_SDC_Catalog'!$A$1:$D$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DataLake_Issues'!$A$1:$C$15</definedName>
@@ -10920,7 +10920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11913,6 +11913,37 @@
       <c r="G30" t="inlineStr">
         <is>
           <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2019_naip_60cm_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>NAIP_AZURE/2019</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>60</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="E31" t="n">
+        <v>82.54000000000001</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>median of 5 Method_Provenance sites; common-grid vs 2019_naip_rgbi.tif: new 84.3 / held 87.38 cm, HF ratio 1.358</t>
         </is>
       </c>
     </row>
@@ -12708,7 +12739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U48"/>
+  <dimension ref="A1:U49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -15165,7 +15196,7 @@
       </c>
       <c r="P24" s="1" t="inlineStr">
         <is>
-          <t>OCTOBER. No NAIP metadata record (2015/2017/2021 Digital Coast) contains any leaf-on/leaf-off statement - only 'peak crop growing conditions'; the 'NAIP is leaf-on by spec' assumption has no documentary basis.</t>
+          <t>*** SUPERSEDED 2026-08-23 by 2019_naip_60cm_rgbi.tif (the 8 original Azure DOQQs, full study extent; this 69% smoothed re-export is kept for provenance) *** OCTOBER. No NAIP metadata record (2015/2017/2021 Digital Coast) contains any leaf-on/leaf-off statement - only 'peak crop growing conditions'; the 'NAIP is leaf-on by spec' assumption has no documentary basis.</t>
         </is>
       </c>
       <c r="Q24" s="1" t="inlineStr">
@@ -16293,12 +16324,12 @@
       </c>
       <c r="D36" s="1" t="inlineStr">
         <is>
-          <t>0.03732276770595208</t>
+          <t>0.037323</t>
         </is>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>metre</t>
+          <t>metre (Web Mercator, inflated 1/cos(lat))</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
@@ -16308,7 +16339,7 @@
       </c>
       <c r="G36" s="1" t="inlineStr">
         <is>
-          <t>2.507</t>
+          <t>2.51</t>
         </is>
       </c>
       <c r="H36" s="1" t="inlineStr">
@@ -17133,17 +17164,17 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>2023_naip_60cm_rgbi.tif</t>
+          <t>2019_naip_60cm_rgbi.tif</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>2023n (campaign N23f)</t>
+          <t>2019n (campaign N19f)</t>
         </is>
       </c>
       <c r="C45" s="1" t="inlineStr">
         <is>
-          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2023/wa_060cm_2023/47122/ via pipeline/acquire_imagery.py (files)</t>
+          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2019/wa_60cm_2019/47122/ via pipeline/acquire_imagery.py (files)</t>
         </is>
       </c>
       <c r="D45" s="1" t="inlineStr">
@@ -17168,7 +17199,7 @@
       </c>
       <c r="H45" s="1" t="inlineStr">
         <is>
-          <t>82.56 (median of 5 sites; 1.38x its grid); common grid vs held: 83.49 vs 84.61 cm, HF ratio 1.406</t>
+          <t>82.54 (median of 5 sites; 1.38x its grid); common grid vs held: 84.3 vs 87.38 cm, HF ratio 1.358</t>
         </is>
       </c>
       <c r="I45" s="1" t="inlineStr">
@@ -17178,7 +17209,7 @@
       </c>
       <c r="J45" s="1" t="inlineStr">
         <is>
-          <t>2023-10-07</t>
+          <t>2019-10-11</t>
         </is>
       </c>
       <c r="K45" s="1" t="inlineStr">
@@ -17188,7 +17219,7 @@
       </c>
       <c r="L45" s="1" t="inlineStr">
         <is>
-          <t>single (all 8 quads 2023-10-07)</t>
+          <t>single (all 8 quads 2019-10-11)</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr">
@@ -17198,17 +17229,17 @@
       </c>
       <c r="N45" s="1" t="inlineStr">
         <is>
-          <t>https://naipeuwest.blob.core.windows.net/naip?restype=container&amp;comp=list&amp;prefix=v002/wa/2023/wa_060cm_2023/47122/m_47122&amp;maxresults=200</t>
+          <t>https://naipeuwest.blob.core.windows.net/naip?restype=container&amp;comp=list&amp;prefix=v002/wa/2019/wa_60cm_2019/47122/m_47122&amp;maxresults=200</t>
         </is>
       </c>
       <c r="O45" s="1" t="inlineStr">
         <is>
-          <t>m_4712213_ne_10_060_20231007_20240209.tif ... m_4712214_sw_10_060_20231007_20240209.tif (all 8 Edmonds quads carry capture 20231007 + version 20240209; listing saved qc/imagery_date_evidence/raw_records/azure_naip_2023_47122_listing.xml)</t>
+          <t>m_4712213_ne_10_060_20191011.tif ... m_4712214_sw_10_060_20191011.tif (all 8 Edmonds quads carry 20191011; listing saved qc/imagery_date_evidence/raw_records/azure_naip_2019_47122_listing.xml)</t>
         </is>
       </c>
       <c r="P45" s="1" t="inlineStr">
         <is>
-          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\NAIP_AZURE\2023\_acq\N23f\measure.json): 12556x17768 px, 4 bands, EPSG:26910, 727,595,134 B; city coverage 100.0%, study-extent 100.0%; band 4 NIR (std 57.93, NDVI p90 0.529); JPEG 8x8 signature absent. Decision REPLACE: wins=['coverage 100.0 &gt; 66.98', 'HF energy ratio 1.406 (sharper on a common grid)'] losses=[]. confirms the held 2023n date independently; October leaf-state caveat as 2019n/2019s</t>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\NAIP_AZURE\2019\_acq\N19f\measure.json): 12556x17768 px, 4 bands, EPSG:26910, 757,507,269 B; city coverage 100.0%, study-extent 100.0%; band 4 NIR (std 60.69, NDVI p90 0.56); JPEG 8x8 signature absent. Decision REPLACE: wins=['coverage 100.0 &gt; 66.98', 'HF energy ratio 1.358 (sharper on a common grid)'] losses=[]. = the S19/HXIP flight date (same Hexagon acquisition); replaces the smoothed 69% clip; reg-loss waived as a blur artifact of the metric (registration_blur_test.json)</t>
         </is>
       </c>
       <c r="Q45" s="1" t="inlineStr">
@@ -17228,82 +17259,82 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>2002_snoh_1ft_rgb.tif</t>
+          <t>2023_naip_60cm_rgbi.tif</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>2002s (campaign S02)</t>
+          <t>2023n (campaign N23f)</t>
         </is>
       </c>
       <c r="C46" s="1" t="inlineStr">
         <is>
-          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2002/ImageServer via pipeline/acquire_imagery.py (export)</t>
+          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2023/wa_060cm_2023/47122/ via pipeline/acquire_imagery.py (files)</t>
         </is>
       </c>
       <c r="D46" s="1" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>US survey foot</t>
+          <t>metre</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>EPSG:2285</t>
+          <t>EPSG:26910</t>
         </is>
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>30.48</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="H46" s="1" t="inlineStr">
         <is>
-          <t>42.1 (median of 5 sites; 1.38x its grid)</t>
+          <t>82.56 (median of 5 sites; 1.38x its grid); common grid vs held: 83.49 vs 84.61 cm, HF ratio 1.406</t>
         </is>
       </c>
       <c r="I46" s="1" t="inlineStr">
         <is>
-          <t>30.48 (1 ft)</t>
+          <t>60 (delivered DOQQ)</t>
         </is>
       </c>
       <c r="J46" s="1" t="inlineStr">
         <is>
-          <t>NOT FOUND (year from the county service name Aerial_2002 only)</t>
+          <t>2023-10-07</t>
         </is>
       </c>
       <c r="K46" s="1" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>single day</t>
         </is>
       </c>
       <c r="L46" s="1" t="inlineStr">
         <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="M46" s="5" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
+          <t>single (all 8 quads 2023-10-07)</t>
+        </is>
+      </c>
+      <c r="M46" s="4" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="N46" s="1" t="inlineStr">
         <is>
-          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2002/ImageServer</t>
+          <t>https://naipeuwest.blob.core.windows.net/naip?restype=container&amp;comp=list&amp;prefix=v002/wa/2023/wa_060cm_2023/47122/m_47122&amp;maxresults=200</t>
         </is>
       </c>
       <c r="O46" s="1" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m_4712213_ne_10_060_20231007_20240209.tif ... m_4712214_sw_10_060_20231007_20240209.tif (all 8 Edmonds quads carry capture 20231007 + version 20240209; listing saved qc/imagery_date_evidence/raw_records/azure_naip_2023_47122_listing.xml)</t>
         </is>
       </c>
       <c r="P46" s="1" t="inlineStr">
         <is>
-          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S02\measure.json): 25116x35259 px, 3 bands, EPSG:2285, 1,704,437,706 B; city coverage None%, study-extent 87.61%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. NOT the USGS HRO flight: dup test vs 2002_usgs_30cm_rgb r median 0.847 at the 5 sites (same-flight pairs run 0.98-0.997; SnoCo/_acq/S02/dup_test_vs_U02.json) - a second, distinct 2002 acquisition with its own unknown date</t>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\NAIP_AZURE\2023\_acq\N23f\measure.json): 12556x17768 px, 4 bands, EPSG:26910, 727,595,134 B; city coverage 100.0%, study-extent 100.0%; band 4 NIR (std 57.93, NDVI p90 0.529); JPEG 8x8 signature absent. Decision REPLACE: wins=['coverage 100.0 &gt; 66.98', 'HF energy ratio 1.406 (sharper on a common grid)'] losses=[]. confirms the held 2023n date independently; October leaf-state caveat as 2019n/2019s</t>
         </is>
       </c>
       <c r="Q46" s="1" t="inlineStr">
@@ -17323,17 +17354,17 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>2003_snoh_1ft_rgb.tif</t>
+          <t>2002_snoh_1ft_rgb.tif</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>2003s (campaign S03)</t>
+          <t>2002s (campaign S02)</t>
         </is>
       </c>
       <c r="C47" s="1" t="inlineStr">
         <is>
-          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2003/ImageServer via pipeline/acquire_imagery.py (export)</t>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2002/ImageServer via pipeline/acquire_imagery.py (export)</t>
         </is>
       </c>
       <c r="D47" s="1" t="inlineStr">
@@ -17358,7 +17389,7 @@
       </c>
       <c r="H47" s="1" t="inlineStr">
         <is>
-          <t>41.62 (median of 5 sites; 1.37x its grid)</t>
+          <t>42.1 (median of 5 sites; 1.38x its grid)</t>
         </is>
       </c>
       <c r="I47" s="1" t="inlineStr">
@@ -17368,7 +17399,7 @@
       </c>
       <c r="J47" s="1" t="inlineStr">
         <is>
-          <t>NOT FOUND (year from the county service name Aerial_2003 only)</t>
+          <t>NOT FOUND (year from the county service name Aerial_2002 only)</t>
         </is>
       </c>
       <c r="K47" s="1" t="inlineStr">
@@ -17388,7 +17419,7 @@
       </c>
       <c r="N47" s="1" t="inlineStr">
         <is>
-          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2003/ImageServer</t>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2002/ImageServer</t>
         </is>
       </c>
       <c r="O47" s="1" t="inlineStr">
@@ -17398,7 +17429,7 @@
       </c>
       <c r="P47" s="1" t="inlineStr">
         <is>
-          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S03\measure.json): 25116x35259 px, 3 bands, EPSG:2285, 1,501,046,192 B; city coverage None%, study-extent 87.49%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. 2003 = a calendar year the project previously had NO imagery for</t>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S02\measure.json): 25116x35259 px, 3 bands, EPSG:2285, 1,704,437,706 B; city coverage 100.0%, study-extent 87.61%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. NOT the USGS HRO flight: dup test vs 2002_usgs_30cm_rgb r median 0.847 at the 5 sites (same-flight pairs run 0.98-0.997; SnoCo/_acq/S02/dup_test_vs_U02.json) - a second, distinct 2002 acquisition with its own unknown date</t>
         </is>
       </c>
       <c r="Q47" s="1" t="inlineStr">
@@ -17418,17 +17449,17 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>2007_snoh_1ft_rgb.tif</t>
+          <t>2003_snoh_1ft_rgb.tif</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t>2007s (campaign S07)</t>
+          <t>2003s (campaign S03)</t>
         </is>
       </c>
       <c r="C48" s="1" t="inlineStr">
         <is>
-          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2007/ImageServer via pipeline/acquire_imagery.py (export)</t>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2003/ImageServer via pipeline/acquire_imagery.py (export)</t>
         </is>
       </c>
       <c r="D48" s="1" t="inlineStr">
@@ -17453,7 +17484,7 @@
       </c>
       <c r="H48" s="1" t="inlineStr">
         <is>
-          <t>38.53 (median of 5 sites; 1.26x its grid); common grid vs held: 39.58 vs 39.34 cm, HF ratio 1.654</t>
+          <t>41.62 (median of 5 sites; 1.37x its grid)</t>
         </is>
       </c>
       <c r="I48" s="1" t="inlineStr">
@@ -17463,7 +17494,7 @@
       </c>
       <c r="J48" s="1" t="inlineStr">
         <is>
-          <t>NOT FOUND (year from the county service name Aerial_2007 only)</t>
+          <t>NOT FOUND (year from the county service name Aerial_2003 only)</t>
         </is>
       </c>
       <c r="K48" s="1" t="inlineStr">
@@ -17483,7 +17514,7 @@
       </c>
       <c r="N48" s="1" t="inlineStr">
         <is>
-          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2007/ImageServer</t>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2003/ImageServer</t>
         </is>
       </c>
       <c r="O48" s="1" t="inlineStr">
@@ -17493,7 +17524,7 @@
       </c>
       <c r="P48" s="1" t="inlineStr">
         <is>
-          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S07\measure.json): 25116x35259 px, 3 bands, EPSG:2285, 1,548,181,188 B; city coverage None%, study-extent 100.0%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=['HF energy ratio 1.654 (sharper on a common grid)', 'no JPEG block signature (held has one)'] losses=[]. flip test vs 2007_king FAILED (eff 38.5 vs required &lt; 22.95) - complement, King keeps the 2007 key</t>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S03\measure.json): 25116x35259 px, 3 bands, EPSG:2285, 1,501,046,192 B; city coverage 100.0%, study-extent 87.49%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. 2003 = a calendar year the project previously had NO imagery for</t>
         </is>
       </c>
       <c r="Q48" s="1" t="inlineStr">
@@ -17510,8 +17541,103 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>2007_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>2007s (campaign S07)</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2007/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
+        <is>
+          <t>30.48</t>
+        </is>
+      </c>
+      <c r="H49" s="1" t="inlineStr">
+        <is>
+          <t>38.53 (median of 5 sites; 1.26x its grid); common grid vs held: 39.58 vs 39.34 cm, HF ratio 1.654</t>
+        </is>
+      </c>
+      <c r="I49" s="1" t="inlineStr">
+        <is>
+          <t>30.48 (1 ft)</t>
+        </is>
+      </c>
+      <c r="J49" s="1" t="inlineStr">
+        <is>
+          <t>NOT FOUND (year from the county service name Aerial_2007 only)</t>
+        </is>
+      </c>
+      <c r="K49" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L49" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N49" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2007/ImageServer</t>
+        </is>
+      </c>
+      <c r="O49" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P49" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S07\measure.json): 25116x35259 px, 3 bands, EPSG:2285, 1,548,181,188 B; city coverage 100.0%, study-extent 100.0%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=['HF energy ratio 1.654 (sharper on a common grid)', 'no JPEG block signature (held has one)'] losses=[]. flip test vs 2007_king FAILED (eff 38.5 vs required &lt; 22.95) - complement, King keeps the 2007 key</t>
+        </is>
+      </c>
+      <c r="Q49" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R49" s="1" t="inlineStr"/>
+      <c r="S49" s="1" t="inlineStr"/>
+      <c r="T49" s="1" t="inlineStr"/>
+      <c r="U49" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U48"/>
+  <autoFilter ref="A1:U49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18838,7 +18964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P239"/>
+  <dimension ref="A1:P240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -31063,7 +31189,7 @@
       </c>
       <c r="N149" s="1" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>REPLACE 2026-08-23 -&gt; 2019_naip_60cm_rgbi.tif (coverage 100.0 &gt; 66.98; HF energy ratio 1.358 (sharper on a common grid)). no</t>
         </is>
       </c>
       <c r="O149" s="1" t="inlineStr">
@@ -38316,7 +38442,6 @@
           <t>see Pixel_Size_And_Date row</t>
         </is>
       </c>
-      <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
           <t>true GSD 30.48 cm; 3 bands; effective 38.53 cm; EPSG:2285; city coverage 100.0%</t>
@@ -38365,6 +38490,84 @@
       <c r="P239" t="inlineStr">
         <is>
           <t>decision COMPLEMENT: wins=['HF energy ratio 1.654 (sharper on a common grid)', 'no JPEG block signature (held has one)'] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S07</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>NAIP 2019 full-extent DOQQ mosaic (2019-10-11)</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr"/>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>true GSD 60.0 cm; 4 bands; effective 82.54 cm; EPSG:26910; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2019/wa_60cm_2019/47122/</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>https://naipeuwest.blob.core.windows.net/naip/v002/wa/2019/wa_60cm_2019/47122/</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>2019_naip_60cm_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N240" t="inlineStr">
+        <is>
+          <t>this file REPLACES 2019_naip_rgbi.tif</t>
+        </is>
+      </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P240" t="inlineStr">
+        <is>
+          <t>decision REPLACE: wins=['coverage 100.0 &gt; 66.98', 'HF energy ratio 1.358 (sharper on a common grid)'] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\NAIP_AZURE\2019\_acq\N19f</t>
         </is>
       </c>
     </row>
@@ -39238,7 +39441,7 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>RESOLVED 2026-08-23: REPLACE by 2019_naip_60cm_rgbi.tif. no</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
batch 6: keys 2009s/2011s/2012s/2006s/2013s (2011+2006 = new project years; 2012 sellable year exported free, sharper than the King orphan but partial); 1996 = earliest color, held without a year key; 2011s/2012s EPSG:2926 as delivered; catalog 33/33; table 54 rows
</commit_message>
<xml_diff>
--- a/Scripts/imagery_catalog_2026-08-22.xlsx
+++ b/Scripts/imagery_catalog_2026-08-22.xlsx
@@ -33,7 +33,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing_Risk" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MASTER'!$A$1:$P$221</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'KingCo_SDC_Catalog'!$A$1:$D$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DataLake_Issues'!$A$1:$C$15</definedName>
@@ -10920,7 +10920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11944,6 +11944,192 @@
       <c r="G31" t="inlineStr">
         <is>
           <t>median of 5 Method_Provenance sites; common-grid vs 2019_naip_rgbi.tif: new 84.3 / held 87.38 cm, HF ratio 1.358</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2009_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>30.48</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E32" t="n">
+        <v>39.74</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2011_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>30.48</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E33" t="n">
+        <v>38.12</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2012_snoh_9in_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>22.86</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E34" t="n">
+        <v>29.81</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1996_snoh_1m_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>100</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="E35" t="n">
+        <v>136.19</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2006_snoh_1m_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>100</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="E36" t="n">
+        <v>145.46</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2013_snoh_1m_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>100.021</v>
+      </c>
+      <c r="D37" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="E37" t="n">
+        <v>137.5</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-23 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
         </is>
       </c>
     </row>
@@ -12739,7 +12925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U49"/>
+  <dimension ref="A1:U55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -17636,8 +17822,578 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>2009_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>2009s (campaign S09)</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2009/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F50" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="inlineStr">
+        <is>
+          <t>30.48</t>
+        </is>
+      </c>
+      <c r="H50" s="1" t="inlineStr">
+        <is>
+          <t>39.74 (median of 5 sites; 1.3x its grid); common grid vs held: 40.88 vs 39.33 cm, HF ratio 1.128</t>
+        </is>
+      </c>
+      <c r="I50" s="1" t="inlineStr">
+        <is>
+          <t>30.48 (1 ft)</t>
+        </is>
+      </c>
+      <c r="J50" s="1" t="inlineStr">
+        <is>
+          <t>NOT FOUND (year from the county service name Aerial_2009 only)</t>
+        </is>
+      </c>
+      <c r="K50" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L50" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M50" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N50" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2009/ImageServer</t>
+        </is>
+      </c>
+      <c r="O50" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P50" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S09\measure.json): 25117x35260 px, 3 bands, EPSG:2285, 2,348,259,187 B; city coverage 100.0%, study-extent 98.42%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=['coverage 98.42 &gt; 94.92', 'HF energy ratio 1.128 (sharper on a common grid)', 'no JPEG block signature (held has one)'] losses=[]. Aerials Express product per the service; possibly the same flight as 2009_king - identity untested</t>
+        </is>
+      </c>
+      <c r="Q50" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R50" s="1" t="inlineStr"/>
+      <c r="S50" s="1" t="inlineStr"/>
+      <c r="T50" s="1" t="inlineStr"/>
+      <c r="U50" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>2011_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>2011s (campaign S11)</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2011/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2926</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="inlineStr">
+        <is>
+          <t>30.48</t>
+        </is>
+      </c>
+      <c r="H51" s="1" t="inlineStr">
+        <is>
+          <t>38.12 (median of 5 sites; 1.25x its grid)</t>
+        </is>
+      </c>
+      <c r="I51" s="1" t="inlineStr">
+        <is>
+          <t>30.48 (1 ft)</t>
+        </is>
+      </c>
+      <c r="J51" s="1" t="inlineStr">
+        <is>
+          <t>NOT FOUND (year from the county service name Aerial_2011 only)</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L51" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M51" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N51" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2011/ImageServer</t>
+        </is>
+      </c>
+      <c r="O51" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P51" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S11\measure.json): 25117x35259 px, 3 bands, EPSG:2926, 1,987,295,246 B; city coverage 99.63%, study-extent 79.92%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. 2011 = a calendar year the project previously had NO imagery for</t>
+        </is>
+      </c>
+      <c r="Q51" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R51" s="1" t="inlineStr"/>
+      <c r="S51" s="1" t="inlineStr"/>
+      <c r="T51" s="1" t="inlineStr"/>
+      <c r="U51" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>2012_snoh_9in_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>2012s (campaign S12)</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2012/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D52" s="1" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F52" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2926</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="inlineStr">
+        <is>
+          <t>22.86</t>
+        </is>
+      </c>
+      <c r="H52" s="1" t="inlineStr">
+        <is>
+          <t>29.81 (median of 5 sites; 1.3x its grid); common grid vs held: 29.59 vs 38.94 cm, HF ratio 1.571</t>
+        </is>
+      </c>
+      <c r="I52" s="1" t="inlineStr">
+        <is>
+          <t>22.86 (0.75 ft)</t>
+        </is>
+      </c>
+      <c r="J52" s="1" t="inlineStr">
+        <is>
+          <t>NOT FOUND (year from the county service name Aerial_2012 only)</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L52" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M52" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N52" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2012/ImageServer</t>
+        </is>
+      </c>
+      <c r="O52" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P52" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S12\measure.json): 33489x47012 px, 3 bands, EPSG:2926, 3,237,421,325 B; city coverage 99.63%, study-extent 82.29%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=['effective (common grid) 29.59 vs 38.94 cm', 'HF energy ratio 1.571 (sharper on a common grid)', 'no JPEG block signature (held has one)'] losses=['less coverage']. the year the county sells on media; free from the public service; sharper than 2012_king on a common grid but 82.3% coverage</t>
+        </is>
+      </c>
+      <c r="Q52" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R52" s="1" t="inlineStr"/>
+      <c r="S52" s="1" t="inlineStr"/>
+      <c r="T52" s="1" t="inlineStr"/>
+      <c r="U52" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>1996_snoh_1m_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>1996s (campaign S96)</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_1996/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D53" s="1" t="inlineStr">
+        <is>
+          <t>3.280833</t>
+        </is>
+      </c>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="H53" s="1" t="inlineStr">
+        <is>
+          <t>136.19 (median of 5 sites; 1.36x its grid)</t>
+        </is>
+      </c>
+      <c r="I53" s="1" t="inlineStr">
+        <is>
+          <t>100 (1 m)</t>
+        </is>
+      </c>
+      <c r="J53" s="1" t="inlineStr">
+        <is>
+          <t>NOT FOUND (year from the county service name Aerial_1996 only)</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L53" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N53" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_1996/ImageServer</t>
+        </is>
+      </c>
+      <c r="O53" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P53" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S96\measure.json): 7656x10748 px, 3 bands, EPSG:2285, 221,226,039 B; city coverage 100.0%, study-extent 94.13%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. earliest COLOR imagery of Edmonds held; outside the 2000-2024 span, no year key</t>
+        </is>
+      </c>
+      <c r="Q53" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R53" s="1" t="inlineStr"/>
+      <c r="S53" s="1" t="inlineStr"/>
+      <c r="T53" s="1" t="inlineStr"/>
+      <c r="U53" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>2006_snoh_1m_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B54" s="1" t="inlineStr">
+        <is>
+          <t>2006s (campaign S06)</t>
+        </is>
+      </c>
+      <c r="C54" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2006/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D54" s="1" t="inlineStr">
+        <is>
+          <t>3.280833</t>
+        </is>
+      </c>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F54" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="H54" s="1" t="inlineStr">
+        <is>
+          <t>145.46 (median of 5 sites; 1.45x its grid)</t>
+        </is>
+      </c>
+      <c r="I54" s="1" t="inlineStr">
+        <is>
+          <t>100 (1 m)</t>
+        </is>
+      </c>
+      <c r="J54" s="1" t="inlineStr">
+        <is>
+          <t>NOT FOUND (year from the county service name Aerial_2006 only)</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L54" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M54" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N54" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2006/ImageServer</t>
+        </is>
+      </c>
+      <c r="O54" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P54" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S06\measure.json): 7656x10748 px, 3 bands, EPSG:2285, 218,544,136 B; city coverage 100.0%, study-extent 100.0%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. 2006 = a new project year; likely the NAIP 2006 republished (untested)</t>
+        </is>
+      </c>
+      <c r="Q54" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R54" s="1" t="inlineStr"/>
+      <c r="S54" s="1" t="inlineStr"/>
+      <c r="T54" s="1" t="inlineStr"/>
+      <c r="U54" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>2013_snoh_1m_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>2013s (campaign S13)</t>
+        </is>
+      </c>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2013/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D55" s="1" t="inlineStr">
+        <is>
+          <t>3.281527</t>
+        </is>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F55" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G55" s="1" t="inlineStr">
+        <is>
+          <t>100.02</t>
+        </is>
+      </c>
+      <c r="H55" s="1" t="inlineStr">
+        <is>
+          <t>137.5 (median of 5 sites; 1.37x its grid)</t>
+        </is>
+      </c>
+      <c r="I55" s="1" t="inlineStr">
+        <is>
+          <t>100 (1 m)</t>
+        </is>
+      </c>
+      <c r="J55" s="1" t="inlineStr">
+        <is>
+          <t>NOT FOUND (year from the county service name Aerial_2013 only)</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L55" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M55" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N55" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2013/ImageServer</t>
+        </is>
+      </c>
+      <c r="O55" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P55" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S13\measure.json): 7655x10745 px, 3 bands, EPSG:2285, 155,772,878 B; city coverage 100.0%, study-extent 100.0%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. 1-m complement to 2013_king</t>
+        </is>
+      </c>
+      <c r="Q55" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R55" s="1" t="inlineStr"/>
+      <c r="S55" s="1" t="inlineStr"/>
+      <c r="T55" s="1" t="inlineStr"/>
+      <c r="U55" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U49"/>
+  <autoFilter ref="A1:U55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18964,7 +19720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P240"/>
+  <dimension ref="A1:P246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -38519,7 +39275,6 @@
           <t>see Pixel_Size_And_Date row</t>
         </is>
       </c>
-      <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
           <t>true GSD 60.0 cm; 4 bands; effective 82.54 cm; EPSG:26910; city coverage 100.0%</t>
@@ -38568,6 +39323,469 @@
       <c r="P240" t="inlineStr">
         <is>
           <t>decision REPLACE: wins=['coverage 100.0 &gt; 66.98', 'HF energy ratio 1.358 (sharper on a common grid)'] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\NAIP_AZURE\2019\_acq\N19f</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_2009 1-ft RGB (Aerials Express)</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>true GSD 30.48 cm; 3 bands; effective 39.74 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2009/ImageServer</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2009/ImageServer</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>2009_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N241" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P241" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=['coverage 98.42 &gt; 94.92', 'HF energy ratio 1.128 (sharper on a common grid)', 'no JPEG block signature (held has one)'] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S09</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_2011 1-ft RGB (new project year)</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>true GSD 30.48 cm; 3 bands; effective 38.12 cm; EPSG:2926; city coverage 99.63%</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2011/ImageServer</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2011/ImageServer</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>2011_snoh_1ft_rgb.tif</t>
+        </is>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N242" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P242" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S11</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_2012 9-in RGB (sharper than 2012_king, partial)</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>true GSD 22.86 cm; 3 bands; effective 29.81 cm; EPSG:2926; city coverage 99.63%</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2012/ImageServer</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2012/ImageServer</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>2012_snoh_9in_rgb.tif</t>
+        </is>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N243" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P243" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=['effective (common grid) 29.59 vs 38.94 cm', 'HF energy ratio 1.571 (sharper on a common grid)', 'no JPEG block signature (held has one)'] losses=['less coverage']; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S12</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>1996</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_1996 1-m RGB (earliest color)</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>true GSD 100.0 cm; 3 bands; effective 136.19 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_1996/ImageServer</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_1996/ImageServer</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>1996_snoh_1m_rgb.tif</t>
+        </is>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N244" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O244" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P244" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S96</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_2006 1-m RGB (new project year)</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>true GSD 100.0 cm; 3 bands; effective 145.46 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2006/ImageServer</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2006/ImageServer</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>2006_snoh_1m_rgb.tif</t>
+        </is>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N245" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O245" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P245" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S06</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Snohomish Aerial_2013 1-m RGB</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr"/>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>true GSD 100.021 cm; 3 bands; effective 137.5 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2013/ImageServer</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2013/ImageServer</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>2013_snoh_1m_rgb.tif</t>
+        </is>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N246" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O246" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P246" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
3-inch years landed: keys 2020s/2022s/2024s (91 GB, no cache signature, anchor untouched) - DOWNLOAD PROGRAMME COMPLETE: 29 rasters, 5 replaces, 4 new years, NIR 4->10, catalog 36/36, table 57 rows
</commit_message>
<xml_diff>
--- a/Scripts/imagery_catalog_2026-08-22.xlsx
+++ b/Scripts/imagery_catalog_2026-08-22.xlsx
@@ -33,7 +33,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing_Risk" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pixel_Size_And_Date'!$A$1:$U$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MASTER'!$A$1:$P$221</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'KingCo_SDC_Catalog'!$A$1:$D$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DataLake_Issues'!$A$1:$C$15</definedName>
@@ -10920,7 +10920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -12128,6 +12128,99 @@
         </is>
       </c>
       <c r="G37" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2020_snoh_3in_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="E38" t="n">
+        <v>9.77</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-24 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2022_snoh_3in_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E39" t="n">
+        <v>9.52</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-24 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>median of 5 sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2024_snoh_3in_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>SnoCo</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="E40" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>NEW 2026-08-24 (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
         <is>
           <t>median of 5 sites</t>
         </is>
@@ -12925,7 +13018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U55"/>
+  <dimension ref="A1:U58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -18392,8 +18485,281 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>2020_snoh_3in_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B56" s="1" t="inlineStr">
+        <is>
+          <t>2020s (campaign S20)</t>
+        </is>
+      </c>
+      <c r="C56" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2020/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D56" s="1" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="E56" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F56" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G56" s="1" t="inlineStr">
+        <is>
+          <t>7.62</t>
+        </is>
+      </c>
+      <c r="H56" s="1" t="inlineStr">
+        <is>
+          <t>9.77 (median of 5 sites; 1.28x its grid)</t>
+        </is>
+      </c>
+      <c r="I56" s="1" t="inlineStr">
+        <is>
+          <t>7.62 (0.25 ft)</t>
+        </is>
+      </c>
+      <c r="J56" s="1" t="inlineStr">
+        <is>
+          <t>inherited from the 2020_coe_rgb.tif row</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L56" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M56" s="7" t="inlineStr">
+        <is>
+          <t>INFERRED</t>
+        </is>
+      </c>
+      <c r="N56" s="1" t="inlineStr"/>
+      <c r="O56" s="1" t="inlineStr">
+        <is>
+          <t>(date evidence inherited from the 2020_coe_rgb.tif row - same flight, same service)</t>
+        </is>
+      </c>
+      <c r="P56" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S20\measure.json): 100463x141035 px, 3 bands, EPSG:2285, 31,012,508,090 B; city coverage 100.0%, study-extent 98.08%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. same county EagleView 2020 programme the anchor was cut from; ANCHOR NEVER FLIPPED; no JPEG signature (held CoE copy has one)</t>
+        </is>
+      </c>
+      <c r="Q56" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R56" s="1" t="inlineStr"/>
+      <c r="S56" s="1" t="inlineStr"/>
+      <c r="T56" s="1" t="inlineStr"/>
+      <c r="U56" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>2022_snoh_3in_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="inlineStr">
+        <is>
+          <t>2022s (campaign S22)</t>
+        </is>
+      </c>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2022/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D57" s="1" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="E57" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F57" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G57" s="1" t="inlineStr">
+        <is>
+          <t>7.62</t>
+        </is>
+      </c>
+      <c r="H57" s="1" t="inlineStr">
+        <is>
+          <t>9.52 (median of 5 sites; 1.25x its grid)</t>
+        </is>
+      </c>
+      <c r="I57" s="1" t="inlineStr">
+        <is>
+          <t>7.62 (0.25 ft)</t>
+        </is>
+      </c>
+      <c r="J57" s="1" t="inlineStr">
+        <is>
+          <t>inherited from the 2022_coe_rgb.tif row</t>
+        </is>
+      </c>
+      <c r="K57" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L57" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M57" s="7" t="inlineStr">
+        <is>
+          <t>INFERRED</t>
+        </is>
+      </c>
+      <c r="N57" s="1" t="inlineStr"/>
+      <c r="O57" s="1" t="inlineStr">
+        <is>
+          <t>(date evidence inherited from the 2022_coe_rgb.tif row - same flight, same service)</t>
+        </is>
+      </c>
+      <c r="P57" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S22\measure.json): 100463x141035 px, 3 bands, EPSG:2285, 30,182,395,806 B; city coverage 100.0%, study-extent 98.08%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. same county EagleView 2022 programme; no JPEG signature (held CoE copy has one)</t>
+        </is>
+      </c>
+      <c r="Q57" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R57" s="1" t="inlineStr"/>
+      <c r="S57" s="1" t="inlineStr"/>
+      <c r="T57" s="1" t="inlineStr"/>
+      <c r="U57" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>2024_snoh_3in_rgb.tif</t>
+        </is>
+      </c>
+      <c r="B58" s="1" t="inlineStr">
+        <is>
+          <t>2024s (campaign S24)</t>
+        </is>
+      </c>
+      <c r="C58" s="1" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2024/ImageServer via pipeline/acquire_imagery.py (export)</t>
+        </is>
+      </c>
+      <c r="D58" s="1" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="E58" s="1" t="inlineStr">
+        <is>
+          <t>US survey foot</t>
+        </is>
+      </c>
+      <c r="F58" s="1" t="inlineStr">
+        <is>
+          <t>EPSG:2285</t>
+        </is>
+      </c>
+      <c r="G58" s="1" t="inlineStr">
+        <is>
+          <t>7.62</t>
+        </is>
+      </c>
+      <c r="H58" s="1" t="inlineStr">
+        <is>
+          <t>10.2 (median of 5 sites; 1.34x its grid)</t>
+        </is>
+      </c>
+      <c r="I58" s="1" t="inlineStr">
+        <is>
+          <t>7.62 (0.25 ft)</t>
+        </is>
+      </c>
+      <c r="J58" s="1" t="inlineStr">
+        <is>
+          <t>inherited from the 2024_coe_rgb.tif row</t>
+        </is>
+      </c>
+      <c r="K58" s="1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L58" s="1" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="M58" s="7" t="inlineStr">
+        <is>
+          <t>INFERRED</t>
+        </is>
+      </c>
+      <c r="N58" s="1" t="inlineStr"/>
+      <c r="O58" s="1" t="inlineStr">
+        <is>
+          <t>(date evidence inherited from the 2024_coe_rgb.tif row - same flight, same service)</t>
+        </is>
+      </c>
+      <c r="P58" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED on arrival (D:\edmonds-pipeline\Imagery\SnoCo\_acq\S24\measure.json): 100463x141035 px, 3 bands, EPSG:2285, 29,570,524,494 B; city coverage 100.0%, study-extent 98.08%; JPEG 8x8 signature absent. Decision COMPLEMENT: wins=[] losses=[]. same county EagleView 2024 programme; no JPEG signature (held CoE copy has one)</t>
+        </is>
+      </c>
+      <c r="Q58" s="1" t="inlineStr">
+        <is>
+          <t>grid/true/effective MEASURED (acquire_imagery verify)</t>
+        </is>
+      </c>
+      <c r="R58" s="1" t="inlineStr"/>
+      <c r="S58" s="1" t="inlineStr"/>
+      <c r="T58" s="1" t="inlineStr"/>
+      <c r="U58" s="1" t="inlineStr">
+        <is>
+          <t>held imagery (campaign)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U55"/>
+  <autoFilter ref="A1:U58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19720,7 +20086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P246"/>
+  <dimension ref="A1:P249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -39737,7 +40103,6 @@
           <t>see Pixel_Size_And_Date row</t>
         </is>
       </c>
-      <c r="F246" t="inlineStr"/>
       <c r="G246" t="inlineStr">
         <is>
           <t>true GSD 100.021 cm; 3 bands; effective 137.5 cm; EPSG:2285; city coverage 100.0%</t>
@@ -39786,6 +40151,238 @@
       <c r="P246" t="inlineStr">
         <is>
           <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S13</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Snohomish EagleView 3-in RGB (county serving, no cache signature)</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>true GSD 7.62 cm; 3 bands; effective 9.77 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2020/ImageServer</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2020/ImageServer</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K247" t="inlineStr">
+        <is>
+          <t>2020_snoh_3in_rgb.tif</t>
+        </is>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N247" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O247" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P247" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S20</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Snohomish EagleView 3-in RGB (county serving, no cache signature)</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>true GSD 7.62 cm; 3 bands; effective 9.52 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2022/ImageServer</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2022/ImageServer</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K248" t="inlineStr">
+        <is>
+          <t>2022_snoh_3in_rgb.tif</t>
+        </is>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N248" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P248" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S22</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>imagery</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Snohomish EagleView 3-in RGB (county serving, no cache signature)</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>acquire_imagery campaign 2026-08-23</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>see Pixel_Size_And_Date row</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr"/>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>true GSD 7.62 cm; 3 bands; effective 10.2 cm; EPSG:2285; city coverage 100.0%</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2024/ImageServer</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>https://gis.snoco.org/img/rest/services/Imagery/Aerial_2024/ImageServer</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K249" t="inlineStr">
+        <is>
+          <t>2024_snoh_3in_rgb.tif</t>
+        </is>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>none known (measured on arrival)</t>
+        </is>
+      </c>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>n/a (already held)</t>
+        </is>
+      </c>
+      <c r="N249" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="P249" t="inlineStr">
+        <is>
+          <t>decision COMPLEMENT: wins=[] losses=[]; measure.json under D:\edmonds-pipeline\Imagery\SnoCo\_acq\S24</t>
         </is>
       </c>
     </row>

</xml_diff>